<commit_message>
fix: disposition char limit, false-offline flash, AFOR city overwrite, revision diff; ignore Maven target/
</commit_message>
<xml_diff>
--- a/sample AFOR.xlsx
+++ b/sample AFOR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gwent\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\WIMS-BFP-PROTOTYPE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582663FE-F0F1-405D-B24C-446C24E259A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7453CAB-377A-4648-89FE-C4AFEF5B2DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5112" yWindow="180" windowWidth="17280" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AFOR" sheetId="1" r:id="rId1"/>
@@ -6750,111 +6750,33 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6867,14 +6789,92 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -8689,14 +8689,14 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="100" t="s">
+      <c r="A7" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="65"/>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -8719,14 +8719,14 @@
       <c r="Z7" s="3"/>
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="101" t="s">
+      <c r="A8" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="65"/>
-      <c r="C8" s="65"/>
-      <c r="D8" s="65"/>
-      <c r="E8" s="65"/>
-      <c r="F8" s="65"/>
+      <c r="B8" s="66"/>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -8749,14 +8749,14 @@
       <c r="Z8" s="4"/>
     </row>
     <row r="9" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="102" t="s">
+      <c r="A9" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="65"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
+      <c r="B9" s="66"/>
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -8779,14 +8779,14 @@
       <c r="Z9" s="5"/>
     </row>
     <row r="10" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="100" t="s">
+      <c r="A10" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="65"/>
-      <c r="C10" s="65"/>
-      <c r="D10" s="65"/>
-      <c r="E10" s="65"/>
-      <c r="F10" s="65"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -8809,14 +8809,14 @@
       <c r="Z10" s="3"/>
     </row>
     <row r="11" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="100" t="s">
+      <c r="A11" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
+      <c r="B11" s="66"/>
+      <c r="C11" s="66"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="66"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -8839,14 +8839,14 @@
       <c r="Z11" s="3"/>
     </row>
     <row r="12" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="103" t="s">
+      <c r="A12" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="65"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
+      <c r="B12" s="66"/>
+      <c r="C12" s="66"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="66"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -8897,14 +8897,14 @@
       <c r="Z13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="104" t="s">
+      <c r="A14" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="65"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="65"/>
-      <c r="E14" s="65"/>
-      <c r="F14" s="65"/>
+      <c r="B14" s="66"/>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="66"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -8955,14 +8955,14 @@
       <c r="Z15" s="2"/>
     </row>
     <row r="16" spans="1:26" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="96" t="s">
+      <c r="A16" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="65"/>
-      <c r="C16" s="65"/>
-      <c r="D16" s="65"/>
-      <c r="E16" s="65"/>
-      <c r="F16" s="65"/>
+      <c r="B16" s="66"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -9043,16 +9043,16 @@
       <c r="Z18" s="9"/>
     </row>
     <row r="19" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="70">
+      <c r="A19" s="73">
         <v>1</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C19" s="11"/>
-      <c r="D19" s="97"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="58"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="57"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
       <c r="I19" s="9"/>
@@ -9075,18 +9075,18 @@
       <c r="Z19" s="9"/>
     </row>
     <row r="20" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="71"/>
+      <c r="A20" s="74"/>
       <c r="B20" s="11" t="s">
         <v>1953</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="98" t="s">
+      <c r="D20" s="61" t="s">
         <v>1954</v>
       </c>
-      <c r="E20" s="57"/>
-      <c r="F20" s="58"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="57"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
@@ -9109,16 +9109,16 @@
       <c r="Z20" s="9"/>
     </row>
     <row r="21" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="72"/>
+      <c r="A21" s="75"/>
       <c r="B21" s="11"/>
       <c r="C21" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="98" t="s">
+      <c r="D21" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="57"/>
-      <c r="F21" s="58"/>
+      <c r="E21" s="58"/>
+      <c r="F21" s="57"/>
       <c r="G21" s="13"/>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
@@ -9148,11 +9148,11 @@
         <v>13</v>
       </c>
       <c r="C22" s="11"/>
-      <c r="D22" s="99">
-        <v>38221</v>
-      </c>
-      <c r="E22" s="57"/>
-      <c r="F22" s="58"/>
+      <c r="D22" s="77">
+        <v>46202</v>
+      </c>
+      <c r="E22" s="58"/>
+      <c r="F22" s="57"/>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
@@ -9182,11 +9182,11 @@
         <v>14</v>
       </c>
       <c r="C23" s="11"/>
-      <c r="D23" s="91">
-        <v>0.93194444444444446</v>
-      </c>
-      <c r="E23" s="57"/>
-      <c r="F23" s="58"/>
+      <c r="D23" s="71">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="E23" s="58"/>
+      <c r="F23" s="57"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
@@ -9209,7 +9209,7 @@
       <c r="Z23" s="9"/>
     </row>
     <row r="24" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="70">
+      <c r="A24" s="73">
         <v>4</v>
       </c>
       <c r="B24" s="11" t="s">
@@ -9219,8 +9219,8 @@
       <c r="D24" s="60" t="s">
         <v>241</v>
       </c>
-      <c r="E24" s="57"/>
-      <c r="F24" s="58"/>
+      <c r="E24" s="58"/>
+      <c r="F24" s="57"/>
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
@@ -9243,7 +9243,7 @@
       <c r="Z24" s="9"/>
     </row>
     <row r="25" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="71"/>
+      <c r="A25" s="74"/>
       <c r="B25" s="11" t="s">
         <v>16</v>
       </c>
@@ -9251,8 +9251,8 @@
       <c r="D25" s="60" t="s">
         <v>1955</v>
       </c>
-      <c r="E25" s="57"/>
-      <c r="F25" s="58"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="57"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
@@ -9275,7 +9275,7 @@
       <c r="Z25" s="9"/>
     </row>
     <row r="26" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="71"/>
+      <c r="A26" s="74"/>
       <c r="B26" s="11" t="s">
         <v>17</v>
       </c>
@@ -9283,8 +9283,8 @@
       <c r="D26" s="60" t="s">
         <v>1956</v>
       </c>
-      <c r="E26" s="57"/>
-      <c r="F26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="57"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
@@ -9307,7 +9307,7 @@
       <c r="Z26" s="9"/>
     </row>
     <row r="27" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="72"/>
+      <c r="A27" s="75"/>
       <c r="B27" s="11" t="s">
         <v>18</v>
       </c>
@@ -9349,8 +9349,8 @@
       <c r="D28" s="60" t="s">
         <v>1958</v>
       </c>
-      <c r="E28" s="57"/>
-      <c r="F28" s="58"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="57"/>
       <c r="G28" s="16"/>
       <c r="H28" s="9"/>
       <c r="I28" s="9"/>
@@ -9383,8 +9383,8 @@
       <c r="D29" s="60" t="s">
         <v>1959</v>
       </c>
-      <c r="E29" s="57"/>
-      <c r="F29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="57"/>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
       <c r="I29" s="9"/>
@@ -9417,8 +9417,8 @@
       <c r="D30" s="60" t="s">
         <v>1960</v>
       </c>
-      <c r="E30" s="57"/>
-      <c r="F30" s="58"/>
+      <c r="E30" s="58"/>
+      <c r="F30" s="57"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
       <c r="I30" s="9"/>
@@ -9441,18 +9441,18 @@
       <c r="Z30" s="9"/>
     </row>
     <row r="31" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="70">
+      <c r="A31" s="73">
         <v>8</v>
       </c>
-      <c r="B31" s="80" t="s">
+      <c r="B31" s="78" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="63"/>
+      <c r="C31" s="79"/>
       <c r="D31" s="60" t="s">
         <v>1961</v>
       </c>
-      <c r="E31" s="57"/>
-      <c r="F31" s="58"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="57"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
       <c r="I31" s="9"/>
@@ -9475,14 +9475,14 @@
       <c r="Z31" s="9"/>
     </row>
     <row r="32" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="71"/>
-      <c r="B32" s="64"/>
-      <c r="C32" s="66"/>
+      <c r="A32" s="74"/>
+      <c r="B32" s="80"/>
+      <c r="C32" s="81"/>
       <c r="D32" s="60" t="s">
         <v>1962</v>
       </c>
-      <c r="E32" s="57"/>
-      <c r="F32" s="58"/>
+      <c r="E32" s="58"/>
+      <c r="F32" s="57"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
       <c r="I32" s="9"/>
@@ -9505,12 +9505,12 @@
       <c r="Z32" s="9"/>
     </row>
     <row r="33" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="72"/>
-      <c r="B33" s="64"/>
-      <c r="C33" s="66"/>
+      <c r="A33" s="75"/>
+      <c r="B33" s="80"/>
+      <c r="C33" s="81"/>
       <c r="D33" s="60"/>
-      <c r="E33" s="57"/>
-      <c r="F33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="57"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
       <c r="I33" s="9"/>
@@ -9533,18 +9533,18 @@
       <c r="Z33" s="9"/>
     </row>
     <row r="34" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="70">
+      <c r="A34" s="73">
         <v>9</v>
       </c>
-      <c r="B34" s="80" t="s">
+      <c r="B34" s="78" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="63"/>
-      <c r="D34" s="91">
-        <v>5.7638888888888892E-2</v>
-      </c>
-      <c r="E34" s="57"/>
-      <c r="F34" s="58"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="71">
+        <v>0.43680555555555556</v>
+      </c>
+      <c r="E34" s="58"/>
+      <c r="F34" s="57"/>
       <c r="G34" s="9"/>
       <c r="H34" s="9"/>
       <c r="I34" s="9"/>
@@ -9567,14 +9567,14 @@
       <c r="Z34" s="9"/>
     </row>
     <row r="35" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="71"/>
-      <c r="B35" s="64"/>
-      <c r="C35" s="66"/>
-      <c r="D35" s="91">
-        <v>5.9027777777777776E-2</v>
-      </c>
-      <c r="E35" s="57"/>
-      <c r="F35" s="58"/>
+      <c r="A35" s="74"/>
+      <c r="B35" s="80"/>
+      <c r="C35" s="81"/>
+      <c r="D35" s="71">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="E35" s="58"/>
+      <c r="F35" s="57"/>
       <c r="G35" s="9"/>
       <c r="H35" s="9"/>
       <c r="I35" s="9"/>
@@ -9597,12 +9597,12 @@
       <c r="Z35" s="9"/>
     </row>
     <row r="36" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="72"/>
-      <c r="B36" s="67"/>
-      <c r="C36" s="69"/>
+      <c r="A36" s="75"/>
+      <c r="B36" s="85"/>
+      <c r="C36" s="87"/>
       <c r="D36" s="60"/>
-      <c r="E36" s="57"/>
-      <c r="F36" s="58"/>
+      <c r="E36" s="58"/>
+      <c r="F36" s="57"/>
       <c r="G36" s="9"/>
       <c r="H36" s="9"/>
       <c r="I36" s="9"/>
@@ -9625,18 +9625,18 @@
       <c r="Z36" s="9"/>
     </row>
     <row r="37" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="70">
+      <c r="A37" s="73">
         <v>10</v>
       </c>
-      <c r="B37" s="80" t="s">
+      <c r="B37" s="78" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="63"/>
-      <c r="D37" s="91">
-        <v>7.5694444444444439E-2</v>
-      </c>
-      <c r="E37" s="57"/>
-      <c r="F37" s="58"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="71">
+        <v>0.45208333333333334</v>
+      </c>
+      <c r="E37" s="58"/>
+      <c r="F37" s="57"/>
       <c r="G37" s="9"/>
       <c r="H37" s="9"/>
       <c r="I37" s="9"/>
@@ -9659,14 +9659,14 @@
       <c r="Z37" s="9"/>
     </row>
     <row r="38" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="71"/>
-      <c r="B38" s="64"/>
-      <c r="C38" s="66"/>
-      <c r="D38" s="91">
-        <v>8.1944444444444445E-2</v>
-      </c>
-      <c r="E38" s="57"/>
-      <c r="F38" s="58"/>
+      <c r="A38" s="74"/>
+      <c r="B38" s="80"/>
+      <c r="C38" s="81"/>
+      <c r="D38" s="71">
+        <v>0.45694444444444443</v>
+      </c>
+      <c r="E38" s="58"/>
+      <c r="F38" s="57"/>
       <c r="G38" s="9"/>
       <c r="H38" s="9"/>
       <c r="I38" s="9"/>
@@ -9689,12 +9689,12 @@
       <c r="Z38" s="9"/>
     </row>
     <row r="39" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="72"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="69"/>
+      <c r="A39" s="75"/>
+      <c r="B39" s="85"/>
+      <c r="C39" s="87"/>
       <c r="D39" s="60"/>
-      <c r="E39" s="57"/>
-      <c r="F39" s="58"/>
+      <c r="E39" s="58"/>
+      <c r="F39" s="57"/>
       <c r="G39" s="9"/>
       <c r="H39" s="9"/>
       <c r="I39" s="9"/>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="C40" s="11"/>
       <c r="D40" s="92">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E40" s="93"/>
       <c r="F40" s="94"/>
@@ -9754,15 +9754,15 @@
       <c r="A41" s="14">
         <v>12</v>
       </c>
-      <c r="B41" s="81" t="s">
+      <c r="B41" s="97" t="s">
         <v>26</v>
       </c>
-      <c r="C41" s="58"/>
+      <c r="C41" s="57"/>
       <c r="D41" s="60">
         <v>9.8000000000000007</v>
       </c>
-      <c r="E41" s="57"/>
-      <c r="F41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="57"/>
       <c r="G41" s="9"/>
       <c r="H41" s="9"/>
       <c r="I41" s="9"/>
@@ -9788,15 +9788,15 @@
       <c r="A42" s="14">
         <v>13</v>
       </c>
-      <c r="B42" s="82" t="s">
+      <c r="B42" s="101" t="s">
         <v>27</v>
       </c>
-      <c r="C42" s="58"/>
+      <c r="C42" s="57"/>
       <c r="D42" s="95" t="s">
         <v>1963</v>
       </c>
-      <c r="E42" s="57"/>
-      <c r="F42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="57"/>
       <c r="G42" s="9"/>
       <c r="H42" s="9"/>
       <c r="I42" s="9"/>
@@ -9826,11 +9826,11 @@
         <v>28</v>
       </c>
       <c r="C43" s="11"/>
-      <c r="D43" s="91">
-        <v>0.22291666666666668</v>
-      </c>
-      <c r="E43" s="57"/>
-      <c r="F43" s="58"/>
+      <c r="D43" s="71">
+        <v>0.63958333333333328</v>
+      </c>
+      <c r="E43" s="58"/>
+      <c r="F43" s="57"/>
       <c r="G43" s="9"/>
       <c r="H43" s="9"/>
       <c r="I43" s="9"/>
@@ -9863,8 +9863,8 @@
       <c r="D44" s="60">
         <v>21</v>
       </c>
-      <c r="E44" s="57"/>
-      <c r="F44" s="58"/>
+      <c r="E44" s="58"/>
+      <c r="F44" s="57"/>
       <c r="G44" s="9"/>
       <c r="H44" s="9"/>
       <c r="I44" s="9"/>
@@ -9945,7 +9945,7 @@
       <c r="Z46" s="9"/>
     </row>
     <row r="47" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="70">
+      <c r="A47" s="73">
         <v>16</v>
       </c>
       <c r="B47" s="19" t="s">
@@ -9953,8 +9953,8 @@
       </c>
       <c r="C47" s="19"/>
       <c r="D47" s="60"/>
-      <c r="E47" s="57"/>
-      <c r="F47" s="58"/>
+      <c r="E47" s="58"/>
+      <c r="F47" s="57"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
       <c r="I47" s="9"/>
@@ -9977,14 +9977,14 @@
       <c r="Z47" s="9"/>
     </row>
     <row r="48" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="71"/>
+      <c r="A48" s="74"/>
       <c r="B48" s="11"/>
       <c r="C48" s="12" t="s">
         <v>32</v>
       </c>
       <c r="D48" s="60"/>
-      <c r="E48" s="57"/>
-      <c r="F48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="57"/>
       <c r="G48" s="9"/>
       <c r="H48" s="9"/>
       <c r="I48" s="9"/>
@@ -10007,14 +10007,14 @@
       <c r="Z48" s="9"/>
     </row>
     <row r="49" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="71"/>
+      <c r="A49" s="74"/>
       <c r="B49" s="11"/>
       <c r="C49" s="12" t="s">
         <v>33</v>
       </c>
       <c r="D49" s="60"/>
-      <c r="E49" s="57"/>
-      <c r="F49" s="58"/>
+      <c r="E49" s="58"/>
+      <c r="F49" s="57"/>
       <c r="G49" s="9"/>
       <c r="H49" s="9"/>
       <c r="I49" s="9"/>
@@ -10037,17 +10037,17 @@
       <c r="Z49" s="9"/>
     </row>
     <row r="50" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="72"/>
+      <c r="A50" s="75"/>
       <c r="B50" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C50" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D50" s="76" t="s">
+      <c r="D50" s="56" t="s">
         <v>1964</v>
       </c>
-      <c r="E50" s="58"/>
+      <c r="E50" s="57"/>
       <c r="F50" s="19"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
@@ -10074,15 +10074,15 @@
       <c r="A51" s="14">
         <v>17</v>
       </c>
-      <c r="B51" s="81" t="s">
+      <c r="B51" s="97" t="s">
         <v>35</v>
       </c>
-      <c r="C51" s="58"/>
-      <c r="D51" s="76" t="s">
+      <c r="C51" s="57"/>
+      <c r="D51" s="56" t="s">
         <v>1965</v>
       </c>
-      <c r="E51" s="57"/>
-      <c r="F51" s="58"/>
+      <c r="E51" s="58"/>
+      <c r="F51" s="57"/>
       <c r="G51" s="9"/>
       <c r="H51" s="9"/>
       <c r="I51" s="9"/>
@@ -10108,15 +10108,15 @@
       <c r="A52" s="14">
         <v>18</v>
       </c>
-      <c r="B52" s="81" t="s">
+      <c r="B52" s="97" t="s">
         <v>36</v>
       </c>
-      <c r="C52" s="58"/>
-      <c r="D52" s="76" t="s">
+      <c r="C52" s="57"/>
+      <c r="D52" s="56" t="s">
         <v>1987</v>
       </c>
-      <c r="E52" s="57"/>
-      <c r="F52" s="58"/>
+      <c r="E52" s="58"/>
+      <c r="F52" s="57"/>
       <c r="G52" s="9"/>
       <c r="H52" s="9"/>
       <c r="I52" s="9"/>
@@ -10142,15 +10142,15 @@
       <c r="A53" s="14">
         <v>19</v>
       </c>
-      <c r="B53" s="81" t="s">
+      <c r="B53" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="C53" s="58"/>
-      <c r="D53" s="76" t="s">
+      <c r="C53" s="57"/>
+      <c r="D53" s="56" t="s">
         <v>1966</v>
       </c>
-      <c r="E53" s="57"/>
-      <c r="F53" s="58"/>
+      <c r="E53" s="58"/>
+      <c r="F53" s="57"/>
       <c r="G53" s="20"/>
       <c r="H53" s="20"/>
       <c r="I53" s="20"/>
@@ -10176,15 +10176,15 @@
       <c r="A54" s="10">
         <v>20</v>
       </c>
-      <c r="B54" s="81" t="s">
+      <c r="B54" s="97" t="s">
         <v>38</v>
       </c>
-      <c r="C54" s="58"/>
-      <c r="D54" s="107" t="s">
+      <c r="C54" s="57"/>
+      <c r="D54" s="59" t="s">
         <v>1967</v>
       </c>
-      <c r="E54" s="57"/>
-      <c r="F54" s="58"/>
+      <c r="E54" s="58"/>
+      <c r="F54" s="57"/>
       <c r="G54" s="20"/>
       <c r="H54" s="20"/>
       <c r="I54" s="20"/>
@@ -10207,7 +10207,7 @@
       <c r="Z54" s="20"/>
     </row>
     <row r="55" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="70">
+      <c r="A55" s="73">
         <v>21</v>
       </c>
       <c r="B55" s="11" t="s">
@@ -10215,8 +10215,8 @@
       </c>
       <c r="C55" s="19"/>
       <c r="D55" s="60"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="58"/>
+      <c r="E55" s="58"/>
+      <c r="F55" s="57"/>
       <c r="G55" s="9"/>
       <c r="H55" s="9"/>
       <c r="I55" s="9"/>
@@ -10239,16 +10239,16 @@
       <c r="Z55" s="9"/>
     </row>
     <row r="56" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="71"/>
+      <c r="A56" s="74"/>
       <c r="B56" s="19"/>
       <c r="C56" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D56" s="98" t="s">
+      <c r="D56" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="E56" s="57"/>
-      <c r="F56" s="58"/>
+      <c r="E56" s="58"/>
+      <c r="F56" s="57"/>
       <c r="G56" s="9"/>
       <c r="H56" s="9"/>
       <c r="I56" s="9"/>
@@ -10271,18 +10271,18 @@
       <c r="Z56" s="9"/>
     </row>
     <row r="57" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="71"/>
+      <c r="A57" s="74"/>
       <c r="B57" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C57" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="D57" s="75" t="s">
+      <c r="D57" s="62" t="s">
         <v>1968</v>
       </c>
-      <c r="E57" s="57"/>
-      <c r="F57" s="58"/>
+      <c r="E57" s="58"/>
+      <c r="F57" s="57"/>
       <c r="G57" s="9"/>
       <c r="H57" s="9"/>
       <c r="I57" s="9"/>
@@ -10305,16 +10305,16 @@
       <c r="Z57" s="9"/>
     </row>
     <row r="58" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="71"/>
+      <c r="A58" s="74"/>
       <c r="B58" s="19"/>
       <c r="C58" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D58" s="98" t="s">
+      <c r="D58" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="E58" s="57"/>
-      <c r="F58" s="58"/>
+      <c r="E58" s="58"/>
+      <c r="F58" s="57"/>
       <c r="G58" s="9"/>
       <c r="H58" s="9"/>
       <c r="I58" s="9"/>
@@ -10337,16 +10337,16 @@
       <c r="Z58" s="9"/>
     </row>
     <row r="59" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="71"/>
+      <c r="A59" s="74"/>
       <c r="B59" s="19"/>
       <c r="C59" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D59" s="98" t="s">
+      <c r="D59" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="57"/>
-      <c r="F59" s="58"/>
+      <c r="E59" s="58"/>
+      <c r="F59" s="57"/>
       <c r="G59" s="9"/>
       <c r="H59" s="9"/>
       <c r="I59" s="9"/>
@@ -10369,16 +10369,16 @@
       <c r="Z59" s="9"/>
     </row>
     <row r="60" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="71"/>
+      <c r="A60" s="74"/>
       <c r="B60" s="19"/>
       <c r="C60" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D60" s="98" t="s">
+      <c r="D60" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="E60" s="57"/>
-      <c r="F60" s="58"/>
+      <c r="E60" s="58"/>
+      <c r="F60" s="57"/>
       <c r="G60" s="9"/>
       <c r="H60" s="9"/>
       <c r="I60" s="9"/>
@@ -10401,16 +10401,16 @@
       <c r="Z60" s="9"/>
     </row>
     <row r="61" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="72"/>
+      <c r="A61" s="75"/>
       <c r="B61" s="19"/>
       <c r="C61" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="D61" s="98" t="s">
+      <c r="D61" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="E61" s="57"/>
-      <c r="F61" s="58"/>
+      <c r="E61" s="58"/>
+      <c r="F61" s="57"/>
       <c r="G61" s="9"/>
       <c r="H61" s="9"/>
       <c r="I61" s="9"/>
@@ -10440,11 +10440,11 @@
         <v>50</v>
       </c>
       <c r="C62" s="19"/>
-      <c r="D62" s="98">
+      <c r="D62" s="61">
         <v>12</v>
       </c>
-      <c r="E62" s="57"/>
-      <c r="F62" s="58"/>
+      <c r="E62" s="58"/>
+      <c r="F62" s="57"/>
       <c r="G62" s="9"/>
       <c r="H62" s="9"/>
       <c r="I62" s="9"/>
@@ -10474,11 +10474,11 @@
         <v>51</v>
       </c>
       <c r="C63" s="19"/>
-      <c r="D63" s="98">
+      <c r="D63" s="61">
         <v>12</v>
       </c>
-      <c r="E63" s="57"/>
-      <c r="F63" s="58"/>
+      <c r="E63" s="58"/>
+      <c r="F63" s="57"/>
       <c r="G63" s="9"/>
       <c r="H63" s="9"/>
       <c r="I63" s="9"/>
@@ -10508,11 +10508,11 @@
         <v>52</v>
       </c>
       <c r="C64" s="19"/>
-      <c r="D64" s="98">
+      <c r="D64" s="61">
         <v>12</v>
       </c>
-      <c r="E64" s="57"/>
-      <c r="F64" s="58"/>
+      <c r="E64" s="58"/>
+      <c r="F64" s="57"/>
       <c r="G64" s="9"/>
       <c r="H64" s="9"/>
       <c r="I64" s="9"/>
@@ -10542,11 +10542,11 @@
         <v>53</v>
       </c>
       <c r="C65" s="19"/>
-      <c r="D65" s="98">
+      <c r="D65" s="61">
         <v>12</v>
       </c>
-      <c r="E65" s="57"/>
-      <c r="F65" s="58"/>
+      <c r="E65" s="58"/>
+      <c r="F65" s="57"/>
       <c r="G65" s="9"/>
       <c r="H65" s="9"/>
       <c r="I65" s="9"/>
@@ -10576,11 +10576,11 @@
         <v>54</v>
       </c>
       <c r="C66" s="19"/>
-      <c r="D66" s="98">
+      <c r="D66" s="61">
         <v>12</v>
       </c>
-      <c r="E66" s="57"/>
-      <c r="F66" s="58"/>
+      <c r="E66" s="58"/>
+      <c r="F66" s="57"/>
       <c r="G66" s="9"/>
       <c r="H66" s="9"/>
       <c r="I66" s="9"/>
@@ -10661,7 +10661,7 @@
       <c r="Z68" s="9"/>
     </row>
     <row r="69" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="70">
+      <c r="A69" s="73">
         <v>27</v>
       </c>
       <c r="B69" s="19" t="s">
@@ -10669,8 +10669,8 @@
       </c>
       <c r="C69" s="19"/>
       <c r="D69" s="60"/>
-      <c r="E69" s="57"/>
-      <c r="F69" s="58"/>
+      <c r="E69" s="58"/>
+      <c r="F69" s="57"/>
       <c r="G69" s="9"/>
       <c r="H69" s="9"/>
       <c r="I69" s="9"/>
@@ -10693,18 +10693,18 @@
       <c r="Z69" s="9"/>
     </row>
     <row r="70" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="71"/>
+      <c r="A70" s="74"/>
       <c r="B70" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C70" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D70" s="98">
+      <c r="D70" s="61">
         <v>67</v>
       </c>
-      <c r="E70" s="57"/>
-      <c r="F70" s="58"/>
+      <c r="E70" s="58"/>
+      <c r="F70" s="57"/>
       <c r="G70" s="9"/>
       <c r="H70" s="9"/>
       <c r="I70" s="9"/>
@@ -10727,18 +10727,18 @@
       <c r="Z70" s="9"/>
     </row>
     <row r="71" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="71"/>
+      <c r="A71" s="74"/>
       <c r="B71" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C71" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="D71" s="98">
+      <c r="D71" s="61">
         <v>67</v>
       </c>
-      <c r="E71" s="57"/>
-      <c r="F71" s="58"/>
+      <c r="E71" s="58"/>
+      <c r="F71" s="57"/>
       <c r="G71" s="9"/>
       <c r="H71" s="9"/>
       <c r="I71" s="9"/>
@@ -10761,16 +10761,16 @@
       <c r="Z71" s="9"/>
     </row>
     <row r="72" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="71"/>
+      <c r="A72" s="74"/>
       <c r="B72" s="11"/>
       <c r="C72" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="D72" s="98">
+      <c r="D72" s="61">
         <v>67</v>
       </c>
-      <c r="E72" s="57"/>
-      <c r="F72" s="58"/>
+      <c r="E72" s="58"/>
+      <c r="F72" s="57"/>
       <c r="G72" s="9"/>
       <c r="H72" s="9"/>
       <c r="I72" s="9"/>
@@ -10793,18 +10793,18 @@
       <c r="Z72" s="9"/>
     </row>
     <row r="73" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="71"/>
+      <c r="A73" s="74"/>
       <c r="B73" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C73" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="D73" s="98">
+      <c r="D73" s="61">
         <v>67</v>
       </c>
-      <c r="E73" s="57"/>
-      <c r="F73" s="58"/>
+      <c r="E73" s="58"/>
+      <c r="F73" s="57"/>
       <c r="G73" s="9"/>
       <c r="H73" s="9"/>
       <c r="I73" s="9"/>
@@ -10827,18 +10827,18 @@
       <c r="Z73" s="9"/>
     </row>
     <row r="74" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="71"/>
+      <c r="A74" s="74"/>
       <c r="B74" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C74" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D74" s="98">
+      <c r="D74" s="61">
         <v>67</v>
       </c>
-      <c r="E74" s="57"/>
-      <c r="F74" s="58"/>
+      <c r="E74" s="58"/>
+      <c r="F74" s="57"/>
       <c r="G74" s="9"/>
       <c r="H74" s="9"/>
       <c r="I74" s="9"/>
@@ -10861,18 +10861,18 @@
       <c r="Z74" s="9"/>
     </row>
     <row r="75" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="71"/>
+      <c r="A75" s="74"/>
       <c r="B75" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C75" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D75" s="98">
+      <c r="D75" s="61">
         <v>67</v>
       </c>
-      <c r="E75" s="57"/>
-      <c r="F75" s="58"/>
+      <c r="E75" s="58"/>
+      <c r="F75" s="57"/>
       <c r="G75" s="9"/>
       <c r="H75" s="9"/>
       <c r="I75" s="9"/>
@@ -10895,18 +10895,18 @@
       <c r="Z75" s="9"/>
     </row>
     <row r="76" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="71"/>
+      <c r="A76" s="74"/>
       <c r="B76" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C76" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="D76" s="98">
+      <c r="D76" s="61">
         <v>67</v>
       </c>
-      <c r="E76" s="57"/>
-      <c r="F76" s="58"/>
+      <c r="E76" s="58"/>
+      <c r="F76" s="57"/>
       <c r="G76" s="9"/>
       <c r="H76" s="9"/>
       <c r="I76" s="9"/>
@@ -10929,18 +10929,18 @@
       <c r="Z76" s="9"/>
     </row>
     <row r="77" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="72"/>
+      <c r="A77" s="75"/>
       <c r="B77" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C77" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D77" s="75" t="s">
+      <c r="D77" s="62" t="s">
         <v>1969</v>
       </c>
-      <c r="E77" s="57"/>
-      <c r="F77" s="58"/>
+      <c r="E77" s="58"/>
+      <c r="F77" s="57"/>
       <c r="G77" s="9"/>
       <c r="H77" s="9"/>
       <c r="I77" s="9"/>
@@ -10963,7 +10963,7 @@
       <c r="Z77" s="9"/>
     </row>
     <row r="78" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="70">
+      <c r="A78" s="73">
         <v>28</v>
       </c>
       <c r="B78" s="19" t="s">
@@ -10971,8 +10971,8 @@
       </c>
       <c r="C78" s="19"/>
       <c r="D78" s="60"/>
-      <c r="E78" s="57"/>
-      <c r="F78" s="58"/>
+      <c r="E78" s="58"/>
+      <c r="F78" s="57"/>
       <c r="G78" s="9"/>
       <c r="H78" s="9"/>
       <c r="I78" s="9"/>
@@ -10995,18 +10995,18 @@
       <c r="Z78" s="9"/>
     </row>
     <row r="79" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="71"/>
+      <c r="A79" s="74"/>
       <c r="B79" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C79" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="D79" s="98">
+      <c r="D79" s="61">
         <v>67</v>
       </c>
-      <c r="E79" s="57"/>
-      <c r="F79" s="58"/>
+      <c r="E79" s="58"/>
+      <c r="F79" s="57"/>
       <c r="G79" s="9"/>
       <c r="H79" s="9"/>
       <c r="I79" s="9"/>
@@ -11029,18 +11029,18 @@
       <c r="Z79" s="9"/>
     </row>
     <row r="80" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="71"/>
+      <c r="A80" s="74"/>
       <c r="B80" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C80" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="D80" s="98">
+      <c r="D80" s="61">
         <v>67</v>
       </c>
-      <c r="E80" s="57"/>
-      <c r="F80" s="58"/>
+      <c r="E80" s="58"/>
+      <c r="F80" s="57"/>
       <c r="G80" s="9"/>
       <c r="H80" s="9"/>
       <c r="I80" s="9"/>
@@ -11063,18 +11063,18 @@
       <c r="Z80" s="9"/>
     </row>
     <row r="81" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="71"/>
+      <c r="A81" s="74"/>
       <c r="B81" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C81" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="D81" s="98">
+      <c r="D81" s="61">
         <v>67</v>
       </c>
-      <c r="E81" s="57"/>
-      <c r="F81" s="58"/>
+      <c r="E81" s="58"/>
+      <c r="F81" s="57"/>
       <c r="G81" s="9"/>
       <c r="H81" s="9"/>
       <c r="I81" s="9"/>
@@ -11097,18 +11097,18 @@
       <c r="Z81" s="9"/>
     </row>
     <row r="82" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="71"/>
+      <c r="A82" s="74"/>
       <c r="B82" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C82" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="D82" s="75" t="s">
+      <c r="D82" s="62" t="s">
         <v>1970</v>
       </c>
-      <c r="E82" s="57"/>
-      <c r="F82" s="58"/>
+      <c r="E82" s="58"/>
+      <c r="F82" s="57"/>
       <c r="G82" s="9"/>
       <c r="H82" s="9"/>
       <c r="I82" s="9"/>
@@ -11131,18 +11131,18 @@
       <c r="Z82" s="9"/>
     </row>
     <row r="83" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="71"/>
+      <c r="A83" s="74"/>
       <c r="B83" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C83" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="D83" s="98">
+      <c r="D83" s="61">
         <v>67</v>
       </c>
-      <c r="E83" s="57"/>
-      <c r="F83" s="58"/>
+      <c r="E83" s="58"/>
+      <c r="F83" s="57"/>
       <c r="G83" s="9"/>
       <c r="H83" s="9"/>
       <c r="I83" s="9"/>
@@ -11165,18 +11165,18 @@
       <c r="Z83" s="9"/>
     </row>
     <row r="84" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="72"/>
+      <c r="A84" s="75"/>
       <c r="B84" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C84" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D84" s="75" t="s">
+      <c r="D84" s="62" t="s">
         <v>1971</v>
       </c>
-      <c r="E84" s="57"/>
-      <c r="F84" s="58"/>
+      <c r="E84" s="58"/>
+      <c r="F84" s="57"/>
       <c r="G84" s="9"/>
       <c r="H84" s="9"/>
       <c r="I84" s="9"/>
@@ -11206,11 +11206,11 @@
         <v>71</v>
       </c>
       <c r="C85" s="19"/>
-      <c r="D85" s="75" t="s">
+      <c r="D85" s="62" t="s">
         <v>1972</v>
       </c>
-      <c r="E85" s="57"/>
-      <c r="F85" s="58"/>
+      <c r="E85" s="58"/>
+      <c r="F85" s="57"/>
       <c r="G85" s="9"/>
       <c r="H85" s="9"/>
       <c r="I85" s="9"/>
@@ -11297,7 +11297,7 @@
       <c r="Z87" s="9"/>
     </row>
     <row r="88" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="70">
+      <c r="A88" s="73">
         <v>30</v>
       </c>
       <c r="B88" s="24" t="s">
@@ -11308,7 +11308,7 @@
         <v>0.92500000000000004</v>
       </c>
       <c r="E88" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F88" s="52" t="s">
         <v>1973</v>
@@ -11335,7 +11335,7 @@
       <c r="Z88" s="9"/>
     </row>
     <row r="89" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="71"/>
+      <c r="A89" s="74"/>
       <c r="B89" s="24" t="s">
         <v>77</v>
       </c>
@@ -11344,7 +11344,7 @@
         <v>0.96666666666666667</v>
       </c>
       <c r="E89" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F89" s="52" t="s">
         <v>1973</v>
@@ -11371,7 +11371,7 @@
       <c r="Z89" s="9"/>
     </row>
     <row r="90" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="71"/>
+      <c r="A90" s="74"/>
       <c r="B90" s="24" t="s">
         <v>78</v>
       </c>
@@ -11380,7 +11380,7 @@
         <v>1.5972222222222221E-2</v>
       </c>
       <c r="E90" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F90" s="52" t="s">
         <v>1973</v>
@@ -11407,7 +11407,7 @@
       <c r="Z90" s="9"/>
     </row>
     <row r="91" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="71"/>
+      <c r="A91" s="74"/>
       <c r="B91" s="24" t="s">
         <v>79</v>
       </c>
@@ -11416,7 +11416,7 @@
         <v>4.8611111111111112E-2</v>
       </c>
       <c r="E91" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F91" s="52" t="s">
         <v>1973</v>
@@ -11443,7 +11443,7 @@
       <c r="Z91" s="9"/>
     </row>
     <row r="92" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="71"/>
+      <c r="A92" s="74"/>
       <c r="B92" s="24" t="s">
         <v>80</v>
       </c>
@@ -11452,7 +11452,7 @@
         <v>4.9305555555555554E-2</v>
       </c>
       <c r="E92" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F92" s="52" t="s">
         <v>1973</v>
@@ -11479,7 +11479,7 @@
       <c r="Z92" s="9"/>
     </row>
     <row r="93" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="71"/>
+      <c r="A93" s="74"/>
       <c r="B93" s="24" t="s">
         <v>81</v>
       </c>
@@ -11488,7 +11488,7 @@
         <v>0.05</v>
       </c>
       <c r="E93" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F93" s="52" t="s">
         <v>1973</v>
@@ -11515,7 +11515,7 @@
       <c r="Z93" s="9"/>
     </row>
     <row r="94" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="71"/>
+      <c r="A94" s="74"/>
       <c r="B94" s="24" t="s">
         <v>82</v>
       </c>
@@ -11524,7 +11524,7 @@
         <v>5.1388888888888887E-2</v>
       </c>
       <c r="E94" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F94" s="52" t="s">
         <v>1973</v>
@@ -11551,7 +11551,7 @@
       <c r="Z94" s="9"/>
     </row>
     <row r="95" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="71"/>
+      <c r="A95" s="74"/>
       <c r="B95" s="24" t="s">
         <v>83</v>
       </c>
@@ -11560,7 +11560,7 @@
         <v>5.2083333333333336E-2</v>
       </c>
       <c r="E95" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F95" s="52" t="s">
         <v>1973</v>
@@ -11587,7 +11587,7 @@
       <c r="Z95" s="9"/>
     </row>
     <row r="96" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="71"/>
+      <c r="A96" s="74"/>
       <c r="B96" s="24" t="s">
         <v>84</v>
       </c>
@@ -11596,7 +11596,7 @@
         <v>5.2777777777777778E-2</v>
       </c>
       <c r="E96" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F96" s="52" t="s">
         <v>1973</v>
@@ -11623,7 +11623,7 @@
       <c r="Z96" s="9"/>
     </row>
     <row r="97" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="71"/>
+      <c r="A97" s="74"/>
       <c r="B97" s="24" t="s">
         <v>85</v>
       </c>
@@ -11632,7 +11632,7 @@
         <v>5.347222222222222E-2</v>
       </c>
       <c r="E97" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F97" s="52" t="s">
         <v>1973</v>
@@ -11659,7 +11659,7 @@
       <c r="Z97" s="9"/>
     </row>
     <row r="98" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="71"/>
+      <c r="A98" s="74"/>
       <c r="B98" s="24" t="s">
         <v>86</v>
       </c>
@@ -11668,7 +11668,7 @@
         <v>6.1805555555555558E-2</v>
       </c>
       <c r="E98" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F98" s="52" t="s">
         <v>1973</v>
@@ -11695,7 +11695,7 @@
       <c r="Z98" s="9"/>
     </row>
     <row r="99" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="71"/>
+      <c r="A99" s="74"/>
       <c r="B99" s="25" t="s">
         <v>87</v>
       </c>
@@ -11704,7 +11704,7 @@
         <v>9.8611111111111108E-2</v>
       </c>
       <c r="E99" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F99" s="52" t="s">
         <v>1973</v>
@@ -11731,7 +11731,7 @@
       <c r="Z99" s="9"/>
     </row>
     <row r="100" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="72"/>
+      <c r="A100" s="75"/>
       <c r="B100" s="25" t="s">
         <v>88</v>
       </c>
@@ -11740,7 +11740,7 @@
         <v>0.13194444444444445</v>
       </c>
       <c r="E100" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F100" s="52" t="s">
         <v>1973</v>
@@ -11767,16 +11767,16 @@
       <c r="Z100" s="9"/>
     </row>
     <row r="101" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="70">
+      <c r="A101" s="73">
         <v>31</v>
       </c>
-      <c r="B101" s="59" t="s">
+      <c r="B101" s="96" t="s">
         <v>89</v>
       </c>
-      <c r="C101" s="58"/>
-      <c r="D101" s="106"/>
-      <c r="E101" s="57"/>
-      <c r="F101" s="58"/>
+      <c r="C101" s="57"/>
+      <c r="D101" s="63"/>
+      <c r="E101" s="58"/>
+      <c r="F101" s="57"/>
       <c r="G101" s="9"/>
       <c r="H101" s="9"/>
       <c r="I101" s="9"/>
@@ -11799,18 +11799,18 @@
       <c r="Z101" s="9"/>
     </row>
     <row r="102" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="71"/>
+      <c r="A102" s="74"/>
       <c r="B102" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C102" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="D102" s="105" t="s">
+      <c r="D102" s="64" t="s">
         <v>1974</v>
       </c>
-      <c r="E102" s="57"/>
-      <c r="F102" s="58"/>
+      <c r="E102" s="58"/>
+      <c r="F102" s="57"/>
       <c r="G102" s="9"/>
       <c r="H102" s="9"/>
       <c r="I102" s="9"/>
@@ -11833,14 +11833,14 @@
       <c r="Z102" s="9"/>
     </row>
     <row r="103" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="72"/>
+      <c r="A103" s="75"/>
       <c r="B103" s="19"/>
       <c r="C103" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="D103" s="106"/>
-      <c r="E103" s="57"/>
-      <c r="F103" s="58"/>
+      <c r="D103" s="63"/>
+      <c r="E103" s="58"/>
+      <c r="F103" s="57"/>
       <c r="G103" s="9"/>
       <c r="H103" s="9"/>
       <c r="I103" s="9"/>
@@ -11925,7 +11925,7 @@
       <c r="Z105" s="9"/>
     </row>
     <row r="106" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="70">
+      <c r="A106" s="73">
         <v>32</v>
       </c>
       <c r="B106" s="19"/>
@@ -11961,7 +11961,7 @@
       <c r="Z106" s="9"/>
     </row>
     <row r="107" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="71"/>
+      <c r="A107" s="74"/>
       <c r="B107" s="19"/>
       <c r="C107" s="17" t="s">
         <v>96</v>
@@ -11995,7 +11995,7 @@
       <c r="Z107" s="9"/>
     </row>
     <row r="108" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="71"/>
+      <c r="A108" s="74"/>
       <c r="B108" s="19"/>
       <c r="C108" s="17" t="s">
         <v>97</v>
@@ -12029,7 +12029,7 @@
       <c r="Z108" s="9"/>
     </row>
     <row r="109" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="71"/>
+      <c r="A109" s="74"/>
       <c r="B109" s="19"/>
       <c r="C109" s="17" t="s">
         <v>98</v>
@@ -12063,7 +12063,7 @@
       <c r="Z109" s="9"/>
     </row>
     <row r="110" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="71"/>
+      <c r="A110" s="74"/>
       <c r="B110" s="19"/>
       <c r="C110" s="17" t="s">
         <v>99</v>
@@ -12097,7 +12097,7 @@
       <c r="Z110" s="9"/>
     </row>
     <row r="111" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="72"/>
+      <c r="A111" s="75"/>
       <c r="B111" s="19"/>
       <c r="C111" s="17" t="s">
         <v>100</v>
@@ -12164,11 +12164,11 @@
       </c>
       <c r="B113" s="8"/>
       <c r="C113" s="9"/>
-      <c r="D113" s="106" t="s">
+      <c r="D113" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="E113" s="57"/>
-      <c r="F113" s="58"/>
+      <c r="E113" s="58"/>
+      <c r="F113" s="57"/>
       <c r="G113" s="9"/>
       <c r="H113" s="9"/>
       <c r="I113" s="9"/>
@@ -12191,18 +12191,18 @@
       <c r="Z113" s="9"/>
     </row>
     <row r="114" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="70">
+      <c r="A114" s="73">
         <v>33</v>
       </c>
       <c r="B114" s="19" t="s">
         <v>103</v>
       </c>
       <c r="C114" s="19"/>
-      <c r="D114" s="105" t="s">
+      <c r="D114" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E114" s="57"/>
-      <c r="F114" s="58"/>
+      <c r="E114" s="58"/>
+      <c r="F114" s="57"/>
       <c r="G114" s="9"/>
       <c r="H114" s="9"/>
       <c r="I114" s="9"/>
@@ -12225,16 +12225,16 @@
       <c r="Z114" s="9"/>
     </row>
     <row r="115" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="71"/>
+      <c r="A115" s="74"/>
       <c r="B115" s="19" t="s">
         <v>104</v>
       </c>
       <c r="C115" s="19"/>
-      <c r="D115" s="105" t="s">
+      <c r="D115" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E115" s="57"/>
-      <c r="F115" s="58"/>
+      <c r="E115" s="58"/>
+      <c r="F115" s="57"/>
       <c r="G115" s="9"/>
       <c r="H115" s="9"/>
       <c r="I115" s="9"/>
@@ -12257,16 +12257,16 @@
       <c r="Z115" s="9"/>
     </row>
     <row r="116" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="71"/>
+      <c r="A116" s="74"/>
       <c r="B116" s="19" t="s">
         <v>105</v>
       </c>
       <c r="C116" s="19"/>
-      <c r="D116" s="105" t="s">
+      <c r="D116" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E116" s="57"/>
-      <c r="F116" s="58"/>
+      <c r="E116" s="58"/>
+      <c r="F116" s="57"/>
       <c r="G116" s="9"/>
       <c r="H116" s="9"/>
       <c r="I116" s="9"/>
@@ -12289,16 +12289,16 @@
       <c r="Z116" s="9"/>
     </row>
     <row r="117" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="71"/>
+      <c r="A117" s="74"/>
       <c r="B117" s="19" t="s">
         <v>106</v>
       </c>
       <c r="C117" s="19"/>
-      <c r="D117" s="105" t="s">
+      <c r="D117" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E117" s="57"/>
-      <c r="F117" s="58"/>
+      <c r="E117" s="58"/>
+      <c r="F117" s="57"/>
       <c r="G117" s="9"/>
       <c r="H117" s="9"/>
       <c r="I117" s="9"/>
@@ -12321,16 +12321,16 @@
       <c r="Z117" s="9"/>
     </row>
     <row r="118" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="71"/>
+      <c r="A118" s="74"/>
       <c r="B118" s="19" t="s">
         <v>107</v>
       </c>
       <c r="C118" s="19"/>
-      <c r="D118" s="105" t="s">
+      <c r="D118" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E118" s="57"/>
-      <c r="F118" s="58"/>
+      <c r="E118" s="58"/>
+      <c r="F118" s="57"/>
       <c r="G118" s="9"/>
       <c r="H118" s="9"/>
       <c r="I118" s="9"/>
@@ -12353,16 +12353,16 @@
       <c r="Z118" s="9"/>
     </row>
     <row r="119" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="71"/>
+      <c r="A119" s="74"/>
       <c r="B119" s="19" t="s">
         <v>108</v>
       </c>
       <c r="C119" s="19"/>
-      <c r="D119" s="105" t="s">
+      <c r="D119" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E119" s="57"/>
-      <c r="F119" s="58"/>
+      <c r="E119" s="58"/>
+      <c r="F119" s="57"/>
       <c r="G119" s="9"/>
       <c r="H119" s="9"/>
       <c r="I119" s="9"/>
@@ -12385,16 +12385,16 @@
       <c r="Z119" s="9"/>
     </row>
     <row r="120" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="71"/>
+      <c r="A120" s="74"/>
       <c r="B120" s="19" t="s">
         <v>109</v>
       </c>
       <c r="C120" s="19"/>
-      <c r="D120" s="105" t="s">
+      <c r="D120" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E120" s="57"/>
-      <c r="F120" s="58"/>
+      <c r="E120" s="58"/>
+      <c r="F120" s="57"/>
       <c r="G120" s="9"/>
       <c r="H120" s="9"/>
       <c r="I120" s="9"/>
@@ -12417,16 +12417,16 @@
       <c r="Z120" s="9"/>
     </row>
     <row r="121" spans="1:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="72"/>
-      <c r="B121" s="81" t="s">
+      <c r="A121" s="75"/>
+      <c r="B121" s="97" t="s">
         <v>110</v>
       </c>
-      <c r="C121" s="58"/>
-      <c r="D121" s="105" t="s">
+      <c r="C121" s="57"/>
+      <c r="D121" s="64" t="s">
         <v>1976</v>
       </c>
-      <c r="E121" s="57"/>
-      <c r="F121" s="58"/>
+      <c r="E121" s="58"/>
+      <c r="F121" s="57"/>
       <c r="G121" s="9"/>
       <c r="H121" s="9"/>
       <c r="I121" s="9"/>
@@ -12477,16 +12477,16 @@
       <c r="Z122" s="9"/>
     </row>
     <row r="123" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="74" t="s">
+      <c r="A123" s="105" t="s">
         <v>111</v>
       </c>
-      <c r="B123" s="68"/>
-      <c r="C123" s="68"/>
-      <c r="D123" s="69"/>
-      <c r="E123" s="106" t="s">
+      <c r="B123" s="86"/>
+      <c r="C123" s="86"/>
+      <c r="D123" s="87"/>
+      <c r="E123" s="63" t="s">
         <v>112</v>
       </c>
-      <c r="F123" s="58"/>
+      <c r="F123" s="57"/>
       <c r="G123" s="9"/>
       <c r="H123" s="9"/>
       <c r="I123" s="9"/>
@@ -12509,18 +12509,18 @@
       <c r="Z123" s="9"/>
     </row>
     <row r="124" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="70">
+      <c r="A124" s="73">
         <v>34</v>
       </c>
-      <c r="B124" s="75" t="s">
+      <c r="B124" s="62" t="s">
         <v>1977</v>
       </c>
-      <c r="C124" s="57"/>
-      <c r="D124" s="58"/>
-      <c r="E124" s="76" t="s">
+      <c r="C124" s="58"/>
+      <c r="D124" s="57"/>
+      <c r="E124" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F124" s="58"/>
+      <c r="F124" s="57"/>
       <c r="G124" s="9"/>
       <c r="H124" s="9"/>
       <c r="I124" s="9"/>
@@ -12543,16 +12543,16 @@
       <c r="Z124" s="9"/>
     </row>
     <row r="125" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="71"/>
-      <c r="B125" s="75" t="s">
+      <c r="A125" s="74"/>
+      <c r="B125" s="62" t="s">
         <v>1965</v>
       </c>
-      <c r="C125" s="57"/>
-      <c r="D125" s="58"/>
-      <c r="E125" s="76" t="s">
+      <c r="C125" s="58"/>
+      <c r="D125" s="57"/>
+      <c r="E125" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F125" s="58"/>
+      <c r="F125" s="57"/>
       <c r="G125" s="9"/>
       <c r="H125" s="9"/>
       <c r="I125" s="9"/>
@@ -12575,16 +12575,16 @@
       <c r="Z125" s="9"/>
     </row>
     <row r="126" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="71"/>
-      <c r="B126" s="75" t="s">
+      <c r="A126" s="74"/>
+      <c r="B126" s="62" t="s">
         <v>1978</v>
       </c>
-      <c r="C126" s="57"/>
-      <c r="D126" s="58"/>
-      <c r="E126" s="76" t="s">
+      <c r="C126" s="58"/>
+      <c r="D126" s="57"/>
+      <c r="E126" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F126" s="58"/>
+      <c r="F126" s="57"/>
       <c r="G126" s="9"/>
       <c r="H126" s="9"/>
       <c r="I126" s="9"/>
@@ -12607,16 +12607,16 @@
       <c r="Z126" s="9"/>
     </row>
     <row r="127" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="71"/>
-      <c r="B127" s="76" t="s">
+      <c r="A127" s="74"/>
+      <c r="B127" s="56" t="s">
         <v>1979</v>
       </c>
-      <c r="C127" s="77"/>
-      <c r="D127" s="78"/>
-      <c r="E127" s="76" t="s">
+      <c r="C127" s="106"/>
+      <c r="D127" s="107"/>
+      <c r="E127" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F127" s="58"/>
+      <c r="F127" s="57"/>
       <c r="G127" s="9"/>
       <c r="H127" s="9"/>
       <c r="I127" s="9"/>
@@ -12639,12 +12639,12 @@
       <c r="Z127" s="9"/>
     </row>
     <row r="128" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="71"/>
+      <c r="A128" s="74"/>
       <c r="B128" s="60"/>
-      <c r="C128" s="57"/>
-      <c r="D128" s="58"/>
+      <c r="C128" s="58"/>
+      <c r="D128" s="57"/>
       <c r="E128" s="60"/>
-      <c r="F128" s="58"/>
+      <c r="F128" s="57"/>
       <c r="G128" s="9"/>
       <c r="H128" s="9"/>
       <c r="I128" s="9"/>
@@ -12667,12 +12667,12 @@
       <c r="Z128" s="9"/>
     </row>
     <row r="129" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="71"/>
+      <c r="A129" s="74"/>
       <c r="B129" s="60"/>
-      <c r="C129" s="57"/>
-      <c r="D129" s="58"/>
+      <c r="C129" s="58"/>
+      <c r="D129" s="57"/>
       <c r="E129" s="60"/>
-      <c r="F129" s="58"/>
+      <c r="F129" s="57"/>
       <c r="G129" s="9"/>
       <c r="H129" s="9"/>
       <c r="I129" s="9"/>
@@ -12695,12 +12695,12 @@
       <c r="Z129" s="9"/>
     </row>
     <row r="130" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="71"/>
+      <c r="A130" s="74"/>
       <c r="B130" s="60"/>
-      <c r="C130" s="57"/>
-      <c r="D130" s="58"/>
+      <c r="C130" s="58"/>
+      <c r="D130" s="57"/>
       <c r="E130" s="60"/>
-      <c r="F130" s="58"/>
+      <c r="F130" s="57"/>
       <c r="G130" s="9"/>
       <c r="H130" s="9"/>
       <c r="I130" s="9"/>
@@ -12723,12 +12723,12 @@
       <c r="Z130" s="9"/>
     </row>
     <row r="131" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="71"/>
+      <c r="A131" s="74"/>
       <c r="B131" s="60"/>
-      <c r="C131" s="57"/>
-      <c r="D131" s="58"/>
+      <c r="C131" s="58"/>
+      <c r="D131" s="57"/>
       <c r="E131" s="60"/>
-      <c r="F131" s="58"/>
+      <c r="F131" s="57"/>
       <c r="G131" s="9"/>
       <c r="H131" s="9"/>
       <c r="I131" s="9"/>
@@ -12751,12 +12751,12 @@
       <c r="Z131" s="9"/>
     </row>
     <row r="132" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="72"/>
+      <c r="A132" s="75"/>
       <c r="B132" s="60"/>
-      <c r="C132" s="57"/>
-      <c r="D132" s="58"/>
+      <c r="C132" s="58"/>
+      <c r="D132" s="57"/>
       <c r="E132" s="60"/>
-      <c r="F132" s="58"/>
+      <c r="F132" s="57"/>
       <c r="G132" s="9"/>
       <c r="H132" s="9"/>
       <c r="I132" s="9"/>
@@ -12837,14 +12837,14 @@
       <c r="Z134" s="9"/>
     </row>
     <row r="135" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="70">
+      <c r="A135" s="73">
         <v>35</v>
       </c>
-      <c r="B135" s="79"/>
-      <c r="C135" s="62"/>
-      <c r="D135" s="62"/>
-      <c r="E135" s="62"/>
-      <c r="F135" s="63"/>
+      <c r="B135" s="100"/>
+      <c r="C135" s="84"/>
+      <c r="D135" s="84"/>
+      <c r="E135" s="84"/>
+      <c r="F135" s="79"/>
       <c r="G135" s="9"/>
       <c r="H135" s="9"/>
       <c r="I135" s="9"/>
@@ -12867,12 +12867,12 @@
       <c r="Z135" s="9"/>
     </row>
     <row r="136" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="71"/>
-      <c r="B136" s="64"/>
-      <c r="C136" s="65"/>
-      <c r="D136" s="65"/>
-      <c r="E136" s="65"/>
-      <c r="F136" s="66"/>
+      <c r="A136" s="74"/>
+      <c r="B136" s="80"/>
+      <c r="C136" s="66"/>
+      <c r="D136" s="66"/>
+      <c r="E136" s="66"/>
+      <c r="F136" s="81"/>
       <c r="G136" s="9"/>
       <c r="H136" s="9"/>
       <c r="I136" s="9"/>
@@ -12895,12 +12895,12 @@
       <c r="Z136" s="9"/>
     </row>
     <row r="137" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="71"/>
-      <c r="B137" s="64"/>
-      <c r="C137" s="65"/>
-      <c r="D137" s="65"/>
-      <c r="E137" s="65"/>
-      <c r="F137" s="66"/>
+      <c r="A137" s="74"/>
+      <c r="B137" s="80"/>
+      <c r="C137" s="66"/>
+      <c r="D137" s="66"/>
+      <c r="E137" s="66"/>
+      <c r="F137" s="81"/>
       <c r="G137" s="9"/>
       <c r="H137" s="9"/>
       <c r="I137" s="9"/>
@@ -12923,12 +12923,12 @@
       <c r="Z137" s="9"/>
     </row>
     <row r="138" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="71"/>
-      <c r="B138" s="64"/>
-      <c r="C138" s="65"/>
-      <c r="D138" s="65"/>
-      <c r="E138" s="65"/>
-      <c r="F138" s="66"/>
+      <c r="A138" s="74"/>
+      <c r="B138" s="80"/>
+      <c r="C138" s="66"/>
+      <c r="D138" s="66"/>
+      <c r="E138" s="66"/>
+      <c r="F138" s="81"/>
       <c r="G138" s="9"/>
       <c r="H138" s="9"/>
       <c r="I138" s="9"/>
@@ -12951,12 +12951,12 @@
       <c r="Z138" s="9"/>
     </row>
     <row r="139" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="71"/>
-      <c r="B139" s="64"/>
-      <c r="C139" s="65"/>
-      <c r="D139" s="65"/>
-      <c r="E139" s="65"/>
-      <c r="F139" s="66"/>
+      <c r="A139" s="74"/>
+      <c r="B139" s="80"/>
+      <c r="C139" s="66"/>
+      <c r="D139" s="66"/>
+      <c r="E139" s="66"/>
+      <c r="F139" s="81"/>
       <c r="G139" s="9"/>
       <c r="H139" s="9"/>
       <c r="I139" s="9"/>
@@ -12979,12 +12979,12 @@
       <c r="Z139" s="9"/>
     </row>
     <row r="140" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="71"/>
-      <c r="B140" s="64"/>
-      <c r="C140" s="65"/>
-      <c r="D140" s="65"/>
-      <c r="E140" s="65"/>
-      <c r="F140" s="66"/>
+      <c r="A140" s="74"/>
+      <c r="B140" s="80"/>
+      <c r="C140" s="66"/>
+      <c r="D140" s="66"/>
+      <c r="E140" s="66"/>
+      <c r="F140" s="81"/>
       <c r="G140" s="9"/>
       <c r="H140" s="9"/>
       <c r="I140" s="9"/>
@@ -13007,12 +13007,12 @@
       <c r="Z140" s="9"/>
     </row>
     <row r="141" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="71"/>
-      <c r="B141" s="64"/>
-      <c r="C141" s="65"/>
-      <c r="D141" s="65"/>
-      <c r="E141" s="65"/>
-      <c r="F141" s="66"/>
+      <c r="A141" s="74"/>
+      <c r="B141" s="80"/>
+      <c r="C141" s="66"/>
+      <c r="D141" s="66"/>
+      <c r="E141" s="66"/>
+      <c r="F141" s="81"/>
       <c r="G141" s="9"/>
       <c r="H141" s="9"/>
       <c r="I141" s="9"/>
@@ -13035,12 +13035,12 @@
       <c r="Z141" s="9"/>
     </row>
     <row r="142" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="71"/>
-      <c r="B142" s="64"/>
-      <c r="C142" s="65"/>
-      <c r="D142" s="65"/>
-      <c r="E142" s="65"/>
-      <c r="F142" s="66"/>
+      <c r="A142" s="74"/>
+      <c r="B142" s="80"/>
+      <c r="C142" s="66"/>
+      <c r="D142" s="66"/>
+      <c r="E142" s="66"/>
+      <c r="F142" s="81"/>
       <c r="G142" s="9"/>
       <c r="H142" s="9"/>
       <c r="I142" s="9"/>
@@ -13063,12 +13063,12 @@
       <c r="Z142" s="9"/>
     </row>
     <row r="143" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A143" s="71"/>
-      <c r="B143" s="64"/>
-      <c r="C143" s="65"/>
-      <c r="D143" s="65"/>
-      <c r="E143" s="65"/>
-      <c r="F143" s="66"/>
+      <c r="A143" s="74"/>
+      <c r="B143" s="80"/>
+      <c r="C143" s="66"/>
+      <c r="D143" s="66"/>
+      <c r="E143" s="66"/>
+      <c r="F143" s="81"/>
       <c r="G143" s="9"/>
       <c r="H143" s="9"/>
       <c r="I143" s="9"/>
@@ -13091,12 +13091,12 @@
       <c r="Z143" s="9"/>
     </row>
     <row r="144" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="71"/>
-      <c r="B144" s="64"/>
-      <c r="C144" s="65"/>
-      <c r="D144" s="65"/>
-      <c r="E144" s="65"/>
-      <c r="F144" s="66"/>
+      <c r="A144" s="74"/>
+      <c r="B144" s="80"/>
+      <c r="C144" s="66"/>
+      <c r="D144" s="66"/>
+      <c r="E144" s="66"/>
+      <c r="F144" s="81"/>
       <c r="G144" s="9"/>
       <c r="H144" s="9"/>
       <c r="I144" s="9"/>
@@ -13119,12 +13119,12 @@
       <c r="Z144" s="9"/>
     </row>
     <row r="145" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="71"/>
-      <c r="B145" s="64"/>
-      <c r="C145" s="65"/>
-      <c r="D145" s="65"/>
-      <c r="E145" s="65"/>
-      <c r="F145" s="66"/>
+      <c r="A145" s="74"/>
+      <c r="B145" s="80"/>
+      <c r="C145" s="66"/>
+      <c r="D145" s="66"/>
+      <c r="E145" s="66"/>
+      <c r="F145" s="81"/>
       <c r="G145" s="9"/>
       <c r="H145" s="9"/>
       <c r="I145" s="9"/>
@@ -13147,12 +13147,12 @@
       <c r="Z145" s="9"/>
     </row>
     <row r="146" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="71"/>
-      <c r="B146" s="64"/>
-      <c r="C146" s="65"/>
-      <c r="D146" s="65"/>
-      <c r="E146" s="65"/>
-      <c r="F146" s="66"/>
+      <c r="A146" s="74"/>
+      <c r="B146" s="80"/>
+      <c r="C146" s="66"/>
+      <c r="D146" s="66"/>
+      <c r="E146" s="66"/>
+      <c r="F146" s="81"/>
       <c r="G146" s="9"/>
       <c r="H146" s="9"/>
       <c r="I146" s="9"/>
@@ -13175,12 +13175,12 @@
       <c r="Z146" s="9"/>
     </row>
     <row r="147" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="71"/>
-      <c r="B147" s="64"/>
-      <c r="C147" s="65"/>
-      <c r="D147" s="65"/>
-      <c r="E147" s="65"/>
-      <c r="F147" s="66"/>
+      <c r="A147" s="74"/>
+      <c r="B147" s="80"/>
+      <c r="C147" s="66"/>
+      <c r="D147" s="66"/>
+      <c r="E147" s="66"/>
+      <c r="F147" s="81"/>
       <c r="G147" s="9"/>
       <c r="H147" s="9"/>
       <c r="I147" s="9"/>
@@ -13203,12 +13203,12 @@
       <c r="Z147" s="9"/>
     </row>
     <row r="148" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="71"/>
-      <c r="B148" s="64"/>
-      <c r="C148" s="65"/>
-      <c r="D148" s="65"/>
-      <c r="E148" s="65"/>
-      <c r="F148" s="66"/>
+      <c r="A148" s="74"/>
+      <c r="B148" s="80"/>
+      <c r="C148" s="66"/>
+      <c r="D148" s="66"/>
+      <c r="E148" s="66"/>
+      <c r="F148" s="81"/>
       <c r="G148" s="9"/>
       <c r="H148" s="9"/>
       <c r="I148" s="9"/>
@@ -13231,12 +13231,12 @@
       <c r="Z148" s="9"/>
     </row>
     <row r="149" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="71"/>
-      <c r="B149" s="64"/>
-      <c r="C149" s="65"/>
-      <c r="D149" s="65"/>
-      <c r="E149" s="65"/>
-      <c r="F149" s="66"/>
+      <c r="A149" s="74"/>
+      <c r="B149" s="80"/>
+      <c r="C149" s="66"/>
+      <c r="D149" s="66"/>
+      <c r="E149" s="66"/>
+      <c r="F149" s="81"/>
       <c r="G149" s="9"/>
       <c r="H149" s="9"/>
       <c r="I149" s="9"/>
@@ -13259,12 +13259,12 @@
       <c r="Z149" s="9"/>
     </row>
     <row r="150" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="71"/>
-      <c r="B150" s="64"/>
-      <c r="C150" s="65"/>
-      <c r="D150" s="65"/>
-      <c r="E150" s="65"/>
-      <c r="F150" s="66"/>
+      <c r="A150" s="74"/>
+      <c r="B150" s="80"/>
+      <c r="C150" s="66"/>
+      <c r="D150" s="66"/>
+      <c r="E150" s="66"/>
+      <c r="F150" s="81"/>
       <c r="G150" s="9"/>
       <c r="H150" s="9"/>
       <c r="I150" s="9"/>
@@ -13287,12 +13287,12 @@
       <c r="Z150" s="9"/>
     </row>
     <row r="151" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="71"/>
-      <c r="B151" s="64"/>
-      <c r="C151" s="65"/>
-      <c r="D151" s="65"/>
-      <c r="E151" s="65"/>
-      <c r="F151" s="66"/>
+      <c r="A151" s="74"/>
+      <c r="B151" s="80"/>
+      <c r="C151" s="66"/>
+      <c r="D151" s="66"/>
+      <c r="E151" s="66"/>
+      <c r="F151" s="81"/>
       <c r="G151" s="9"/>
       <c r="H151" s="9"/>
       <c r="I151" s="9"/>
@@ -13315,12 +13315,12 @@
       <c r="Z151" s="9"/>
     </row>
     <row r="152" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="71"/>
-      <c r="B152" s="64"/>
-      <c r="C152" s="65"/>
-      <c r="D152" s="65"/>
-      <c r="E152" s="65"/>
-      <c r="F152" s="66"/>
+      <c r="A152" s="74"/>
+      <c r="B152" s="80"/>
+      <c r="C152" s="66"/>
+      <c r="D152" s="66"/>
+      <c r="E152" s="66"/>
+      <c r="F152" s="81"/>
       <c r="G152" s="9"/>
       <c r="H152" s="9"/>
       <c r="I152" s="9"/>
@@ -13343,12 +13343,12 @@
       <c r="Z152" s="9"/>
     </row>
     <row r="153" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="71"/>
-      <c r="B153" s="64"/>
-      <c r="C153" s="65"/>
-      <c r="D153" s="65"/>
-      <c r="E153" s="65"/>
-      <c r="F153" s="66"/>
+      <c r="A153" s="74"/>
+      <c r="B153" s="80"/>
+      <c r="C153" s="66"/>
+      <c r="D153" s="66"/>
+      <c r="E153" s="66"/>
+      <c r="F153" s="81"/>
       <c r="G153" s="9"/>
       <c r="H153" s="9"/>
       <c r="I153" s="9"/>
@@ -13371,12 +13371,12 @@
       <c r="Z153" s="9"/>
     </row>
     <row r="154" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="71"/>
-      <c r="B154" s="64"/>
-      <c r="C154" s="65"/>
-      <c r="D154" s="65"/>
-      <c r="E154" s="65"/>
-      <c r="F154" s="66"/>
+      <c r="A154" s="74"/>
+      <c r="B154" s="80"/>
+      <c r="C154" s="66"/>
+      <c r="D154" s="66"/>
+      <c r="E154" s="66"/>
+      <c r="F154" s="81"/>
       <c r="G154" s="9"/>
       <c r="H154" s="9"/>
       <c r="I154" s="9"/>
@@ -13399,12 +13399,12 @@
       <c r="Z154" s="9"/>
     </row>
     <row r="155" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="71"/>
-      <c r="B155" s="64"/>
-      <c r="C155" s="65"/>
-      <c r="D155" s="65"/>
-      <c r="E155" s="65"/>
-      <c r="F155" s="66"/>
+      <c r="A155" s="74"/>
+      <c r="B155" s="80"/>
+      <c r="C155" s="66"/>
+      <c r="D155" s="66"/>
+      <c r="E155" s="66"/>
+      <c r="F155" s="81"/>
       <c r="G155" s="9"/>
       <c r="H155" s="9"/>
       <c r="I155" s="9"/>
@@ -13427,12 +13427,12 @@
       <c r="Z155" s="9"/>
     </row>
     <row r="156" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="71"/>
-      <c r="B156" s="64"/>
-      <c r="C156" s="65"/>
-      <c r="D156" s="65"/>
-      <c r="E156" s="65"/>
-      <c r="F156" s="66"/>
+      <c r="A156" s="74"/>
+      <c r="B156" s="80"/>
+      <c r="C156" s="66"/>
+      <c r="D156" s="66"/>
+      <c r="E156" s="66"/>
+      <c r="F156" s="81"/>
       <c r="G156" s="9"/>
       <c r="H156" s="9"/>
       <c r="I156" s="9"/>
@@ -13455,12 +13455,12 @@
       <c r="Z156" s="9"/>
     </row>
     <row r="157" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="72"/>
-      <c r="B157" s="67"/>
-      <c r="C157" s="68"/>
-      <c r="D157" s="68"/>
-      <c r="E157" s="68"/>
-      <c r="F157" s="69"/>
+      <c r="A157" s="75"/>
+      <c r="B157" s="85"/>
+      <c r="C157" s="86"/>
+      <c r="D157" s="86"/>
+      <c r="E157" s="86"/>
+      <c r="F157" s="87"/>
       <c r="G157" s="9"/>
       <c r="H157" s="9"/>
       <c r="I157" s="9"/>
@@ -13541,16 +13541,16 @@
       <c r="Z159" s="9"/>
     </row>
     <row r="160" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="70">
+      <c r="A160" s="73">
         <v>36</v>
       </c>
-      <c r="B160" s="86" t="s">
+      <c r="B160" s="82" t="s">
         <v>115</v>
       </c>
-      <c r="C160" s="57"/>
-      <c r="D160" s="57"/>
-      <c r="E160" s="57"/>
-      <c r="F160" s="58"/>
+      <c r="C160" s="58"/>
+      <c r="D160" s="58"/>
+      <c r="E160" s="58"/>
+      <c r="F160" s="57"/>
       <c r="G160" s="9"/>
       <c r="H160" s="9"/>
       <c r="I160" s="9"/>
@@ -13573,14 +13573,14 @@
       <c r="Z160" s="9"/>
     </row>
     <row r="161" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="71"/>
-      <c r="B161" s="87" t="s">
+      <c r="A161" s="74"/>
+      <c r="B161" s="83" t="s">
         <v>1981</v>
       </c>
-      <c r="C161" s="62"/>
-      <c r="D161" s="62"/>
-      <c r="E161" s="62"/>
-      <c r="F161" s="63"/>
+      <c r="C161" s="84"/>
+      <c r="D161" s="84"/>
+      <c r="E161" s="84"/>
+      <c r="F161" s="79"/>
       <c r="G161" s="9"/>
       <c r="H161" s="9"/>
       <c r="I161" s="9"/>
@@ -13603,12 +13603,12 @@
       <c r="Z161" s="9"/>
     </row>
     <row r="162" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="71"/>
-      <c r="B162" s="67"/>
-      <c r="C162" s="68"/>
-      <c r="D162" s="68"/>
-      <c r="E162" s="68"/>
-      <c r="F162" s="69"/>
+      <c r="A162" s="74"/>
+      <c r="B162" s="85"/>
+      <c r="C162" s="86"/>
+      <c r="D162" s="86"/>
+      <c r="E162" s="86"/>
+      <c r="F162" s="87"/>
       <c r="G162" s="9"/>
       <c r="H162" s="9"/>
       <c r="I162" s="9"/>
@@ -13631,12 +13631,12 @@
       <c r="Z162" s="9"/>
     </row>
     <row r="163" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A163" s="71"/>
+      <c r="A163" s="74"/>
       <c r="B163" s="88"/>
-      <c r="C163" s="57"/>
-      <c r="D163" s="57"/>
-      <c r="E163" s="57"/>
-      <c r="F163" s="58"/>
+      <c r="C163" s="58"/>
+      <c r="D163" s="58"/>
+      <c r="E163" s="58"/>
+      <c r="F163" s="57"/>
       <c r="G163" s="9"/>
       <c r="H163" s="9"/>
       <c r="I163" s="9"/>
@@ -13659,14 +13659,14 @@
       <c r="Z163" s="9"/>
     </row>
     <row r="164" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A164" s="71"/>
-      <c r="B164" s="85" t="s">
+      <c r="A164" s="74"/>
+      <c r="B164" s="89" t="s">
         <v>116</v>
       </c>
-      <c r="C164" s="62"/>
-      <c r="D164" s="62"/>
-      <c r="E164" s="62"/>
-      <c r="F164" s="63"/>
+      <c r="C164" s="84"/>
+      <c r="D164" s="84"/>
+      <c r="E164" s="84"/>
+      <c r="F164" s="79"/>
       <c r="G164" s="9"/>
       <c r="H164" s="9"/>
       <c r="I164" s="9"/>
@@ -13689,12 +13689,12 @@
       <c r="Z164" s="9"/>
     </row>
     <row r="165" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A165" s="71"/>
-      <c r="B165" s="64"/>
-      <c r="C165" s="65"/>
-      <c r="D165" s="65"/>
-      <c r="E165" s="65"/>
-      <c r="F165" s="66"/>
+      <c r="A165" s="74"/>
+      <c r="B165" s="80"/>
+      <c r="C165" s="66"/>
+      <c r="D165" s="66"/>
+      <c r="E165" s="66"/>
+      <c r="F165" s="81"/>
       <c r="G165" s="9"/>
       <c r="H165" s="9"/>
       <c r="I165" s="9"/>
@@ -13717,12 +13717,12 @@
       <c r="Z165" s="9"/>
     </row>
     <row r="166" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="71"/>
-      <c r="B166" s="64"/>
-      <c r="C166" s="65"/>
-      <c r="D166" s="65"/>
-      <c r="E166" s="65"/>
-      <c r="F166" s="66"/>
+      <c r="A166" s="74"/>
+      <c r="B166" s="80"/>
+      <c r="C166" s="66"/>
+      <c r="D166" s="66"/>
+      <c r="E166" s="66"/>
+      <c r="F166" s="81"/>
       <c r="G166" s="9"/>
       <c r="H166" s="9"/>
       <c r="I166" s="9"/>
@@ -13745,12 +13745,12 @@
       <c r="Z166" s="9"/>
     </row>
     <row r="167" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="71"/>
-      <c r="B167" s="67"/>
-      <c r="C167" s="68"/>
-      <c r="D167" s="68"/>
-      <c r="E167" s="68"/>
-      <c r="F167" s="69"/>
+      <c r="A167" s="74"/>
+      <c r="B167" s="85"/>
+      <c r="C167" s="86"/>
+      <c r="D167" s="86"/>
+      <c r="E167" s="86"/>
+      <c r="F167" s="87"/>
       <c r="G167" s="9"/>
       <c r="H167" s="9"/>
       <c r="I167" s="9"/>
@@ -13773,7 +13773,7 @@
       <c r="Z167" s="9"/>
     </row>
     <row r="168" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="71"/>
+      <c r="A168" s="74"/>
       <c r="B168" s="47" t="s">
         <v>1982</v>
       </c>
@@ -13803,14 +13803,14 @@
       <c r="Z168" s="9"/>
     </row>
     <row r="169" spans="1:26" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A169" s="71"/>
-      <c r="B169" s="89" t="s">
+      <c r="A169" s="74"/>
+      <c r="B169" s="90" t="s">
         <v>1983</v>
       </c>
-      <c r="C169" s="57"/>
-      <c r="D169" s="57"/>
-      <c r="E169" s="57"/>
-      <c r="F169" s="58"/>
+      <c r="C169" s="58"/>
+      <c r="D169" s="58"/>
+      <c r="E169" s="58"/>
+      <c r="F169" s="57"/>
       <c r="G169" s="29"/>
       <c r="H169" s="29"/>
       <c r="I169" s="29"/>
@@ -13833,14 +13833,14 @@
       <c r="Z169" s="29"/>
     </row>
     <row r="170" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="71"/>
-      <c r="B170" s="90" t="s">
+      <c r="A170" s="74"/>
+      <c r="B170" s="91" t="s">
         <v>117</v>
       </c>
-      <c r="C170" s="57"/>
-      <c r="D170" s="57"/>
-      <c r="E170" s="57"/>
-      <c r="F170" s="58"/>
+      <c r="C170" s="58"/>
+      <c r="D170" s="58"/>
+      <c r="E170" s="58"/>
+      <c r="F170" s="57"/>
       <c r="G170" s="9"/>
       <c r="H170" s="9"/>
       <c r="I170" s="9"/>
@@ -13863,14 +13863,14 @@
       <c r="Z170" s="9"/>
     </row>
     <row r="171" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A171" s="71"/>
-      <c r="B171" s="85" t="s">
+      <c r="A171" s="74"/>
+      <c r="B171" s="89" t="s">
         <v>118</v>
       </c>
-      <c r="C171" s="62"/>
-      <c r="D171" s="62"/>
-      <c r="E171" s="62"/>
-      <c r="F171" s="63"/>
+      <c r="C171" s="84"/>
+      <c r="D171" s="84"/>
+      <c r="E171" s="84"/>
+      <c r="F171" s="79"/>
       <c r="G171" s="9"/>
       <c r="H171" s="9"/>
       <c r="I171" s="9"/>
@@ -13893,12 +13893,12 @@
       <c r="Z171" s="9"/>
     </row>
     <row r="172" spans="1:26" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A172" s="71"/>
-      <c r="B172" s="67"/>
-      <c r="C172" s="68"/>
-      <c r="D172" s="68"/>
-      <c r="E172" s="68"/>
-      <c r="F172" s="69"/>
+      <c r="A172" s="74"/>
+      <c r="B172" s="85"/>
+      <c r="C172" s="86"/>
+      <c r="D172" s="86"/>
+      <c r="E172" s="86"/>
+      <c r="F172" s="87"/>
       <c r="G172" s="9"/>
       <c r="H172" s="9"/>
       <c r="I172" s="9"/>
@@ -13921,7 +13921,7 @@
       <c r="Z172" s="9"/>
     </row>
     <row r="173" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="71"/>
+      <c r="A173" s="74"/>
       <c r="B173" s="19" t="s">
         <v>119</v>
       </c>
@@ -13951,14 +13951,14 @@
       <c r="Z173" s="9"/>
     </row>
     <row r="174" spans="1:26" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="71"/>
-      <c r="B174" s="56" t="s">
+      <c r="A174" s="74"/>
+      <c r="B174" s="102" t="s">
         <v>120</v>
       </c>
-      <c r="C174" s="57"/>
-      <c r="D174" s="57"/>
-      <c r="E174" s="57"/>
-      <c r="F174" s="58"/>
+      <c r="C174" s="58"/>
+      <c r="D174" s="58"/>
+      <c r="E174" s="58"/>
+      <c r="F174" s="57"/>
       <c r="G174" s="9"/>
       <c r="H174" s="9"/>
       <c r="I174" s="9"/>
@@ -13981,14 +13981,14 @@
       <c r="Z174" s="9"/>
     </row>
     <row r="175" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A175" s="71"/>
-      <c r="B175" s="59" t="s">
+      <c r="A175" s="74"/>
+      <c r="B175" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="C175" s="57"/>
-      <c r="D175" s="57"/>
-      <c r="E175" s="57"/>
-      <c r="F175" s="58"/>
+      <c r="C175" s="58"/>
+      <c r="D175" s="58"/>
+      <c r="E175" s="58"/>
+      <c r="F175" s="57"/>
       <c r="G175" s="9"/>
       <c r="H175" s="9"/>
       <c r="I175" s="9"/>
@@ -14011,14 +14011,14 @@
       <c r="Z175" s="9"/>
     </row>
     <row r="176" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A176" s="71"/>
-      <c r="B176" s="59" t="s">
+      <c r="A176" s="74"/>
+      <c r="B176" s="96" t="s">
         <v>122</v>
       </c>
-      <c r="C176" s="57"/>
-      <c r="D176" s="57"/>
-      <c r="E176" s="57"/>
-      <c r="F176" s="58"/>
+      <c r="C176" s="58"/>
+      <c r="D176" s="58"/>
+      <c r="E176" s="58"/>
+      <c r="F176" s="57"/>
       <c r="G176" s="9"/>
       <c r="H176" s="9"/>
       <c r="I176" s="9"/>
@@ -14041,12 +14041,12 @@
       <c r="Z176" s="9"/>
     </row>
     <row r="177" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A177" s="71"/>
+      <c r="A177" s="74"/>
       <c r="B177" s="60"/>
-      <c r="C177" s="57"/>
-      <c r="D177" s="57"/>
-      <c r="E177" s="57"/>
-      <c r="F177" s="58"/>
+      <c r="C177" s="58"/>
+      <c r="D177" s="58"/>
+      <c r="E177" s="58"/>
+      <c r="F177" s="57"/>
       <c r="G177" s="9"/>
       <c r="H177" s="9"/>
       <c r="I177" s="9"/>
@@ -14069,14 +14069,14 @@
       <c r="Z177" s="9"/>
     </row>
     <row r="178" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A178" s="71"/>
-      <c r="B178" s="85" t="s">
+      <c r="A178" s="74"/>
+      <c r="B178" s="89" t="s">
         <v>123</v>
       </c>
-      <c r="C178" s="62"/>
-      <c r="D178" s="62"/>
-      <c r="E178" s="62"/>
-      <c r="F178" s="63"/>
+      <c r="C178" s="84"/>
+      <c r="D178" s="84"/>
+      <c r="E178" s="84"/>
+      <c r="F178" s="79"/>
       <c r="G178" s="9"/>
       <c r="H178" s="9"/>
       <c r="I178" s="9"/>
@@ -14099,12 +14099,12 @@
       <c r="Z178" s="9"/>
     </row>
     <row r="179" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A179" s="71"/>
-      <c r="B179" s="67"/>
-      <c r="C179" s="68"/>
-      <c r="D179" s="68"/>
-      <c r="E179" s="68"/>
-      <c r="F179" s="69"/>
+      <c r="A179" s="74"/>
+      <c r="B179" s="85"/>
+      <c r="C179" s="86"/>
+      <c r="D179" s="86"/>
+      <c r="E179" s="86"/>
+      <c r="F179" s="87"/>
       <c r="G179" s="9"/>
       <c r="H179" s="9"/>
       <c r="I179" s="9"/>
@@ -14127,7 +14127,7 @@
       <c r="Z179" s="9"/>
     </row>
     <row r="180" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A180" s="71"/>
+      <c r="A180" s="74"/>
       <c r="B180" s="19" t="s">
         <v>124</v>
       </c>
@@ -14157,7 +14157,7 @@
       <c r="Z180" s="9"/>
     </row>
     <row r="181" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A181" s="71"/>
+      <c r="A181" s="74"/>
       <c r="B181" s="19" t="s">
         <v>125</v>
       </c>
@@ -14187,7 +14187,7 @@
       <c r="Z181" s="9"/>
     </row>
     <row r="182" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A182" s="71"/>
+      <c r="A182" s="74"/>
       <c r="B182" s="19" t="s">
         <v>126</v>
       </c>
@@ -14217,14 +14217,14 @@
       <c r="Z182" s="9"/>
     </row>
     <row r="183" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A183" s="71"/>
-      <c r="B183" s="59" t="s">
+      <c r="A183" s="74"/>
+      <c r="B183" s="96" t="s">
         <v>127</v>
       </c>
-      <c r="C183" s="57"/>
-      <c r="D183" s="57"/>
-      <c r="E183" s="57"/>
-      <c r="F183" s="58"/>
+      <c r="C183" s="58"/>
+      <c r="D183" s="58"/>
+      <c r="E183" s="58"/>
+      <c r="F183" s="57"/>
       <c r="G183" s="9"/>
       <c r="H183" s="9"/>
       <c r="I183" s="9"/>
@@ -14247,12 +14247,12 @@
       <c r="Z183" s="9"/>
     </row>
     <row r="184" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A184" s="71"/>
+      <c r="A184" s="74"/>
       <c r="B184" s="60"/>
-      <c r="C184" s="57"/>
-      <c r="D184" s="57"/>
-      <c r="E184" s="57"/>
-      <c r="F184" s="58"/>
+      <c r="C184" s="58"/>
+      <c r="D184" s="58"/>
+      <c r="E184" s="58"/>
+      <c r="F184" s="57"/>
       <c r="G184" s="9"/>
       <c r="H184" s="9"/>
       <c r="I184" s="9"/>
@@ -14275,14 +14275,14 @@
       <c r="Z184" s="9"/>
     </row>
     <row r="185" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A185" s="71"/>
-      <c r="B185" s="85" t="s">
+      <c r="A185" s="74"/>
+      <c r="B185" s="89" t="s">
         <v>128</v>
       </c>
-      <c r="C185" s="62"/>
-      <c r="D185" s="62"/>
-      <c r="E185" s="62"/>
-      <c r="F185" s="63"/>
+      <c r="C185" s="84"/>
+      <c r="D185" s="84"/>
+      <c r="E185" s="84"/>
+      <c r="F185" s="79"/>
       <c r="G185" s="9"/>
       <c r="H185" s="9"/>
       <c r="I185" s="9"/>
@@ -14305,12 +14305,12 @@
       <c r="Z185" s="9"/>
     </row>
     <row r="186" spans="1:26" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A186" s="71"/>
-      <c r="B186" s="67"/>
-      <c r="C186" s="68"/>
-      <c r="D186" s="68"/>
-      <c r="E186" s="68"/>
-      <c r="F186" s="69"/>
+      <c r="A186" s="74"/>
+      <c r="B186" s="85"/>
+      <c r="C186" s="86"/>
+      <c r="D186" s="86"/>
+      <c r="E186" s="86"/>
+      <c r="F186" s="87"/>
       <c r="G186" s="9"/>
       <c r="H186" s="9"/>
       <c r="I186" s="9"/>
@@ -14333,14 +14333,14 @@
       <c r="Z186" s="9"/>
     </row>
     <row r="187" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A187" s="71"/>
-      <c r="B187" s="59" t="s">
+      <c r="A187" s="74"/>
+      <c r="B187" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="C187" s="57"/>
-      <c r="D187" s="57"/>
-      <c r="E187" s="57"/>
-      <c r="F187" s="58"/>
+      <c r="C187" s="58"/>
+      <c r="D187" s="58"/>
+      <c r="E187" s="58"/>
+      <c r="F187" s="57"/>
       <c r="G187" s="9"/>
       <c r="H187" s="9"/>
       <c r="I187" s="9"/>
@@ -14363,12 +14363,12 @@
       <c r="Z187" s="9"/>
     </row>
     <row r="188" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A188" s="71"/>
-      <c r="B188" s="59"/>
-      <c r="C188" s="57"/>
-      <c r="D188" s="57"/>
-      <c r="E188" s="57"/>
-      <c r="F188" s="58"/>
+      <c r="A188" s="74"/>
+      <c r="B188" s="96"/>
+      <c r="C188" s="58"/>
+      <c r="D188" s="58"/>
+      <c r="E188" s="58"/>
+      <c r="F188" s="57"/>
       <c r="G188" s="9"/>
       <c r="H188" s="9"/>
       <c r="I188" s="9"/>
@@ -14391,14 +14391,14 @@
       <c r="Z188" s="9"/>
     </row>
     <row r="189" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A189" s="71"/>
-      <c r="B189" s="75" t="s">
+      <c r="A189" s="74"/>
+      <c r="B189" s="62" t="s">
         <v>1984</v>
       </c>
-      <c r="C189" s="57"/>
-      <c r="D189" s="57"/>
-      <c r="E189" s="57"/>
-      <c r="F189" s="58"/>
+      <c r="C189" s="58"/>
+      <c r="D189" s="58"/>
+      <c r="E189" s="58"/>
+      <c r="F189" s="57"/>
       <c r="G189" s="9"/>
       <c r="H189" s="9"/>
       <c r="I189" s="9"/>
@@ -14421,12 +14421,12 @@
       <c r="Z189" s="9"/>
     </row>
     <row r="190" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="71"/>
-      <c r="B190" s="59"/>
-      <c r="C190" s="57"/>
-      <c r="D190" s="57"/>
-      <c r="E190" s="57"/>
-      <c r="F190" s="58"/>
+      <c r="A190" s="74"/>
+      <c r="B190" s="96"/>
+      <c r="C190" s="58"/>
+      <c r="D190" s="58"/>
+      <c r="E190" s="58"/>
+      <c r="F190" s="57"/>
       <c r="G190" s="9"/>
       <c r="H190" s="9"/>
       <c r="I190" s="9"/>
@@ -14449,12 +14449,12 @@
       <c r="Z190" s="9"/>
     </row>
     <row r="191" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A191" s="71"/>
-      <c r="B191" s="59"/>
-      <c r="C191" s="57"/>
-      <c r="D191" s="57"/>
-      <c r="E191" s="57"/>
-      <c r="F191" s="58"/>
+      <c r="A191" s="74"/>
+      <c r="B191" s="96"/>
+      <c r="C191" s="58"/>
+      <c r="D191" s="58"/>
+      <c r="E191" s="58"/>
+      <c r="F191" s="57"/>
       <c r="G191" s="9"/>
       <c r="H191" s="9"/>
       <c r="I191" s="9"/>
@@ -14477,12 +14477,12 @@
       <c r="Z191" s="9"/>
     </row>
     <row r="192" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A192" s="72"/>
-      <c r="B192" s="59"/>
-      <c r="C192" s="57"/>
-      <c r="D192" s="57"/>
-      <c r="E192" s="57"/>
-      <c r="F192" s="58"/>
+      <c r="A192" s="75"/>
+      <c r="B192" s="96"/>
+      <c r="C192" s="58"/>
+      <c r="D192" s="58"/>
+      <c r="E192" s="58"/>
+      <c r="F192" s="57"/>
       <c r="G192" s="9"/>
       <c r="H192" s="9"/>
       <c r="I192" s="9"/>
@@ -14563,18 +14563,18 @@
       <c r="Z194" s="9"/>
     </row>
     <row r="195" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A195" s="70">
+      <c r="A195" s="73">
         <v>37</v>
       </c>
       <c r="B195" s="54" t="s">
         <v>1953</v>
       </c>
-      <c r="C195" s="59" t="s">
+      <c r="C195" s="96" t="s">
         <v>131</v>
       </c>
-      <c r="D195" s="57"/>
-      <c r="E195" s="57"/>
-      <c r="F195" s="58"/>
+      <c r="D195" s="58"/>
+      <c r="E195" s="58"/>
+      <c r="F195" s="57"/>
       <c r="G195" s="9"/>
       <c r="H195" s="9"/>
       <c r="I195" s="9"/>
@@ -14597,16 +14597,16 @@
       <c r="Z195" s="9"/>
     </row>
     <row r="196" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A196" s="71"/>
+      <c r="A196" s="74"/>
       <c r="B196" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C196" s="59" t="s">
+      <c r="C196" s="96" t="s">
         <v>132</v>
       </c>
-      <c r="D196" s="57"/>
-      <c r="E196" s="57"/>
-      <c r="F196" s="58"/>
+      <c r="D196" s="58"/>
+      <c r="E196" s="58"/>
+      <c r="F196" s="57"/>
       <c r="G196" s="9"/>
       <c r="H196" s="9"/>
       <c r="I196" s="9"/>
@@ -14629,16 +14629,16 @@
       <c r="Z196" s="9"/>
     </row>
     <row r="197" spans="1:26" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A197" s="71"/>
+      <c r="A197" s="74"/>
       <c r="B197" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C197" s="81" t="s">
+      <c r="C197" s="97" t="s">
         <v>133</v>
       </c>
-      <c r="D197" s="57"/>
-      <c r="E197" s="57"/>
-      <c r="F197" s="58"/>
+      <c r="D197" s="58"/>
+      <c r="E197" s="58"/>
+      <c r="F197" s="57"/>
       <c r="G197" s="9"/>
       <c r="H197" s="9"/>
       <c r="I197" s="9"/>
@@ -14661,16 +14661,16 @@
       <c r="Z197" s="9"/>
     </row>
     <row r="198" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A198" s="71"/>
+      <c r="A198" s="74"/>
       <c r="B198" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C198" s="59" t="s">
+      <c r="C198" s="96" t="s">
         <v>134</v>
       </c>
-      <c r="D198" s="57"/>
-      <c r="E198" s="57"/>
-      <c r="F198" s="58"/>
+      <c r="D198" s="58"/>
+      <c r="E198" s="58"/>
+      <c r="F198" s="57"/>
       <c r="G198" s="9"/>
       <c r="H198" s="9"/>
       <c r="I198" s="9"/>
@@ -14693,16 +14693,16 @@
       <c r="Z198" s="9"/>
     </row>
     <row r="199" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A199" s="71"/>
+      <c r="A199" s="74"/>
       <c r="B199" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C199" s="59" t="s">
+      <c r="C199" s="96" t="s">
         <v>135</v>
       </c>
-      <c r="D199" s="57"/>
-      <c r="E199" s="57"/>
-      <c r="F199" s="58"/>
+      <c r="D199" s="58"/>
+      <c r="E199" s="58"/>
+      <c r="F199" s="57"/>
       <c r="G199" s="9"/>
       <c r="H199" s="9"/>
       <c r="I199" s="9"/>
@@ -14725,16 +14725,16 @@
       <c r="Z199" s="9"/>
     </row>
     <row r="200" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="71"/>
+      <c r="A200" s="74"/>
       <c r="B200" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C200" s="59" t="s">
+      <c r="C200" s="96" t="s">
         <v>136</v>
       </c>
-      <c r="D200" s="57"/>
-      <c r="E200" s="57"/>
-      <c r="F200" s="58"/>
+      <c r="D200" s="58"/>
+      <c r="E200" s="58"/>
+      <c r="F200" s="57"/>
       <c r="G200" s="9"/>
       <c r="H200" s="9"/>
       <c r="I200" s="9"/>
@@ -14757,16 +14757,16 @@
       <c r="Z200" s="9"/>
     </row>
     <row r="201" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A201" s="71"/>
+      <c r="A201" s="74"/>
       <c r="B201" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C201" s="59" t="s">
+      <c r="C201" s="96" t="s">
         <v>137</v>
       </c>
-      <c r="D201" s="57"/>
-      <c r="E201" s="57"/>
-      <c r="F201" s="57"/>
+      <c r="D201" s="58"/>
+      <c r="E201" s="58"/>
+      <c r="F201" s="58"/>
       <c r="G201" s="9"/>
       <c r="H201" s="9"/>
       <c r="I201" s="9"/>
@@ -14789,16 +14789,16 @@
       <c r="Z201" s="9"/>
     </row>
     <row r="202" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A202" s="71"/>
+      <c r="A202" s="74"/>
       <c r="B202" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C202" s="59" t="s">
+      <c r="C202" s="96" t="s">
         <v>138</v>
       </c>
-      <c r="D202" s="57"/>
-      <c r="E202" s="57"/>
-      <c r="F202" s="58"/>
+      <c r="D202" s="58"/>
+      <c r="E202" s="58"/>
+      <c r="F202" s="57"/>
       <c r="G202" s="9"/>
       <c r="H202" s="9"/>
       <c r="I202" s="9"/>
@@ -14821,16 +14821,16 @@
       <c r="Z202" s="9"/>
     </row>
     <row r="203" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A203" s="71"/>
+      <c r="A203" s="74"/>
       <c r="B203" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C203" s="59" t="s">
+      <c r="C203" s="96" t="s">
         <v>139</v>
       </c>
-      <c r="D203" s="57"/>
-      <c r="E203" s="57"/>
-      <c r="F203" s="58"/>
+      <c r="D203" s="58"/>
+      <c r="E203" s="58"/>
+      <c r="F203" s="57"/>
       <c r="G203" s="9"/>
       <c r="H203" s="9"/>
       <c r="I203" s="9"/>
@@ -14853,16 +14853,16 @@
       <c r="Z203" s="9"/>
     </row>
     <row r="204" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A204" s="71"/>
+      <c r="A204" s="74"/>
       <c r="B204" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C204" s="59" t="s">
+      <c r="C204" s="96" t="s">
         <v>140</v>
       </c>
-      <c r="D204" s="57"/>
-      <c r="E204" s="57"/>
-      <c r="F204" s="58"/>
+      <c r="D204" s="58"/>
+      <c r="E204" s="58"/>
+      <c r="F204" s="57"/>
       <c r="G204" s="9"/>
       <c r="H204" s="9"/>
       <c r="I204" s="9"/>
@@ -14885,16 +14885,16 @@
       <c r="Z204" s="9"/>
     </row>
     <row r="205" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A205" s="71"/>
+      <c r="A205" s="74"/>
       <c r="B205" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C205" s="59" t="s">
+      <c r="C205" s="96" t="s">
         <v>141</v>
       </c>
-      <c r="D205" s="57"/>
-      <c r="E205" s="57"/>
-      <c r="F205" s="58"/>
+      <c r="D205" s="58"/>
+      <c r="E205" s="58"/>
+      <c r="F205" s="57"/>
       <c r="G205" s="9"/>
       <c r="H205" s="9"/>
       <c r="I205" s="9"/>
@@ -14917,16 +14917,16 @@
       <c r="Z205" s="9"/>
     </row>
     <row r="206" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A206" s="71"/>
+      <c r="A206" s="74"/>
       <c r="B206" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C206" s="59" t="s">
+      <c r="C206" s="96" t="s">
         <v>142</v>
       </c>
-      <c r="D206" s="57"/>
-      <c r="E206" s="57"/>
-      <c r="F206" s="58"/>
+      <c r="D206" s="58"/>
+      <c r="E206" s="58"/>
+      <c r="F206" s="57"/>
       <c r="G206" s="9"/>
       <c r="H206" s="9"/>
       <c r="I206" s="9"/>
@@ -14949,16 +14949,16 @@
       <c r="Z206" s="9"/>
     </row>
     <row r="207" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A207" s="71"/>
+      <c r="A207" s="74"/>
       <c r="B207" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C207" s="59" t="s">
+      <c r="C207" s="96" t="s">
         <v>143</v>
       </c>
-      <c r="D207" s="57"/>
-      <c r="E207" s="57"/>
-      <c r="F207" s="58"/>
+      <c r="D207" s="58"/>
+      <c r="E207" s="58"/>
+      <c r="F207" s="57"/>
       <c r="G207" s="9"/>
       <c r="H207" s="9"/>
       <c r="I207" s="9"/>
@@ -14981,16 +14981,16 @@
       <c r="Z207" s="9"/>
     </row>
     <row r="208" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A208" s="71"/>
+      <c r="A208" s="74"/>
       <c r="B208" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C208" s="59" t="s">
+      <c r="C208" s="96" t="s">
         <v>144</v>
       </c>
-      <c r="D208" s="57"/>
-      <c r="E208" s="57"/>
-      <c r="F208" s="58"/>
+      <c r="D208" s="58"/>
+      <c r="E208" s="58"/>
+      <c r="F208" s="57"/>
       <c r="G208" s="9"/>
       <c r="H208" s="9"/>
       <c r="I208" s="9"/>
@@ -15013,16 +15013,16 @@
       <c r="Z208" s="9"/>
     </row>
     <row r="209" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A209" s="71"/>
+      <c r="A209" s="74"/>
       <c r="B209" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C209" s="59" t="s">
+      <c r="C209" s="96" t="s">
         <v>145</v>
       </c>
-      <c r="D209" s="57"/>
-      <c r="E209" s="57"/>
-      <c r="F209" s="58"/>
+      <c r="D209" s="58"/>
+      <c r="E209" s="58"/>
+      <c r="F209" s="57"/>
       <c r="G209" s="9"/>
       <c r="H209" s="9"/>
       <c r="I209" s="9"/>
@@ -15045,16 +15045,16 @@
       <c r="Z209" s="9"/>
     </row>
     <row r="210" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="71"/>
+      <c r="A210" s="74"/>
       <c r="B210" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C210" s="59" t="s">
+      <c r="C210" s="96" t="s">
         <v>146</v>
       </c>
-      <c r="D210" s="57"/>
-      <c r="E210" s="57"/>
-      <c r="F210" s="58"/>
+      <c r="D210" s="58"/>
+      <c r="E210" s="58"/>
+      <c r="F210" s="57"/>
       <c r="G210" s="9"/>
       <c r="H210" s="9"/>
       <c r="I210" s="9"/>
@@ -15077,16 +15077,16 @@
       <c r="Z210" s="9"/>
     </row>
     <row r="211" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="71"/>
+      <c r="A211" s="74"/>
       <c r="B211" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C211" s="59" t="s">
+      <c r="C211" s="96" t="s">
         <v>147</v>
       </c>
-      <c r="D211" s="57"/>
-      <c r="E211" s="57"/>
-      <c r="F211" s="58"/>
+      <c r="D211" s="58"/>
+      <c r="E211" s="58"/>
+      <c r="F211" s="57"/>
       <c r="G211" s="9"/>
       <c r="H211" s="9"/>
       <c r="I211" s="9"/>
@@ -15109,16 +15109,16 @@
       <c r="Z211" s="9"/>
     </row>
     <row r="212" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="71"/>
+      <c r="A212" s="74"/>
       <c r="B212" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C212" s="59" t="s">
+      <c r="C212" s="96" t="s">
         <v>148</v>
       </c>
-      <c r="D212" s="57"/>
-      <c r="E212" s="57"/>
-      <c r="F212" s="58"/>
+      <c r="D212" s="58"/>
+      <c r="E212" s="58"/>
+      <c r="F212" s="57"/>
       <c r="G212" s="9"/>
       <c r="H212" s="9"/>
       <c r="I212" s="9"/>
@@ -15141,16 +15141,16 @@
       <c r="Z212" s="9"/>
     </row>
     <row r="213" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A213" s="71"/>
+      <c r="A213" s="74"/>
       <c r="B213" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C213" s="59" t="s">
+      <c r="C213" s="96" t="s">
         <v>149</v>
       </c>
-      <c r="D213" s="57"/>
-      <c r="E213" s="57"/>
-      <c r="F213" s="58"/>
+      <c r="D213" s="58"/>
+      <c r="E213" s="58"/>
+      <c r="F213" s="57"/>
       <c r="G213" s="9"/>
       <c r="H213" s="9"/>
       <c r="I213" s="9"/>
@@ -15173,16 +15173,16 @@
       <c r="Z213" s="9"/>
     </row>
     <row r="214" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A214" s="71"/>
+      <c r="A214" s="74"/>
       <c r="B214" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C214" s="59" t="s">
+      <c r="C214" s="96" t="s">
         <v>150</v>
       </c>
-      <c r="D214" s="57"/>
-      <c r="E214" s="57"/>
-      <c r="F214" s="58"/>
+      <c r="D214" s="58"/>
+      <c r="E214" s="58"/>
+      <c r="F214" s="57"/>
       <c r="G214" s="9"/>
       <c r="H214" s="9"/>
       <c r="I214" s="9"/>
@@ -15205,16 +15205,16 @@
       <c r="Z214" s="9"/>
     </row>
     <row r="215" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A215" s="71"/>
+      <c r="A215" s="74"/>
       <c r="B215" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C215" s="59" t="s">
+      <c r="C215" s="96" t="s">
         <v>151</v>
       </c>
-      <c r="D215" s="57"/>
-      <c r="E215" s="57"/>
-      <c r="F215" s="58"/>
+      <c r="D215" s="58"/>
+      <c r="E215" s="58"/>
+      <c r="F215" s="57"/>
       <c r="G215" s="9"/>
       <c r="H215" s="9"/>
       <c r="I215" s="9"/>
@@ -15237,16 +15237,16 @@
       <c r="Z215" s="9"/>
     </row>
     <row r="216" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A216" s="71"/>
+      <c r="A216" s="74"/>
       <c r="B216" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C216" s="59" t="s">
+      <c r="C216" s="96" t="s">
         <v>152</v>
       </c>
-      <c r="D216" s="57"/>
-      <c r="E216" s="57"/>
-      <c r="F216" s="58"/>
+      <c r="D216" s="58"/>
+      <c r="E216" s="58"/>
+      <c r="F216" s="57"/>
       <c r="G216" s="9"/>
       <c r="H216" s="9"/>
       <c r="I216" s="9"/>
@@ -15269,16 +15269,16 @@
       <c r="Z216" s="9"/>
     </row>
     <row r="217" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A217" s="71"/>
+      <c r="A217" s="74"/>
       <c r="B217" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C217" s="59" t="s">
+      <c r="C217" s="96" t="s">
         <v>153</v>
       </c>
-      <c r="D217" s="57"/>
-      <c r="E217" s="57"/>
-      <c r="F217" s="58"/>
+      <c r="D217" s="58"/>
+      <c r="E217" s="58"/>
+      <c r="F217" s="57"/>
       <c r="G217" s="9"/>
       <c r="H217" s="9"/>
       <c r="I217" s="9"/>
@@ -15301,16 +15301,16 @@
       <c r="Z217" s="9"/>
     </row>
     <row r="218" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A218" s="71"/>
+      <c r="A218" s="74"/>
       <c r="B218" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C218" s="59" t="s">
+      <c r="C218" s="96" t="s">
         <v>154</v>
       </c>
-      <c r="D218" s="57"/>
-      <c r="E218" s="57"/>
-      <c r="F218" s="58"/>
+      <c r="D218" s="58"/>
+      <c r="E218" s="58"/>
+      <c r="F218" s="57"/>
       <c r="G218" s="9"/>
       <c r="H218" s="9"/>
       <c r="I218" s="9"/>
@@ -15333,16 +15333,16 @@
       <c r="Z218" s="9"/>
     </row>
     <row r="219" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A219" s="72"/>
+      <c r="A219" s="75"/>
       <c r="B219" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C219" s="83" t="s">
+      <c r="C219" s="98" t="s">
         <v>1985</v>
       </c>
-      <c r="D219" s="57"/>
-      <c r="E219" s="57"/>
-      <c r="F219" s="58"/>
+      <c r="D219" s="58"/>
+      <c r="E219" s="58"/>
+      <c r="F219" s="57"/>
       <c r="G219" s="9"/>
       <c r="H219" s="9"/>
       <c r="I219" s="9"/>
@@ -15423,16 +15423,16 @@
       <c r="Z221" s="9"/>
     </row>
     <row r="222" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A222" s="73">
+      <c r="A222" s="104">
         <v>38</v>
       </c>
-      <c r="B222" s="84" t="s">
+      <c r="B222" s="99" t="s">
         <v>156</v>
       </c>
-      <c r="C222" s="62"/>
-      <c r="D222" s="62"/>
-      <c r="E222" s="62"/>
-      <c r="F222" s="63"/>
+      <c r="C222" s="84"/>
+      <c r="D222" s="84"/>
+      <c r="E222" s="84"/>
+      <c r="F222" s="79"/>
       <c r="G222" s="9"/>
       <c r="H222" s="9"/>
       <c r="I222" s="9"/>
@@ -15455,12 +15455,12 @@
       <c r="Z222" s="9"/>
     </row>
     <row r="223" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A223" s="71"/>
-      <c r="B223" s="64"/>
-      <c r="C223" s="65"/>
-      <c r="D223" s="65"/>
-      <c r="E223" s="65"/>
-      <c r="F223" s="66"/>
+      <c r="A223" s="74"/>
+      <c r="B223" s="80"/>
+      <c r="C223" s="66"/>
+      <c r="D223" s="66"/>
+      <c r="E223" s="66"/>
+      <c r="F223" s="81"/>
       <c r="G223" s="9"/>
       <c r="H223" s="9"/>
       <c r="I223" s="9"/>
@@ -15483,12 +15483,12 @@
       <c r="Z223" s="9"/>
     </row>
     <row r="224" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A224" s="71"/>
-      <c r="B224" s="64"/>
-      <c r="C224" s="65"/>
-      <c r="D224" s="65"/>
-      <c r="E224" s="65"/>
-      <c r="F224" s="66"/>
+      <c r="A224" s="74"/>
+      <c r="B224" s="80"/>
+      <c r="C224" s="66"/>
+      <c r="D224" s="66"/>
+      <c r="E224" s="66"/>
+      <c r="F224" s="81"/>
       <c r="G224" s="9"/>
       <c r="H224" s="9"/>
       <c r="I224" s="9"/>
@@ -15511,12 +15511,12 @@
       <c r="Z224" s="9"/>
     </row>
     <row r="225" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A225" s="72"/>
-      <c r="B225" s="67"/>
-      <c r="C225" s="68"/>
-      <c r="D225" s="68"/>
-      <c r="E225" s="68"/>
-      <c r="F225" s="69"/>
+      <c r="A225" s="75"/>
+      <c r="B225" s="85"/>
+      <c r="C225" s="86"/>
+      <c r="D225" s="86"/>
+      <c r="E225" s="86"/>
+      <c r="F225" s="87"/>
       <c r="G225" s="9"/>
       <c r="H225" s="9"/>
       <c r="I225" s="9"/>
@@ -15625,16 +15625,16 @@
       <c r="Z228" s="9"/>
     </row>
     <row r="229" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A229" s="70">
+      <c r="A229" s="73">
         <v>39</v>
       </c>
-      <c r="B229" s="61" t="s">
+      <c r="B229" s="103" t="s">
         <v>158</v>
       </c>
-      <c r="C229" s="62"/>
-      <c r="D229" s="62"/>
-      <c r="E229" s="62"/>
-      <c r="F229" s="63"/>
+      <c r="C229" s="84"/>
+      <c r="D229" s="84"/>
+      <c r="E229" s="84"/>
+      <c r="F229" s="79"/>
       <c r="G229" s="9"/>
       <c r="H229" s="9"/>
       <c r="I229" s="9"/>
@@ -15657,12 +15657,12 @@
       <c r="Z229" s="9"/>
     </row>
     <row r="230" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A230" s="71"/>
-      <c r="B230" s="64"/>
-      <c r="C230" s="65"/>
-      <c r="D230" s="65"/>
-      <c r="E230" s="65"/>
-      <c r="F230" s="66"/>
+      <c r="A230" s="74"/>
+      <c r="B230" s="80"/>
+      <c r="C230" s="66"/>
+      <c r="D230" s="66"/>
+      <c r="E230" s="66"/>
+      <c r="F230" s="81"/>
       <c r="G230" s="9"/>
       <c r="H230" s="9"/>
       <c r="I230" s="9"/>
@@ -15685,12 +15685,12 @@
       <c r="Z230" s="9"/>
     </row>
     <row r="231" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A231" s="71"/>
-      <c r="B231" s="64"/>
-      <c r="C231" s="65"/>
-      <c r="D231" s="65"/>
-      <c r="E231" s="65"/>
-      <c r="F231" s="66"/>
+      <c r="A231" s="74"/>
+      <c r="B231" s="80"/>
+      <c r="C231" s="66"/>
+      <c r="D231" s="66"/>
+      <c r="E231" s="66"/>
+      <c r="F231" s="81"/>
       <c r="G231" s="9"/>
       <c r="H231" s="9"/>
       <c r="I231" s="9"/>
@@ -15713,12 +15713,12 @@
       <c r="Z231" s="9"/>
     </row>
     <row r="232" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A232" s="71"/>
-      <c r="B232" s="64"/>
-      <c r="C232" s="65"/>
-      <c r="D232" s="65"/>
-      <c r="E232" s="65"/>
-      <c r="F232" s="66"/>
+      <c r="A232" s="74"/>
+      <c r="B232" s="80"/>
+      <c r="C232" s="66"/>
+      <c r="D232" s="66"/>
+      <c r="E232" s="66"/>
+      <c r="F232" s="81"/>
       <c r="G232" s="9"/>
       <c r="H232" s="9"/>
       <c r="I232" s="9"/>
@@ -15741,12 +15741,12 @@
       <c r="Z232" s="9"/>
     </row>
     <row r="233" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A233" s="71"/>
-      <c r="B233" s="64"/>
-      <c r="C233" s="65"/>
-      <c r="D233" s="65"/>
-      <c r="E233" s="65"/>
-      <c r="F233" s="66"/>
+      <c r="A233" s="74"/>
+      <c r="B233" s="80"/>
+      <c r="C233" s="66"/>
+      <c r="D233" s="66"/>
+      <c r="E233" s="66"/>
+      <c r="F233" s="81"/>
       <c r="G233" s="9"/>
       <c r="H233" s="9"/>
       <c r="I233" s="9"/>
@@ -15769,12 +15769,12 @@
       <c r="Z233" s="9"/>
     </row>
     <row r="234" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A234" s="71"/>
-      <c r="B234" s="64"/>
-      <c r="C234" s="65"/>
-      <c r="D234" s="65"/>
-      <c r="E234" s="65"/>
-      <c r="F234" s="66"/>
+      <c r="A234" s="74"/>
+      <c r="B234" s="80"/>
+      <c r="C234" s="66"/>
+      <c r="D234" s="66"/>
+      <c r="E234" s="66"/>
+      <c r="F234" s="81"/>
       <c r="G234" s="9"/>
       <c r="H234" s="9"/>
       <c r="I234" s="9"/>
@@ -15797,12 +15797,12 @@
       <c r="Z234" s="9"/>
     </row>
     <row r="235" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A235" s="72"/>
-      <c r="B235" s="67"/>
-      <c r="C235" s="68"/>
-      <c r="D235" s="68"/>
-      <c r="E235" s="68"/>
-      <c r="F235" s="69"/>
+      <c r="A235" s="75"/>
+      <c r="B235" s="85"/>
+      <c r="C235" s="86"/>
+      <c r="D235" s="86"/>
+      <c r="E235" s="86"/>
+      <c r="F235" s="87"/>
       <c r="G235" s="9"/>
       <c r="H235" s="9"/>
       <c r="I235" s="9"/>
@@ -37258,79 +37258,90 @@
     </row>
   </sheetData>
   <mergeCells count="181">
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="D56:F56"/>
-    <mergeCell ref="D57:F57"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="D59:F59"/>
-    <mergeCell ref="D60:F60"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="D62:F62"/>
-    <mergeCell ref="D63:F63"/>
-    <mergeCell ref="D64:F64"/>
-    <mergeCell ref="D65:F65"/>
-    <mergeCell ref="D66:F66"/>
-    <mergeCell ref="D69:F69"/>
-    <mergeCell ref="D70:F70"/>
-    <mergeCell ref="D71:F71"/>
-    <mergeCell ref="D72:F72"/>
-    <mergeCell ref="D73:F73"/>
-    <mergeCell ref="D74:F74"/>
-    <mergeCell ref="D75:F75"/>
-    <mergeCell ref="D76:F76"/>
-    <mergeCell ref="D77:F77"/>
-    <mergeCell ref="D78:F78"/>
-    <mergeCell ref="E128:F128"/>
-    <mergeCell ref="D79:F79"/>
-    <mergeCell ref="D80:F80"/>
-    <mergeCell ref="D81:F81"/>
-    <mergeCell ref="D82:F82"/>
-    <mergeCell ref="D83:F83"/>
-    <mergeCell ref="D84:F84"/>
-    <mergeCell ref="D85:F85"/>
-    <mergeCell ref="D101:F101"/>
-    <mergeCell ref="D102:F102"/>
-    <mergeCell ref="E125:F125"/>
-    <mergeCell ref="D103:F103"/>
-    <mergeCell ref="D113:F113"/>
-    <mergeCell ref="D114:F114"/>
-    <mergeCell ref="D115:F115"/>
-    <mergeCell ref="D116:F116"/>
-    <mergeCell ref="D117:F117"/>
-    <mergeCell ref="E126:F126"/>
-    <mergeCell ref="E127:F127"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="B31:C33"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="B174:F174"/>
+    <mergeCell ref="B175:F175"/>
+    <mergeCell ref="B176:F176"/>
+    <mergeCell ref="B177:F177"/>
+    <mergeCell ref="B229:F235"/>
+    <mergeCell ref="A55:A61"/>
+    <mergeCell ref="A69:A77"/>
+    <mergeCell ref="A114:A121"/>
+    <mergeCell ref="A124:A132"/>
+    <mergeCell ref="A135:A157"/>
+    <mergeCell ref="A160:A192"/>
+    <mergeCell ref="A195:A219"/>
+    <mergeCell ref="A222:A225"/>
+    <mergeCell ref="A229:A235"/>
+    <mergeCell ref="A78:A84"/>
+    <mergeCell ref="A88:A100"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A106:A111"/>
+    <mergeCell ref="A123:D123"/>
+    <mergeCell ref="B124:D124"/>
+    <mergeCell ref="B125:D125"/>
+    <mergeCell ref="B126:D126"/>
+    <mergeCell ref="B127:D127"/>
+    <mergeCell ref="B128:D128"/>
+    <mergeCell ref="B129:D129"/>
+    <mergeCell ref="B130:D130"/>
+    <mergeCell ref="B131:D131"/>
+    <mergeCell ref="B132:D132"/>
+    <mergeCell ref="B135:F157"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="B34:C36"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:C39"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="B121:C121"/>
+    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="E124:F124"/>
+    <mergeCell ref="C219:F219"/>
+    <mergeCell ref="B222:F225"/>
+    <mergeCell ref="C212:F212"/>
+    <mergeCell ref="C213:F213"/>
+    <mergeCell ref="C214:F214"/>
+    <mergeCell ref="C215:F215"/>
+    <mergeCell ref="C216:F216"/>
+    <mergeCell ref="C217:F217"/>
+    <mergeCell ref="C218:F218"/>
+    <mergeCell ref="C210:F210"/>
+    <mergeCell ref="C211:F211"/>
+    <mergeCell ref="C203:F203"/>
+    <mergeCell ref="C204:F204"/>
+    <mergeCell ref="C205:F205"/>
+    <mergeCell ref="C206:F206"/>
+    <mergeCell ref="C207:F207"/>
+    <mergeCell ref="C208:F208"/>
+    <mergeCell ref="C209:F209"/>
+    <mergeCell ref="C201:F201"/>
+    <mergeCell ref="C202:F202"/>
+    <mergeCell ref="B192:F192"/>
+    <mergeCell ref="C195:F195"/>
+    <mergeCell ref="C196:F196"/>
+    <mergeCell ref="C197:F197"/>
+    <mergeCell ref="C198:F198"/>
+    <mergeCell ref="C199:F199"/>
+    <mergeCell ref="C200:F200"/>
+    <mergeCell ref="B190:F190"/>
+    <mergeCell ref="B191:F191"/>
+    <mergeCell ref="B178:F179"/>
+    <mergeCell ref="B183:F183"/>
+    <mergeCell ref="B184:F184"/>
+    <mergeCell ref="B185:F186"/>
+    <mergeCell ref="B187:F187"/>
+    <mergeCell ref="B188:F188"/>
+    <mergeCell ref="B189:F189"/>
     <mergeCell ref="B160:F160"/>
     <mergeCell ref="B161:F162"/>
     <mergeCell ref="B163:F163"/>
@@ -37355,90 +37366,79 @@
     <mergeCell ref="D119:F119"/>
     <mergeCell ref="D120:F120"/>
     <mergeCell ref="D121:F121"/>
-    <mergeCell ref="B190:F190"/>
-    <mergeCell ref="B191:F191"/>
-    <mergeCell ref="B178:F179"/>
-    <mergeCell ref="B183:F183"/>
-    <mergeCell ref="B184:F184"/>
-    <mergeCell ref="B185:F186"/>
-    <mergeCell ref="B187:F187"/>
-    <mergeCell ref="B188:F188"/>
-    <mergeCell ref="B189:F189"/>
-    <mergeCell ref="C201:F201"/>
-    <mergeCell ref="C202:F202"/>
-    <mergeCell ref="B192:F192"/>
-    <mergeCell ref="C195:F195"/>
-    <mergeCell ref="C196:F196"/>
-    <mergeCell ref="C197:F197"/>
-    <mergeCell ref="C198:F198"/>
-    <mergeCell ref="C199:F199"/>
-    <mergeCell ref="C200:F200"/>
-    <mergeCell ref="C210:F210"/>
-    <mergeCell ref="C211:F211"/>
-    <mergeCell ref="C203:F203"/>
-    <mergeCell ref="C204:F204"/>
-    <mergeCell ref="C205:F205"/>
-    <mergeCell ref="C206:F206"/>
-    <mergeCell ref="C207:F207"/>
-    <mergeCell ref="C208:F208"/>
-    <mergeCell ref="C209:F209"/>
-    <mergeCell ref="C219:F219"/>
-    <mergeCell ref="B222:F225"/>
-    <mergeCell ref="C212:F212"/>
-    <mergeCell ref="C213:F213"/>
-    <mergeCell ref="C214:F214"/>
-    <mergeCell ref="C215:F215"/>
-    <mergeCell ref="C216:F216"/>
-    <mergeCell ref="C217:F217"/>
-    <mergeCell ref="C218:F218"/>
-    <mergeCell ref="B129:D129"/>
-    <mergeCell ref="B130:D130"/>
-    <mergeCell ref="B131:D131"/>
-    <mergeCell ref="B132:D132"/>
-    <mergeCell ref="B135:F157"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="B34:C36"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:C39"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="B121:C121"/>
-    <mergeCell ref="E123:F123"/>
-    <mergeCell ref="E124:F124"/>
-    <mergeCell ref="B174:F174"/>
-    <mergeCell ref="B175:F175"/>
-    <mergeCell ref="B176:F176"/>
-    <mergeCell ref="B177:F177"/>
-    <mergeCell ref="B229:F235"/>
-    <mergeCell ref="A55:A61"/>
-    <mergeCell ref="A69:A77"/>
-    <mergeCell ref="A114:A121"/>
-    <mergeCell ref="A124:A132"/>
-    <mergeCell ref="A135:A157"/>
-    <mergeCell ref="A160:A192"/>
-    <mergeCell ref="A195:A219"/>
-    <mergeCell ref="A222:A225"/>
-    <mergeCell ref="A229:A235"/>
-    <mergeCell ref="A78:A84"/>
-    <mergeCell ref="A88:A100"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A106:A111"/>
-    <mergeCell ref="A123:D123"/>
-    <mergeCell ref="B124:D124"/>
-    <mergeCell ref="B125:D125"/>
-    <mergeCell ref="B126:D126"/>
-    <mergeCell ref="B127:D127"/>
-    <mergeCell ref="B128:D128"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="B31:C33"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="E128:F128"/>
+    <mergeCell ref="D79:F79"/>
+    <mergeCell ref="D80:F80"/>
+    <mergeCell ref="D81:F81"/>
+    <mergeCell ref="D82:F82"/>
+    <mergeCell ref="D83:F83"/>
+    <mergeCell ref="D84:F84"/>
+    <mergeCell ref="D85:F85"/>
+    <mergeCell ref="D101:F101"/>
+    <mergeCell ref="D102:F102"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="D103:F103"/>
+    <mergeCell ref="D113:F113"/>
+    <mergeCell ref="D114:F114"/>
+    <mergeCell ref="D115:F115"/>
+    <mergeCell ref="D116:F116"/>
+    <mergeCell ref="D117:F117"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="D70:F70"/>
+    <mergeCell ref="D71:F71"/>
+    <mergeCell ref="D72:F72"/>
+    <mergeCell ref="D73:F73"/>
+    <mergeCell ref="D74:F74"/>
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="D76:F76"/>
+    <mergeCell ref="D77:F77"/>
+    <mergeCell ref="D78:F78"/>
+    <mergeCell ref="D59:F59"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="D63:F63"/>
+    <mergeCell ref="D64:F64"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="D55:F55"/>
+    <mergeCell ref="D56:F56"/>
+    <mergeCell ref="D57:F57"/>
+    <mergeCell ref="D58:F58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="5" orientation="landscape"/>
@@ -37484,10 +37484,10 @@
       <c r="G1" s="108" t="s">
         <v>165</v>
       </c>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="81"/>
       <c r="L1" s="32"/>
       <c r="M1" s="33" t="s">
         <v>166</v>

</xml_diff>

<commit_message>
Fix/offline pwa improvements (#481)
* fix: disposition char limit, false-offline flash, AFOR city overwrite, revision diff; ignore Maven target/

* fix: PWA improvements

* fix: lint

* fix: lint more
</commit_message>
<xml_diff>
--- a/sample AFOR.xlsx
+++ b/sample AFOR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gwent\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\WIMS-BFP-PROTOTYPE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582663FE-F0F1-405D-B24C-446C24E259A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7453CAB-377A-4648-89FE-C4AFEF5B2DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5112" yWindow="180" windowWidth="17280" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AFOR" sheetId="1" r:id="rId1"/>
@@ -6750,111 +6750,33 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6867,14 +6789,92 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -8689,14 +8689,14 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="100" t="s">
+      <c r="A7" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="65"/>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -8719,14 +8719,14 @@
       <c r="Z7" s="3"/>
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="101" t="s">
+      <c r="A8" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="65"/>
-      <c r="C8" s="65"/>
-      <c r="D8" s="65"/>
-      <c r="E8" s="65"/>
-      <c r="F8" s="65"/>
+      <c r="B8" s="66"/>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -8749,14 +8749,14 @@
       <c r="Z8" s="4"/>
     </row>
     <row r="9" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="102" t="s">
+      <c r="A9" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="65"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
+      <c r="B9" s="66"/>
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -8779,14 +8779,14 @@
       <c r="Z9" s="5"/>
     </row>
     <row r="10" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="100" t="s">
+      <c r="A10" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="65"/>
-      <c r="C10" s="65"/>
-      <c r="D10" s="65"/>
-      <c r="E10" s="65"/>
-      <c r="F10" s="65"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -8809,14 +8809,14 @@
       <c r="Z10" s="3"/>
     </row>
     <row r="11" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="100" t="s">
+      <c r="A11" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
+      <c r="B11" s="66"/>
+      <c r="C11" s="66"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="66"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -8839,14 +8839,14 @@
       <c r="Z11" s="3"/>
     </row>
     <row r="12" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="103" t="s">
+      <c r="A12" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="65"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
+      <c r="B12" s="66"/>
+      <c r="C12" s="66"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="66"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -8897,14 +8897,14 @@
       <c r="Z13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="104" t="s">
+      <c r="A14" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="65"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="65"/>
-      <c r="E14" s="65"/>
-      <c r="F14" s="65"/>
+      <c r="B14" s="66"/>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="66"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -8955,14 +8955,14 @@
       <c r="Z15" s="2"/>
     </row>
     <row r="16" spans="1:26" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="96" t="s">
+      <c r="A16" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="65"/>
-      <c r="C16" s="65"/>
-      <c r="D16" s="65"/>
-      <c r="E16" s="65"/>
-      <c r="F16" s="65"/>
+      <c r="B16" s="66"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -9043,16 +9043,16 @@
       <c r="Z18" s="9"/>
     </row>
     <row r="19" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="70">
+      <c r="A19" s="73">
         <v>1</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C19" s="11"/>
-      <c r="D19" s="97"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="58"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="57"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
       <c r="I19" s="9"/>
@@ -9075,18 +9075,18 @@
       <c r="Z19" s="9"/>
     </row>
     <row r="20" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="71"/>
+      <c r="A20" s="74"/>
       <c r="B20" s="11" t="s">
         <v>1953</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="98" t="s">
+      <c r="D20" s="61" t="s">
         <v>1954</v>
       </c>
-      <c r="E20" s="57"/>
-      <c r="F20" s="58"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="57"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
@@ -9109,16 +9109,16 @@
       <c r="Z20" s="9"/>
     </row>
     <row r="21" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="72"/>
+      <c r="A21" s="75"/>
       <c r="B21" s="11"/>
       <c r="C21" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="98" t="s">
+      <c r="D21" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="57"/>
-      <c r="F21" s="58"/>
+      <c r="E21" s="58"/>
+      <c r="F21" s="57"/>
       <c r="G21" s="13"/>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
@@ -9148,11 +9148,11 @@
         <v>13</v>
       </c>
       <c r="C22" s="11"/>
-      <c r="D22" s="99">
-        <v>38221</v>
-      </c>
-      <c r="E22" s="57"/>
-      <c r="F22" s="58"/>
+      <c r="D22" s="77">
+        <v>46202</v>
+      </c>
+      <c r="E22" s="58"/>
+      <c r="F22" s="57"/>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
@@ -9182,11 +9182,11 @@
         <v>14</v>
       </c>
       <c r="C23" s="11"/>
-      <c r="D23" s="91">
-        <v>0.93194444444444446</v>
-      </c>
-      <c r="E23" s="57"/>
-      <c r="F23" s="58"/>
+      <c r="D23" s="71">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="E23" s="58"/>
+      <c r="F23" s="57"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
@@ -9209,7 +9209,7 @@
       <c r="Z23" s="9"/>
     </row>
     <row r="24" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="70">
+      <c r="A24" s="73">
         <v>4</v>
       </c>
       <c r="B24" s="11" t="s">
@@ -9219,8 +9219,8 @@
       <c r="D24" s="60" t="s">
         <v>241</v>
       </c>
-      <c r="E24" s="57"/>
-      <c r="F24" s="58"/>
+      <c r="E24" s="58"/>
+      <c r="F24" s="57"/>
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
@@ -9243,7 +9243,7 @@
       <c r="Z24" s="9"/>
     </row>
     <row r="25" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="71"/>
+      <c r="A25" s="74"/>
       <c r="B25" s="11" t="s">
         <v>16</v>
       </c>
@@ -9251,8 +9251,8 @@
       <c r="D25" s="60" t="s">
         <v>1955</v>
       </c>
-      <c r="E25" s="57"/>
-      <c r="F25" s="58"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="57"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
@@ -9275,7 +9275,7 @@
       <c r="Z25" s="9"/>
     </row>
     <row r="26" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="71"/>
+      <c r="A26" s="74"/>
       <c r="B26" s="11" t="s">
         <v>17</v>
       </c>
@@ -9283,8 +9283,8 @@
       <c r="D26" s="60" t="s">
         <v>1956</v>
       </c>
-      <c r="E26" s="57"/>
-      <c r="F26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="57"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
@@ -9307,7 +9307,7 @@
       <c r="Z26" s="9"/>
     </row>
     <row r="27" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="72"/>
+      <c r="A27" s="75"/>
       <c r="B27" s="11" t="s">
         <v>18</v>
       </c>
@@ -9349,8 +9349,8 @@
       <c r="D28" s="60" t="s">
         <v>1958</v>
       </c>
-      <c r="E28" s="57"/>
-      <c r="F28" s="58"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="57"/>
       <c r="G28" s="16"/>
       <c r="H28" s="9"/>
       <c r="I28" s="9"/>
@@ -9383,8 +9383,8 @@
       <c r="D29" s="60" t="s">
         <v>1959</v>
       </c>
-      <c r="E29" s="57"/>
-      <c r="F29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="57"/>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
       <c r="I29" s="9"/>
@@ -9417,8 +9417,8 @@
       <c r="D30" s="60" t="s">
         <v>1960</v>
       </c>
-      <c r="E30" s="57"/>
-      <c r="F30" s="58"/>
+      <c r="E30" s="58"/>
+      <c r="F30" s="57"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
       <c r="I30" s="9"/>
@@ -9441,18 +9441,18 @@
       <c r="Z30" s="9"/>
     </row>
     <row r="31" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="70">
+      <c r="A31" s="73">
         <v>8</v>
       </c>
-      <c r="B31" s="80" t="s">
+      <c r="B31" s="78" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="63"/>
+      <c r="C31" s="79"/>
       <c r="D31" s="60" t="s">
         <v>1961</v>
       </c>
-      <c r="E31" s="57"/>
-      <c r="F31" s="58"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="57"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
       <c r="I31" s="9"/>
@@ -9475,14 +9475,14 @@
       <c r="Z31" s="9"/>
     </row>
     <row r="32" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="71"/>
-      <c r="B32" s="64"/>
-      <c r="C32" s="66"/>
+      <c r="A32" s="74"/>
+      <c r="B32" s="80"/>
+      <c r="C32" s="81"/>
       <c r="D32" s="60" t="s">
         <v>1962</v>
       </c>
-      <c r="E32" s="57"/>
-      <c r="F32" s="58"/>
+      <c r="E32" s="58"/>
+      <c r="F32" s="57"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
       <c r="I32" s="9"/>
@@ -9505,12 +9505,12 @@
       <c r="Z32" s="9"/>
     </row>
     <row r="33" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="72"/>
-      <c r="B33" s="64"/>
-      <c r="C33" s="66"/>
+      <c r="A33" s="75"/>
+      <c r="B33" s="80"/>
+      <c r="C33" s="81"/>
       <c r="D33" s="60"/>
-      <c r="E33" s="57"/>
-      <c r="F33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="57"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
       <c r="I33" s="9"/>
@@ -9533,18 +9533,18 @@
       <c r="Z33" s="9"/>
     </row>
     <row r="34" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="70">
+      <c r="A34" s="73">
         <v>9</v>
       </c>
-      <c r="B34" s="80" t="s">
+      <c r="B34" s="78" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="63"/>
-      <c r="D34" s="91">
-        <v>5.7638888888888892E-2</v>
-      </c>
-      <c r="E34" s="57"/>
-      <c r="F34" s="58"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="71">
+        <v>0.43680555555555556</v>
+      </c>
+      <c r="E34" s="58"/>
+      <c r="F34" s="57"/>
       <c r="G34" s="9"/>
       <c r="H34" s="9"/>
       <c r="I34" s="9"/>
@@ -9567,14 +9567,14 @@
       <c r="Z34" s="9"/>
     </row>
     <row r="35" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="71"/>
-      <c r="B35" s="64"/>
-      <c r="C35" s="66"/>
-      <c r="D35" s="91">
-        <v>5.9027777777777776E-2</v>
-      </c>
-      <c r="E35" s="57"/>
-      <c r="F35" s="58"/>
+      <c r="A35" s="74"/>
+      <c r="B35" s="80"/>
+      <c r="C35" s="81"/>
+      <c r="D35" s="71">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="E35" s="58"/>
+      <c r="F35" s="57"/>
       <c r="G35" s="9"/>
       <c r="H35" s="9"/>
       <c r="I35" s="9"/>
@@ -9597,12 +9597,12 @@
       <c r="Z35" s="9"/>
     </row>
     <row r="36" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="72"/>
-      <c r="B36" s="67"/>
-      <c r="C36" s="69"/>
+      <c r="A36" s="75"/>
+      <c r="B36" s="85"/>
+      <c r="C36" s="87"/>
       <c r="D36" s="60"/>
-      <c r="E36" s="57"/>
-      <c r="F36" s="58"/>
+      <c r="E36" s="58"/>
+      <c r="F36" s="57"/>
       <c r="G36" s="9"/>
       <c r="H36" s="9"/>
       <c r="I36" s="9"/>
@@ -9625,18 +9625,18 @@
       <c r="Z36" s="9"/>
     </row>
     <row r="37" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="70">
+      <c r="A37" s="73">
         <v>10</v>
       </c>
-      <c r="B37" s="80" t="s">
+      <c r="B37" s="78" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="63"/>
-      <c r="D37" s="91">
-        <v>7.5694444444444439E-2</v>
-      </c>
-      <c r="E37" s="57"/>
-      <c r="F37" s="58"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="71">
+        <v>0.45208333333333334</v>
+      </c>
+      <c r="E37" s="58"/>
+      <c r="F37" s="57"/>
       <c r="G37" s="9"/>
       <c r="H37" s="9"/>
       <c r="I37" s="9"/>
@@ -9659,14 +9659,14 @@
       <c r="Z37" s="9"/>
     </row>
     <row r="38" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="71"/>
-      <c r="B38" s="64"/>
-      <c r="C38" s="66"/>
-      <c r="D38" s="91">
-        <v>8.1944444444444445E-2</v>
-      </c>
-      <c r="E38" s="57"/>
-      <c r="F38" s="58"/>
+      <c r="A38" s="74"/>
+      <c r="B38" s="80"/>
+      <c r="C38" s="81"/>
+      <c r="D38" s="71">
+        <v>0.45694444444444443</v>
+      </c>
+      <c r="E38" s="58"/>
+      <c r="F38" s="57"/>
       <c r="G38" s="9"/>
       <c r="H38" s="9"/>
       <c r="I38" s="9"/>
@@ -9689,12 +9689,12 @@
       <c r="Z38" s="9"/>
     </row>
     <row r="39" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="72"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="69"/>
+      <c r="A39" s="75"/>
+      <c r="B39" s="85"/>
+      <c r="C39" s="87"/>
       <c r="D39" s="60"/>
-      <c r="E39" s="57"/>
-      <c r="F39" s="58"/>
+      <c r="E39" s="58"/>
+      <c r="F39" s="57"/>
       <c r="G39" s="9"/>
       <c r="H39" s="9"/>
       <c r="I39" s="9"/>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="C40" s="11"/>
       <c r="D40" s="92">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E40" s="93"/>
       <c r="F40" s="94"/>
@@ -9754,15 +9754,15 @@
       <c r="A41" s="14">
         <v>12</v>
       </c>
-      <c r="B41" s="81" t="s">
+      <c r="B41" s="97" t="s">
         <v>26</v>
       </c>
-      <c r="C41" s="58"/>
+      <c r="C41" s="57"/>
       <c r="D41" s="60">
         <v>9.8000000000000007</v>
       </c>
-      <c r="E41" s="57"/>
-      <c r="F41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="57"/>
       <c r="G41" s="9"/>
       <c r="H41" s="9"/>
       <c r="I41" s="9"/>
@@ -9788,15 +9788,15 @@
       <c r="A42" s="14">
         <v>13</v>
       </c>
-      <c r="B42" s="82" t="s">
+      <c r="B42" s="101" t="s">
         <v>27</v>
       </c>
-      <c r="C42" s="58"/>
+      <c r="C42" s="57"/>
       <c r="D42" s="95" t="s">
         <v>1963</v>
       </c>
-      <c r="E42" s="57"/>
-      <c r="F42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="57"/>
       <c r="G42" s="9"/>
       <c r="H42" s="9"/>
       <c r="I42" s="9"/>
@@ -9826,11 +9826,11 @@
         <v>28</v>
       </c>
       <c r="C43" s="11"/>
-      <c r="D43" s="91">
-        <v>0.22291666666666668</v>
-      </c>
-      <c r="E43" s="57"/>
-      <c r="F43" s="58"/>
+      <c r="D43" s="71">
+        <v>0.63958333333333328</v>
+      </c>
+      <c r="E43" s="58"/>
+      <c r="F43" s="57"/>
       <c r="G43" s="9"/>
       <c r="H43" s="9"/>
       <c r="I43" s="9"/>
@@ -9863,8 +9863,8 @@
       <c r="D44" s="60">
         <v>21</v>
       </c>
-      <c r="E44" s="57"/>
-      <c r="F44" s="58"/>
+      <c r="E44" s="58"/>
+      <c r="F44" s="57"/>
       <c r="G44" s="9"/>
       <c r="H44" s="9"/>
       <c r="I44" s="9"/>
@@ -9945,7 +9945,7 @@
       <c r="Z46" s="9"/>
     </row>
     <row r="47" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="70">
+      <c r="A47" s="73">
         <v>16</v>
       </c>
       <c r="B47" s="19" t="s">
@@ -9953,8 +9953,8 @@
       </c>
       <c r="C47" s="19"/>
       <c r="D47" s="60"/>
-      <c r="E47" s="57"/>
-      <c r="F47" s="58"/>
+      <c r="E47" s="58"/>
+      <c r="F47" s="57"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
       <c r="I47" s="9"/>
@@ -9977,14 +9977,14 @@
       <c r="Z47" s="9"/>
     </row>
     <row r="48" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="71"/>
+      <c r="A48" s="74"/>
       <c r="B48" s="11"/>
       <c r="C48" s="12" t="s">
         <v>32</v>
       </c>
       <c r="D48" s="60"/>
-      <c r="E48" s="57"/>
-      <c r="F48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="57"/>
       <c r="G48" s="9"/>
       <c r="H48" s="9"/>
       <c r="I48" s="9"/>
@@ -10007,14 +10007,14 @@
       <c r="Z48" s="9"/>
     </row>
     <row r="49" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="71"/>
+      <c r="A49" s="74"/>
       <c r="B49" s="11"/>
       <c r="C49" s="12" t="s">
         <v>33</v>
       </c>
       <c r="D49" s="60"/>
-      <c r="E49" s="57"/>
-      <c r="F49" s="58"/>
+      <c r="E49" s="58"/>
+      <c r="F49" s="57"/>
       <c r="G49" s="9"/>
       <c r="H49" s="9"/>
       <c r="I49" s="9"/>
@@ -10037,17 +10037,17 @@
       <c r="Z49" s="9"/>
     </row>
     <row r="50" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="72"/>
+      <c r="A50" s="75"/>
       <c r="B50" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C50" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D50" s="76" t="s">
+      <c r="D50" s="56" t="s">
         <v>1964</v>
       </c>
-      <c r="E50" s="58"/>
+      <c r="E50" s="57"/>
       <c r="F50" s="19"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
@@ -10074,15 +10074,15 @@
       <c r="A51" s="14">
         <v>17</v>
       </c>
-      <c r="B51" s="81" t="s">
+      <c r="B51" s="97" t="s">
         <v>35</v>
       </c>
-      <c r="C51" s="58"/>
-      <c r="D51" s="76" t="s">
+      <c r="C51" s="57"/>
+      <c r="D51" s="56" t="s">
         <v>1965</v>
       </c>
-      <c r="E51" s="57"/>
-      <c r="F51" s="58"/>
+      <c r="E51" s="58"/>
+      <c r="F51" s="57"/>
       <c r="G51" s="9"/>
       <c r="H51" s="9"/>
       <c r="I51" s="9"/>
@@ -10108,15 +10108,15 @@
       <c r="A52" s="14">
         <v>18</v>
       </c>
-      <c r="B52" s="81" t="s">
+      <c r="B52" s="97" t="s">
         <v>36</v>
       </c>
-      <c r="C52" s="58"/>
-      <c r="D52" s="76" t="s">
+      <c r="C52" s="57"/>
+      <c r="D52" s="56" t="s">
         <v>1987</v>
       </c>
-      <c r="E52" s="57"/>
-      <c r="F52" s="58"/>
+      <c r="E52" s="58"/>
+      <c r="F52" s="57"/>
       <c r="G52" s="9"/>
       <c r="H52" s="9"/>
       <c r="I52" s="9"/>
@@ -10142,15 +10142,15 @@
       <c r="A53" s="14">
         <v>19</v>
       </c>
-      <c r="B53" s="81" t="s">
+      <c r="B53" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="C53" s="58"/>
-      <c r="D53" s="76" t="s">
+      <c r="C53" s="57"/>
+      <c r="D53" s="56" t="s">
         <v>1966</v>
       </c>
-      <c r="E53" s="57"/>
-      <c r="F53" s="58"/>
+      <c r="E53" s="58"/>
+      <c r="F53" s="57"/>
       <c r="G53" s="20"/>
       <c r="H53" s="20"/>
       <c r="I53" s="20"/>
@@ -10176,15 +10176,15 @@
       <c r="A54" s="10">
         <v>20</v>
       </c>
-      <c r="B54" s="81" t="s">
+      <c r="B54" s="97" t="s">
         <v>38</v>
       </c>
-      <c r="C54" s="58"/>
-      <c r="D54" s="107" t="s">
+      <c r="C54" s="57"/>
+      <c r="D54" s="59" t="s">
         <v>1967</v>
       </c>
-      <c r="E54" s="57"/>
-      <c r="F54" s="58"/>
+      <c r="E54" s="58"/>
+      <c r="F54" s="57"/>
       <c r="G54" s="20"/>
       <c r="H54" s="20"/>
       <c r="I54" s="20"/>
@@ -10207,7 +10207,7 @@
       <c r="Z54" s="20"/>
     </row>
     <row r="55" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="70">
+      <c r="A55" s="73">
         <v>21</v>
       </c>
       <c r="B55" s="11" t="s">
@@ -10215,8 +10215,8 @@
       </c>
       <c r="C55" s="19"/>
       <c r="D55" s="60"/>
-      <c r="E55" s="57"/>
-      <c r="F55" s="58"/>
+      <c r="E55" s="58"/>
+      <c r="F55" s="57"/>
       <c r="G55" s="9"/>
       <c r="H55" s="9"/>
       <c r="I55" s="9"/>
@@ -10239,16 +10239,16 @@
       <c r="Z55" s="9"/>
     </row>
     <row r="56" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="71"/>
+      <c r="A56" s="74"/>
       <c r="B56" s="19"/>
       <c r="C56" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D56" s="98" t="s">
+      <c r="D56" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="E56" s="57"/>
-      <c r="F56" s="58"/>
+      <c r="E56" s="58"/>
+      <c r="F56" s="57"/>
       <c r="G56" s="9"/>
       <c r="H56" s="9"/>
       <c r="I56" s="9"/>
@@ -10271,18 +10271,18 @@
       <c r="Z56" s="9"/>
     </row>
     <row r="57" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="71"/>
+      <c r="A57" s="74"/>
       <c r="B57" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C57" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="D57" s="75" t="s">
+      <c r="D57" s="62" t="s">
         <v>1968</v>
       </c>
-      <c r="E57" s="57"/>
-      <c r="F57" s="58"/>
+      <c r="E57" s="58"/>
+      <c r="F57" s="57"/>
       <c r="G57" s="9"/>
       <c r="H57" s="9"/>
       <c r="I57" s="9"/>
@@ -10305,16 +10305,16 @@
       <c r="Z57" s="9"/>
     </row>
     <row r="58" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="71"/>
+      <c r="A58" s="74"/>
       <c r="B58" s="19"/>
       <c r="C58" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D58" s="98" t="s">
+      <c r="D58" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="E58" s="57"/>
-      <c r="F58" s="58"/>
+      <c r="E58" s="58"/>
+      <c r="F58" s="57"/>
       <c r="G58" s="9"/>
       <c r="H58" s="9"/>
       <c r="I58" s="9"/>
@@ -10337,16 +10337,16 @@
       <c r="Z58" s="9"/>
     </row>
     <row r="59" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="71"/>
+      <c r="A59" s="74"/>
       <c r="B59" s="19"/>
       <c r="C59" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D59" s="98" t="s">
+      <c r="D59" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="57"/>
-      <c r="F59" s="58"/>
+      <c r="E59" s="58"/>
+      <c r="F59" s="57"/>
       <c r="G59" s="9"/>
       <c r="H59" s="9"/>
       <c r="I59" s="9"/>
@@ -10369,16 +10369,16 @@
       <c r="Z59" s="9"/>
     </row>
     <row r="60" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="71"/>
+      <c r="A60" s="74"/>
       <c r="B60" s="19"/>
       <c r="C60" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D60" s="98" t="s">
+      <c r="D60" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="E60" s="57"/>
-      <c r="F60" s="58"/>
+      <c r="E60" s="58"/>
+      <c r="F60" s="57"/>
       <c r="G60" s="9"/>
       <c r="H60" s="9"/>
       <c r="I60" s="9"/>
@@ -10401,16 +10401,16 @@
       <c r="Z60" s="9"/>
     </row>
     <row r="61" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="72"/>
+      <c r="A61" s="75"/>
       <c r="B61" s="19"/>
       <c r="C61" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="D61" s="98" t="s">
+      <c r="D61" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="E61" s="57"/>
-      <c r="F61" s="58"/>
+      <c r="E61" s="58"/>
+      <c r="F61" s="57"/>
       <c r="G61" s="9"/>
       <c r="H61" s="9"/>
       <c r="I61" s="9"/>
@@ -10440,11 +10440,11 @@
         <v>50</v>
       </c>
       <c r="C62" s="19"/>
-      <c r="D62" s="98">
+      <c r="D62" s="61">
         <v>12</v>
       </c>
-      <c r="E62" s="57"/>
-      <c r="F62" s="58"/>
+      <c r="E62" s="58"/>
+      <c r="F62" s="57"/>
       <c r="G62" s="9"/>
       <c r="H62" s="9"/>
       <c r="I62" s="9"/>
@@ -10474,11 +10474,11 @@
         <v>51</v>
       </c>
       <c r="C63" s="19"/>
-      <c r="D63" s="98">
+      <c r="D63" s="61">
         <v>12</v>
       </c>
-      <c r="E63" s="57"/>
-      <c r="F63" s="58"/>
+      <c r="E63" s="58"/>
+      <c r="F63" s="57"/>
       <c r="G63" s="9"/>
       <c r="H63" s="9"/>
       <c r="I63" s="9"/>
@@ -10508,11 +10508,11 @@
         <v>52</v>
       </c>
       <c r="C64" s="19"/>
-      <c r="D64" s="98">
+      <c r="D64" s="61">
         <v>12</v>
       </c>
-      <c r="E64" s="57"/>
-      <c r="F64" s="58"/>
+      <c r="E64" s="58"/>
+      <c r="F64" s="57"/>
       <c r="G64" s="9"/>
       <c r="H64" s="9"/>
       <c r="I64" s="9"/>
@@ -10542,11 +10542,11 @@
         <v>53</v>
       </c>
       <c r="C65" s="19"/>
-      <c r="D65" s="98">
+      <c r="D65" s="61">
         <v>12</v>
       </c>
-      <c r="E65" s="57"/>
-      <c r="F65" s="58"/>
+      <c r="E65" s="58"/>
+      <c r="F65" s="57"/>
       <c r="G65" s="9"/>
       <c r="H65" s="9"/>
       <c r="I65" s="9"/>
@@ -10576,11 +10576,11 @@
         <v>54</v>
       </c>
       <c r="C66" s="19"/>
-      <c r="D66" s="98">
+      <c r="D66" s="61">
         <v>12</v>
       </c>
-      <c r="E66" s="57"/>
-      <c r="F66" s="58"/>
+      <c r="E66" s="58"/>
+      <c r="F66" s="57"/>
       <c r="G66" s="9"/>
       <c r="H66" s="9"/>
       <c r="I66" s="9"/>
@@ -10661,7 +10661,7 @@
       <c r="Z68" s="9"/>
     </row>
     <row r="69" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="70">
+      <c r="A69" s="73">
         <v>27</v>
       </c>
       <c r="B69" s="19" t="s">
@@ -10669,8 +10669,8 @@
       </c>
       <c r="C69" s="19"/>
       <c r="D69" s="60"/>
-      <c r="E69" s="57"/>
-      <c r="F69" s="58"/>
+      <c r="E69" s="58"/>
+      <c r="F69" s="57"/>
       <c r="G69" s="9"/>
       <c r="H69" s="9"/>
       <c r="I69" s="9"/>
@@ -10693,18 +10693,18 @@
       <c r="Z69" s="9"/>
     </row>
     <row r="70" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="71"/>
+      <c r="A70" s="74"/>
       <c r="B70" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C70" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D70" s="98">
+      <c r="D70" s="61">
         <v>67</v>
       </c>
-      <c r="E70" s="57"/>
-      <c r="F70" s="58"/>
+      <c r="E70" s="58"/>
+      <c r="F70" s="57"/>
       <c r="G70" s="9"/>
       <c r="H70" s="9"/>
       <c r="I70" s="9"/>
@@ -10727,18 +10727,18 @@
       <c r="Z70" s="9"/>
     </row>
     <row r="71" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="71"/>
+      <c r="A71" s="74"/>
       <c r="B71" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C71" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="D71" s="98">
+      <c r="D71" s="61">
         <v>67</v>
       </c>
-      <c r="E71" s="57"/>
-      <c r="F71" s="58"/>
+      <c r="E71" s="58"/>
+      <c r="F71" s="57"/>
       <c r="G71" s="9"/>
       <c r="H71" s="9"/>
       <c r="I71" s="9"/>
@@ -10761,16 +10761,16 @@
       <c r="Z71" s="9"/>
     </row>
     <row r="72" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="71"/>
+      <c r="A72" s="74"/>
       <c r="B72" s="11"/>
       <c r="C72" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="D72" s="98">
+      <c r="D72" s="61">
         <v>67</v>
       </c>
-      <c r="E72" s="57"/>
-      <c r="F72" s="58"/>
+      <c r="E72" s="58"/>
+      <c r="F72" s="57"/>
       <c r="G72" s="9"/>
       <c r="H72" s="9"/>
       <c r="I72" s="9"/>
@@ -10793,18 +10793,18 @@
       <c r="Z72" s="9"/>
     </row>
     <row r="73" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="71"/>
+      <c r="A73" s="74"/>
       <c r="B73" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C73" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="D73" s="98">
+      <c r="D73" s="61">
         <v>67</v>
       </c>
-      <c r="E73" s="57"/>
-      <c r="F73" s="58"/>
+      <c r="E73" s="58"/>
+      <c r="F73" s="57"/>
       <c r="G73" s="9"/>
       <c r="H73" s="9"/>
       <c r="I73" s="9"/>
@@ -10827,18 +10827,18 @@
       <c r="Z73" s="9"/>
     </row>
     <row r="74" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="71"/>
+      <c r="A74" s="74"/>
       <c r="B74" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C74" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D74" s="98">
+      <c r="D74" s="61">
         <v>67</v>
       </c>
-      <c r="E74" s="57"/>
-      <c r="F74" s="58"/>
+      <c r="E74" s="58"/>
+      <c r="F74" s="57"/>
       <c r="G74" s="9"/>
       <c r="H74" s="9"/>
       <c r="I74" s="9"/>
@@ -10861,18 +10861,18 @@
       <c r="Z74" s="9"/>
     </row>
     <row r="75" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="71"/>
+      <c r="A75" s="74"/>
       <c r="B75" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C75" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D75" s="98">
+      <c r="D75" s="61">
         <v>67</v>
       </c>
-      <c r="E75" s="57"/>
-      <c r="F75" s="58"/>
+      <c r="E75" s="58"/>
+      <c r="F75" s="57"/>
       <c r="G75" s="9"/>
       <c r="H75" s="9"/>
       <c r="I75" s="9"/>
@@ -10895,18 +10895,18 @@
       <c r="Z75" s="9"/>
     </row>
     <row r="76" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="71"/>
+      <c r="A76" s="74"/>
       <c r="B76" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C76" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="D76" s="98">
+      <c r="D76" s="61">
         <v>67</v>
       </c>
-      <c r="E76" s="57"/>
-      <c r="F76" s="58"/>
+      <c r="E76" s="58"/>
+      <c r="F76" s="57"/>
       <c r="G76" s="9"/>
       <c r="H76" s="9"/>
       <c r="I76" s="9"/>
@@ -10929,18 +10929,18 @@
       <c r="Z76" s="9"/>
     </row>
     <row r="77" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="72"/>
+      <c r="A77" s="75"/>
       <c r="B77" s="48" t="s">
         <v>1953</v>
       </c>
       <c r="C77" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D77" s="75" t="s">
+      <c r="D77" s="62" t="s">
         <v>1969</v>
       </c>
-      <c r="E77" s="57"/>
-      <c r="F77" s="58"/>
+      <c r="E77" s="58"/>
+      <c r="F77" s="57"/>
       <c r="G77" s="9"/>
       <c r="H77" s="9"/>
       <c r="I77" s="9"/>
@@ -10963,7 +10963,7 @@
       <c r="Z77" s="9"/>
     </row>
     <row r="78" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="70">
+      <c r="A78" s="73">
         <v>28</v>
       </c>
       <c r="B78" s="19" t="s">
@@ -10971,8 +10971,8 @@
       </c>
       <c r="C78" s="19"/>
       <c r="D78" s="60"/>
-      <c r="E78" s="57"/>
-      <c r="F78" s="58"/>
+      <c r="E78" s="58"/>
+      <c r="F78" s="57"/>
       <c r="G78" s="9"/>
       <c r="H78" s="9"/>
       <c r="I78" s="9"/>
@@ -10995,18 +10995,18 @@
       <c r="Z78" s="9"/>
     </row>
     <row r="79" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="71"/>
+      <c r="A79" s="74"/>
       <c r="B79" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C79" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="D79" s="98">
+      <c r="D79" s="61">
         <v>67</v>
       </c>
-      <c r="E79" s="57"/>
-      <c r="F79" s="58"/>
+      <c r="E79" s="58"/>
+      <c r="F79" s="57"/>
       <c r="G79" s="9"/>
       <c r="H79" s="9"/>
       <c r="I79" s="9"/>
@@ -11029,18 +11029,18 @@
       <c r="Z79" s="9"/>
     </row>
     <row r="80" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="71"/>
+      <c r="A80" s="74"/>
       <c r="B80" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C80" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="D80" s="98">
+      <c r="D80" s="61">
         <v>67</v>
       </c>
-      <c r="E80" s="57"/>
-      <c r="F80" s="58"/>
+      <c r="E80" s="58"/>
+      <c r="F80" s="57"/>
       <c r="G80" s="9"/>
       <c r="H80" s="9"/>
       <c r="I80" s="9"/>
@@ -11063,18 +11063,18 @@
       <c r="Z80" s="9"/>
     </row>
     <row r="81" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="71"/>
+      <c r="A81" s="74"/>
       <c r="B81" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C81" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="D81" s="98">
+      <c r="D81" s="61">
         <v>67</v>
       </c>
-      <c r="E81" s="57"/>
-      <c r="F81" s="58"/>
+      <c r="E81" s="58"/>
+      <c r="F81" s="57"/>
       <c r="G81" s="9"/>
       <c r="H81" s="9"/>
       <c r="I81" s="9"/>
@@ -11097,18 +11097,18 @@
       <c r="Z81" s="9"/>
     </row>
     <row r="82" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="71"/>
+      <c r="A82" s="74"/>
       <c r="B82" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C82" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="D82" s="75" t="s">
+      <c r="D82" s="62" t="s">
         <v>1970</v>
       </c>
-      <c r="E82" s="57"/>
-      <c r="F82" s="58"/>
+      <c r="E82" s="58"/>
+      <c r="F82" s="57"/>
       <c r="G82" s="9"/>
       <c r="H82" s="9"/>
       <c r="I82" s="9"/>
@@ -11131,18 +11131,18 @@
       <c r="Z82" s="9"/>
     </row>
     <row r="83" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="71"/>
+      <c r="A83" s="74"/>
       <c r="B83" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C83" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="D83" s="98">
+      <c r="D83" s="61">
         <v>67</v>
       </c>
-      <c r="E83" s="57"/>
-      <c r="F83" s="58"/>
+      <c r="E83" s="58"/>
+      <c r="F83" s="57"/>
       <c r="G83" s="9"/>
       <c r="H83" s="9"/>
       <c r="I83" s="9"/>
@@ -11165,18 +11165,18 @@
       <c r="Z83" s="9"/>
     </row>
     <row r="84" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="72"/>
+      <c r="A84" s="75"/>
       <c r="B84" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C84" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D84" s="75" t="s">
+      <c r="D84" s="62" t="s">
         <v>1971</v>
       </c>
-      <c r="E84" s="57"/>
-      <c r="F84" s="58"/>
+      <c r="E84" s="58"/>
+      <c r="F84" s="57"/>
       <c r="G84" s="9"/>
       <c r="H84" s="9"/>
       <c r="I84" s="9"/>
@@ -11206,11 +11206,11 @@
         <v>71</v>
       </c>
       <c r="C85" s="19"/>
-      <c r="D85" s="75" t="s">
+      <c r="D85" s="62" t="s">
         <v>1972</v>
       </c>
-      <c r="E85" s="57"/>
-      <c r="F85" s="58"/>
+      <c r="E85" s="58"/>
+      <c r="F85" s="57"/>
       <c r="G85" s="9"/>
       <c r="H85" s="9"/>
       <c r="I85" s="9"/>
@@ -11297,7 +11297,7 @@
       <c r="Z87" s="9"/>
     </row>
     <row r="88" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="70">
+      <c r="A88" s="73">
         <v>30</v>
       </c>
       <c r="B88" s="24" t="s">
@@ -11308,7 +11308,7 @@
         <v>0.92500000000000004</v>
       </c>
       <c r="E88" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F88" s="52" t="s">
         <v>1973</v>
@@ -11335,7 +11335,7 @@
       <c r="Z88" s="9"/>
     </row>
     <row r="89" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="71"/>
+      <c r="A89" s="74"/>
       <c r="B89" s="24" t="s">
         <v>77</v>
       </c>
@@ -11344,7 +11344,7 @@
         <v>0.96666666666666667</v>
       </c>
       <c r="E89" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F89" s="52" t="s">
         <v>1973</v>
@@ -11371,7 +11371,7 @@
       <c r="Z89" s="9"/>
     </row>
     <row r="90" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="71"/>
+      <c r="A90" s="74"/>
       <c r="B90" s="24" t="s">
         <v>78</v>
       </c>
@@ -11380,7 +11380,7 @@
         <v>1.5972222222222221E-2</v>
       </c>
       <c r="E90" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F90" s="52" t="s">
         <v>1973</v>
@@ -11407,7 +11407,7 @@
       <c r="Z90" s="9"/>
     </row>
     <row r="91" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="71"/>
+      <c r="A91" s="74"/>
       <c r="B91" s="24" t="s">
         <v>79</v>
       </c>
@@ -11416,7 +11416,7 @@
         <v>4.8611111111111112E-2</v>
       </c>
       <c r="E91" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F91" s="52" t="s">
         <v>1973</v>
@@ -11443,7 +11443,7 @@
       <c r="Z91" s="9"/>
     </row>
     <row r="92" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="71"/>
+      <c r="A92" s="74"/>
       <c r="B92" s="24" t="s">
         <v>80</v>
       </c>
@@ -11452,7 +11452,7 @@
         <v>4.9305555555555554E-2</v>
       </c>
       <c r="E92" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F92" s="52" t="s">
         <v>1973</v>
@@ -11479,7 +11479,7 @@
       <c r="Z92" s="9"/>
     </row>
     <row r="93" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="71"/>
+      <c r="A93" s="74"/>
       <c r="B93" s="24" t="s">
         <v>81</v>
       </c>
@@ -11488,7 +11488,7 @@
         <v>0.05</v>
       </c>
       <c r="E93" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F93" s="52" t="s">
         <v>1973</v>
@@ -11515,7 +11515,7 @@
       <c r="Z93" s="9"/>
     </row>
     <row r="94" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="71"/>
+      <c r="A94" s="74"/>
       <c r="B94" s="24" t="s">
         <v>82</v>
       </c>
@@ -11524,7 +11524,7 @@
         <v>5.1388888888888887E-2</v>
       </c>
       <c r="E94" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F94" s="52" t="s">
         <v>1973</v>
@@ -11551,7 +11551,7 @@
       <c r="Z94" s="9"/>
     </row>
     <row r="95" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="71"/>
+      <c r="A95" s="74"/>
       <c r="B95" s="24" t="s">
         <v>83</v>
       </c>
@@ -11560,7 +11560,7 @@
         <v>5.2083333333333336E-2</v>
       </c>
       <c r="E95" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F95" s="52" t="s">
         <v>1973</v>
@@ -11587,7 +11587,7 @@
       <c r="Z95" s="9"/>
     </row>
     <row r="96" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="71"/>
+      <c r="A96" s="74"/>
       <c r="B96" s="24" t="s">
         <v>84</v>
       </c>
@@ -11596,7 +11596,7 @@
         <v>5.2777777777777778E-2</v>
       </c>
       <c r="E96" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F96" s="52" t="s">
         <v>1973</v>
@@ -11623,7 +11623,7 @@
       <c r="Z96" s="9"/>
     </row>
     <row r="97" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="71"/>
+      <c r="A97" s="74"/>
       <c r="B97" s="24" t="s">
         <v>85</v>
       </c>
@@ -11632,7 +11632,7 @@
         <v>5.347222222222222E-2</v>
       </c>
       <c r="E97" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F97" s="52" t="s">
         <v>1973</v>
@@ -11659,7 +11659,7 @@
       <c r="Z97" s="9"/>
     </row>
     <row r="98" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="71"/>
+      <c r="A98" s="74"/>
       <c r="B98" s="24" t="s">
         <v>86</v>
       </c>
@@ -11668,7 +11668,7 @@
         <v>6.1805555555555558E-2</v>
       </c>
       <c r="E98" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F98" s="52" t="s">
         <v>1973</v>
@@ -11695,7 +11695,7 @@
       <c r="Z98" s="9"/>
     </row>
     <row r="99" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="71"/>
+      <c r="A99" s="74"/>
       <c r="B99" s="25" t="s">
         <v>87</v>
       </c>
@@ -11704,7 +11704,7 @@
         <v>9.8611111111111108E-2</v>
       </c>
       <c r="E99" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F99" s="52" t="s">
         <v>1973</v>
@@ -11731,7 +11731,7 @@
       <c r="Z99" s="9"/>
     </row>
     <row r="100" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="72"/>
+      <c r="A100" s="75"/>
       <c r="B100" s="25" t="s">
         <v>88</v>
       </c>
@@ -11740,7 +11740,7 @@
         <v>0.13194444444444445</v>
       </c>
       <c r="E100" s="51">
-        <v>38221</v>
+        <v>46202</v>
       </c>
       <c r="F100" s="52" t="s">
         <v>1973</v>
@@ -11767,16 +11767,16 @@
       <c r="Z100" s="9"/>
     </row>
     <row r="101" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="70">
+      <c r="A101" s="73">
         <v>31</v>
       </c>
-      <c r="B101" s="59" t="s">
+      <c r="B101" s="96" t="s">
         <v>89</v>
       </c>
-      <c r="C101" s="58"/>
-      <c r="D101" s="106"/>
-      <c r="E101" s="57"/>
-      <c r="F101" s="58"/>
+      <c r="C101" s="57"/>
+      <c r="D101" s="63"/>
+      <c r="E101" s="58"/>
+      <c r="F101" s="57"/>
       <c r="G101" s="9"/>
       <c r="H101" s="9"/>
       <c r="I101" s="9"/>
@@ -11799,18 +11799,18 @@
       <c r="Z101" s="9"/>
     </row>
     <row r="102" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="71"/>
+      <c r="A102" s="74"/>
       <c r="B102" s="47" t="s">
         <v>1953</v>
       </c>
       <c r="C102" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="D102" s="105" t="s">
+      <c r="D102" s="64" t="s">
         <v>1974</v>
       </c>
-      <c r="E102" s="57"/>
-      <c r="F102" s="58"/>
+      <c r="E102" s="58"/>
+      <c r="F102" s="57"/>
       <c r="G102" s="9"/>
       <c r="H102" s="9"/>
       <c r="I102" s="9"/>
@@ -11833,14 +11833,14 @@
       <c r="Z102" s="9"/>
     </row>
     <row r="103" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="72"/>
+      <c r="A103" s="75"/>
       <c r="B103" s="19"/>
       <c r="C103" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="D103" s="106"/>
-      <c r="E103" s="57"/>
-      <c r="F103" s="58"/>
+      <c r="D103" s="63"/>
+      <c r="E103" s="58"/>
+      <c r="F103" s="57"/>
       <c r="G103" s="9"/>
       <c r="H103" s="9"/>
       <c r="I103" s="9"/>
@@ -11925,7 +11925,7 @@
       <c r="Z105" s="9"/>
     </row>
     <row r="106" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="70">
+      <c r="A106" s="73">
         <v>32</v>
       </c>
       <c r="B106" s="19"/>
@@ -11961,7 +11961,7 @@
       <c r="Z106" s="9"/>
     </row>
     <row r="107" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="71"/>
+      <c r="A107" s="74"/>
       <c r="B107" s="19"/>
       <c r="C107" s="17" t="s">
         <v>96</v>
@@ -11995,7 +11995,7 @@
       <c r="Z107" s="9"/>
     </row>
     <row r="108" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="71"/>
+      <c r="A108" s="74"/>
       <c r="B108" s="19"/>
       <c r="C108" s="17" t="s">
         <v>97</v>
@@ -12029,7 +12029,7 @@
       <c r="Z108" s="9"/>
     </row>
     <row r="109" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="71"/>
+      <c r="A109" s="74"/>
       <c r="B109" s="19"/>
       <c r="C109" s="17" t="s">
         <v>98</v>
@@ -12063,7 +12063,7 @@
       <c r="Z109" s="9"/>
     </row>
     <row r="110" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="71"/>
+      <c r="A110" s="74"/>
       <c r="B110" s="19"/>
       <c r="C110" s="17" t="s">
         <v>99</v>
@@ -12097,7 +12097,7 @@
       <c r="Z110" s="9"/>
     </row>
     <row r="111" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="72"/>
+      <c r="A111" s="75"/>
       <c r="B111" s="19"/>
       <c r="C111" s="17" t="s">
         <v>100</v>
@@ -12164,11 +12164,11 @@
       </c>
       <c r="B113" s="8"/>
       <c r="C113" s="9"/>
-      <c r="D113" s="106" t="s">
+      <c r="D113" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="E113" s="57"/>
-      <c r="F113" s="58"/>
+      <c r="E113" s="58"/>
+      <c r="F113" s="57"/>
       <c r="G113" s="9"/>
       <c r="H113" s="9"/>
       <c r="I113" s="9"/>
@@ -12191,18 +12191,18 @@
       <c r="Z113" s="9"/>
     </row>
     <row r="114" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="70">
+      <c r="A114" s="73">
         <v>33</v>
       </c>
       <c r="B114" s="19" t="s">
         <v>103</v>
       </c>
       <c r="C114" s="19"/>
-      <c r="D114" s="105" t="s">
+      <c r="D114" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E114" s="57"/>
-      <c r="F114" s="58"/>
+      <c r="E114" s="58"/>
+      <c r="F114" s="57"/>
       <c r="G114" s="9"/>
       <c r="H114" s="9"/>
       <c r="I114" s="9"/>
@@ -12225,16 +12225,16 @@
       <c r="Z114" s="9"/>
     </row>
     <row r="115" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="71"/>
+      <c r="A115" s="74"/>
       <c r="B115" s="19" t="s">
         <v>104</v>
       </c>
       <c r="C115" s="19"/>
-      <c r="D115" s="105" t="s">
+      <c r="D115" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E115" s="57"/>
-      <c r="F115" s="58"/>
+      <c r="E115" s="58"/>
+      <c r="F115" s="57"/>
       <c r="G115" s="9"/>
       <c r="H115" s="9"/>
       <c r="I115" s="9"/>
@@ -12257,16 +12257,16 @@
       <c r="Z115" s="9"/>
     </row>
     <row r="116" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="71"/>
+      <c r="A116" s="74"/>
       <c r="B116" s="19" t="s">
         <v>105</v>
       </c>
       <c r="C116" s="19"/>
-      <c r="D116" s="105" t="s">
+      <c r="D116" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E116" s="57"/>
-      <c r="F116" s="58"/>
+      <c r="E116" s="58"/>
+      <c r="F116" s="57"/>
       <c r="G116" s="9"/>
       <c r="H116" s="9"/>
       <c r="I116" s="9"/>
@@ -12289,16 +12289,16 @@
       <c r="Z116" s="9"/>
     </row>
     <row r="117" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="71"/>
+      <c r="A117" s="74"/>
       <c r="B117" s="19" t="s">
         <v>106</v>
       </c>
       <c r="C117" s="19"/>
-      <c r="D117" s="105" t="s">
+      <c r="D117" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E117" s="57"/>
-      <c r="F117" s="58"/>
+      <c r="E117" s="58"/>
+      <c r="F117" s="57"/>
       <c r="G117" s="9"/>
       <c r="H117" s="9"/>
       <c r="I117" s="9"/>
@@ -12321,16 +12321,16 @@
       <c r="Z117" s="9"/>
     </row>
     <row r="118" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="71"/>
+      <c r="A118" s="74"/>
       <c r="B118" s="19" t="s">
         <v>107</v>
       </c>
       <c r="C118" s="19"/>
-      <c r="D118" s="105" t="s">
+      <c r="D118" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E118" s="57"/>
-      <c r="F118" s="58"/>
+      <c r="E118" s="58"/>
+      <c r="F118" s="57"/>
       <c r="G118" s="9"/>
       <c r="H118" s="9"/>
       <c r="I118" s="9"/>
@@ -12353,16 +12353,16 @@
       <c r="Z118" s="9"/>
     </row>
     <row r="119" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="71"/>
+      <c r="A119" s="74"/>
       <c r="B119" s="19" t="s">
         <v>108</v>
       </c>
       <c r="C119" s="19"/>
-      <c r="D119" s="105" t="s">
+      <c r="D119" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E119" s="57"/>
-      <c r="F119" s="58"/>
+      <c r="E119" s="58"/>
+      <c r="F119" s="57"/>
       <c r="G119" s="9"/>
       <c r="H119" s="9"/>
       <c r="I119" s="9"/>
@@ -12385,16 +12385,16 @@
       <c r="Z119" s="9"/>
     </row>
     <row r="120" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="71"/>
+      <c r="A120" s="74"/>
       <c r="B120" s="19" t="s">
         <v>109</v>
       </c>
       <c r="C120" s="19"/>
-      <c r="D120" s="105" t="s">
+      <c r="D120" s="64" t="s">
         <v>1975</v>
       </c>
-      <c r="E120" s="57"/>
-      <c r="F120" s="58"/>
+      <c r="E120" s="58"/>
+      <c r="F120" s="57"/>
       <c r="G120" s="9"/>
       <c r="H120" s="9"/>
       <c r="I120" s="9"/>
@@ -12417,16 +12417,16 @@
       <c r="Z120" s="9"/>
     </row>
     <row r="121" spans="1:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="72"/>
-      <c r="B121" s="81" t="s">
+      <c r="A121" s="75"/>
+      <c r="B121" s="97" t="s">
         <v>110</v>
       </c>
-      <c r="C121" s="58"/>
-      <c r="D121" s="105" t="s">
+      <c r="C121" s="57"/>
+      <c r="D121" s="64" t="s">
         <v>1976</v>
       </c>
-      <c r="E121" s="57"/>
-      <c r="F121" s="58"/>
+      <c r="E121" s="58"/>
+      <c r="F121" s="57"/>
       <c r="G121" s="9"/>
       <c r="H121" s="9"/>
       <c r="I121" s="9"/>
@@ -12477,16 +12477,16 @@
       <c r="Z122" s="9"/>
     </row>
     <row r="123" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="74" t="s">
+      <c r="A123" s="105" t="s">
         <v>111</v>
       </c>
-      <c r="B123" s="68"/>
-      <c r="C123" s="68"/>
-      <c r="D123" s="69"/>
-      <c r="E123" s="106" t="s">
+      <c r="B123" s="86"/>
+      <c r="C123" s="86"/>
+      <c r="D123" s="87"/>
+      <c r="E123" s="63" t="s">
         <v>112</v>
       </c>
-      <c r="F123" s="58"/>
+      <c r="F123" s="57"/>
       <c r="G123" s="9"/>
       <c r="H123" s="9"/>
       <c r="I123" s="9"/>
@@ -12509,18 +12509,18 @@
       <c r="Z123" s="9"/>
     </row>
     <row r="124" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="70">
+      <c r="A124" s="73">
         <v>34</v>
       </c>
-      <c r="B124" s="75" t="s">
+      <c r="B124" s="62" t="s">
         <v>1977</v>
       </c>
-      <c r="C124" s="57"/>
-      <c r="D124" s="58"/>
-      <c r="E124" s="76" t="s">
+      <c r="C124" s="58"/>
+      <c r="D124" s="57"/>
+      <c r="E124" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F124" s="58"/>
+      <c r="F124" s="57"/>
       <c r="G124" s="9"/>
       <c r="H124" s="9"/>
       <c r="I124" s="9"/>
@@ -12543,16 +12543,16 @@
       <c r="Z124" s="9"/>
     </row>
     <row r="125" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="71"/>
-      <c r="B125" s="75" t="s">
+      <c r="A125" s="74"/>
+      <c r="B125" s="62" t="s">
         <v>1965</v>
       </c>
-      <c r="C125" s="57"/>
-      <c r="D125" s="58"/>
-      <c r="E125" s="76" t="s">
+      <c r="C125" s="58"/>
+      <c r="D125" s="57"/>
+      <c r="E125" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F125" s="58"/>
+      <c r="F125" s="57"/>
       <c r="G125" s="9"/>
       <c r="H125" s="9"/>
       <c r="I125" s="9"/>
@@ -12575,16 +12575,16 @@
       <c r="Z125" s="9"/>
     </row>
     <row r="126" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="71"/>
-      <c r="B126" s="75" t="s">
+      <c r="A126" s="74"/>
+      <c r="B126" s="62" t="s">
         <v>1978</v>
       </c>
-      <c r="C126" s="57"/>
-      <c r="D126" s="58"/>
-      <c r="E126" s="76" t="s">
+      <c r="C126" s="58"/>
+      <c r="D126" s="57"/>
+      <c r="E126" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F126" s="58"/>
+      <c r="F126" s="57"/>
       <c r="G126" s="9"/>
       <c r="H126" s="9"/>
       <c r="I126" s="9"/>
@@ -12607,16 +12607,16 @@
       <c r="Z126" s="9"/>
     </row>
     <row r="127" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="71"/>
-      <c r="B127" s="76" t="s">
+      <c r="A127" s="74"/>
+      <c r="B127" s="56" t="s">
         <v>1979</v>
       </c>
-      <c r="C127" s="77"/>
-      <c r="D127" s="78"/>
-      <c r="E127" s="76" t="s">
+      <c r="C127" s="106"/>
+      <c r="D127" s="107"/>
+      <c r="E127" s="56" t="s">
         <v>1980</v>
       </c>
-      <c r="F127" s="58"/>
+      <c r="F127" s="57"/>
       <c r="G127" s="9"/>
       <c r="H127" s="9"/>
       <c r="I127" s="9"/>
@@ -12639,12 +12639,12 @@
       <c r="Z127" s="9"/>
     </row>
     <row r="128" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="71"/>
+      <c r="A128" s="74"/>
       <c r="B128" s="60"/>
-      <c r="C128" s="57"/>
-      <c r="D128" s="58"/>
+      <c r="C128" s="58"/>
+      <c r="D128" s="57"/>
       <c r="E128" s="60"/>
-      <c r="F128" s="58"/>
+      <c r="F128" s="57"/>
       <c r="G128" s="9"/>
       <c r="H128" s="9"/>
       <c r="I128" s="9"/>
@@ -12667,12 +12667,12 @@
       <c r="Z128" s="9"/>
     </row>
     <row r="129" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="71"/>
+      <c r="A129" s="74"/>
       <c r="B129" s="60"/>
-      <c r="C129" s="57"/>
-      <c r="D129" s="58"/>
+      <c r="C129" s="58"/>
+      <c r="D129" s="57"/>
       <c r="E129" s="60"/>
-      <c r="F129" s="58"/>
+      <c r="F129" s="57"/>
       <c r="G129" s="9"/>
       <c r="H129" s="9"/>
       <c r="I129" s="9"/>
@@ -12695,12 +12695,12 @@
       <c r="Z129" s="9"/>
     </row>
     <row r="130" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="71"/>
+      <c r="A130" s="74"/>
       <c r="B130" s="60"/>
-      <c r="C130" s="57"/>
-      <c r="D130" s="58"/>
+      <c r="C130" s="58"/>
+      <c r="D130" s="57"/>
       <c r="E130" s="60"/>
-      <c r="F130" s="58"/>
+      <c r="F130" s="57"/>
       <c r="G130" s="9"/>
       <c r="H130" s="9"/>
       <c r="I130" s="9"/>
@@ -12723,12 +12723,12 @@
       <c r="Z130" s="9"/>
     </row>
     <row r="131" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="71"/>
+      <c r="A131" s="74"/>
       <c r="B131" s="60"/>
-      <c r="C131" s="57"/>
-      <c r="D131" s="58"/>
+      <c r="C131" s="58"/>
+      <c r="D131" s="57"/>
       <c r="E131" s="60"/>
-      <c r="F131" s="58"/>
+      <c r="F131" s="57"/>
       <c r="G131" s="9"/>
       <c r="H131" s="9"/>
       <c r="I131" s="9"/>
@@ -12751,12 +12751,12 @@
       <c r="Z131" s="9"/>
     </row>
     <row r="132" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="72"/>
+      <c r="A132" s="75"/>
       <c r="B132" s="60"/>
-      <c r="C132" s="57"/>
-      <c r="D132" s="58"/>
+      <c r="C132" s="58"/>
+      <c r="D132" s="57"/>
       <c r="E132" s="60"/>
-      <c r="F132" s="58"/>
+      <c r="F132" s="57"/>
       <c r="G132" s="9"/>
       <c r="H132" s="9"/>
       <c r="I132" s="9"/>
@@ -12837,14 +12837,14 @@
       <c r="Z134" s="9"/>
     </row>
     <row r="135" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="70">
+      <c r="A135" s="73">
         <v>35</v>
       </c>
-      <c r="B135" s="79"/>
-      <c r="C135" s="62"/>
-      <c r="D135" s="62"/>
-      <c r="E135" s="62"/>
-      <c r="F135" s="63"/>
+      <c r="B135" s="100"/>
+      <c r="C135" s="84"/>
+      <c r="D135" s="84"/>
+      <c r="E135" s="84"/>
+      <c r="F135" s="79"/>
       <c r="G135" s="9"/>
       <c r="H135" s="9"/>
       <c r="I135" s="9"/>
@@ -12867,12 +12867,12 @@
       <c r="Z135" s="9"/>
     </row>
     <row r="136" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="71"/>
-      <c r="B136" s="64"/>
-      <c r="C136" s="65"/>
-      <c r="D136" s="65"/>
-      <c r="E136" s="65"/>
-      <c r="F136" s="66"/>
+      <c r="A136" s="74"/>
+      <c r="B136" s="80"/>
+      <c r="C136" s="66"/>
+      <c r="D136" s="66"/>
+      <c r="E136" s="66"/>
+      <c r="F136" s="81"/>
       <c r="G136" s="9"/>
       <c r="H136" s="9"/>
       <c r="I136" s="9"/>
@@ -12895,12 +12895,12 @@
       <c r="Z136" s="9"/>
     </row>
     <row r="137" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="71"/>
-      <c r="B137" s="64"/>
-      <c r="C137" s="65"/>
-      <c r="D137" s="65"/>
-      <c r="E137" s="65"/>
-      <c r="F137" s="66"/>
+      <c r="A137" s="74"/>
+      <c r="B137" s="80"/>
+      <c r="C137" s="66"/>
+      <c r="D137" s="66"/>
+      <c r="E137" s="66"/>
+      <c r="F137" s="81"/>
       <c r="G137" s="9"/>
       <c r="H137" s="9"/>
       <c r="I137" s="9"/>
@@ -12923,12 +12923,12 @@
       <c r="Z137" s="9"/>
     </row>
     <row r="138" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="71"/>
-      <c r="B138" s="64"/>
-      <c r="C138" s="65"/>
-      <c r="D138" s="65"/>
-      <c r="E138" s="65"/>
-      <c r="F138" s="66"/>
+      <c r="A138" s="74"/>
+      <c r="B138" s="80"/>
+      <c r="C138" s="66"/>
+      <c r="D138" s="66"/>
+      <c r="E138" s="66"/>
+      <c r="F138" s="81"/>
       <c r="G138" s="9"/>
       <c r="H138" s="9"/>
       <c r="I138" s="9"/>
@@ -12951,12 +12951,12 @@
       <c r="Z138" s="9"/>
     </row>
     <row r="139" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="71"/>
-      <c r="B139" s="64"/>
-      <c r="C139" s="65"/>
-      <c r="D139" s="65"/>
-      <c r="E139" s="65"/>
-      <c r="F139" s="66"/>
+      <c r="A139" s="74"/>
+      <c r="B139" s="80"/>
+      <c r="C139" s="66"/>
+      <c r="D139" s="66"/>
+      <c r="E139" s="66"/>
+      <c r="F139" s="81"/>
       <c r="G139" s="9"/>
       <c r="H139" s="9"/>
       <c r="I139" s="9"/>
@@ -12979,12 +12979,12 @@
       <c r="Z139" s="9"/>
     </row>
     <row r="140" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="71"/>
-      <c r="B140" s="64"/>
-      <c r="C140" s="65"/>
-      <c r="D140" s="65"/>
-      <c r="E140" s="65"/>
-      <c r="F140" s="66"/>
+      <c r="A140" s="74"/>
+      <c r="B140" s="80"/>
+      <c r="C140" s="66"/>
+      <c r="D140" s="66"/>
+      <c r="E140" s="66"/>
+      <c r="F140" s="81"/>
       <c r="G140" s="9"/>
       <c r="H140" s="9"/>
       <c r="I140" s="9"/>
@@ -13007,12 +13007,12 @@
       <c r="Z140" s="9"/>
     </row>
     <row r="141" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="71"/>
-      <c r="B141" s="64"/>
-      <c r="C141" s="65"/>
-      <c r="D141" s="65"/>
-      <c r="E141" s="65"/>
-      <c r="F141" s="66"/>
+      <c r="A141" s="74"/>
+      <c r="B141" s="80"/>
+      <c r="C141" s="66"/>
+      <c r="D141" s="66"/>
+      <c r="E141" s="66"/>
+      <c r="F141" s="81"/>
       <c r="G141" s="9"/>
       <c r="H141" s="9"/>
       <c r="I141" s="9"/>
@@ -13035,12 +13035,12 @@
       <c r="Z141" s="9"/>
     </row>
     <row r="142" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="71"/>
-      <c r="B142" s="64"/>
-      <c r="C142" s="65"/>
-      <c r="D142" s="65"/>
-      <c r="E142" s="65"/>
-      <c r="F142" s="66"/>
+      <c r="A142" s="74"/>
+      <c r="B142" s="80"/>
+      <c r="C142" s="66"/>
+      <c r="D142" s="66"/>
+      <c r="E142" s="66"/>
+      <c r="F142" s="81"/>
       <c r="G142" s="9"/>
       <c r="H142" s="9"/>
       <c r="I142" s="9"/>
@@ -13063,12 +13063,12 @@
       <c r="Z142" s="9"/>
     </row>
     <row r="143" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A143" s="71"/>
-      <c r="B143" s="64"/>
-      <c r="C143" s="65"/>
-      <c r="D143" s="65"/>
-      <c r="E143" s="65"/>
-      <c r="F143" s="66"/>
+      <c r="A143" s="74"/>
+      <c r="B143" s="80"/>
+      <c r="C143" s="66"/>
+      <c r="D143" s="66"/>
+      <c r="E143" s="66"/>
+      <c r="F143" s="81"/>
       <c r="G143" s="9"/>
       <c r="H143" s="9"/>
       <c r="I143" s="9"/>
@@ -13091,12 +13091,12 @@
       <c r="Z143" s="9"/>
     </row>
     <row r="144" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="71"/>
-      <c r="B144" s="64"/>
-      <c r="C144" s="65"/>
-      <c r="D144" s="65"/>
-      <c r="E144" s="65"/>
-      <c r="F144" s="66"/>
+      <c r="A144" s="74"/>
+      <c r="B144" s="80"/>
+      <c r="C144" s="66"/>
+      <c r="D144" s="66"/>
+      <c r="E144" s="66"/>
+      <c r="F144" s="81"/>
       <c r="G144" s="9"/>
       <c r="H144" s="9"/>
       <c r="I144" s="9"/>
@@ -13119,12 +13119,12 @@
       <c r="Z144" s="9"/>
     </row>
     <row r="145" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="71"/>
-      <c r="B145" s="64"/>
-      <c r="C145" s="65"/>
-      <c r="D145" s="65"/>
-      <c r="E145" s="65"/>
-      <c r="F145" s="66"/>
+      <c r="A145" s="74"/>
+      <c r="B145" s="80"/>
+      <c r="C145" s="66"/>
+      <c r="D145" s="66"/>
+      <c r="E145" s="66"/>
+      <c r="F145" s="81"/>
       <c r="G145" s="9"/>
       <c r="H145" s="9"/>
       <c r="I145" s="9"/>
@@ -13147,12 +13147,12 @@
       <c r="Z145" s="9"/>
     </row>
     <row r="146" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="71"/>
-      <c r="B146" s="64"/>
-      <c r="C146" s="65"/>
-      <c r="D146" s="65"/>
-      <c r="E146" s="65"/>
-      <c r="F146" s="66"/>
+      <c r="A146" s="74"/>
+      <c r="B146" s="80"/>
+      <c r="C146" s="66"/>
+      <c r="D146" s="66"/>
+      <c r="E146" s="66"/>
+      <c r="F146" s="81"/>
       <c r="G146" s="9"/>
       <c r="H146" s="9"/>
       <c r="I146" s="9"/>
@@ -13175,12 +13175,12 @@
       <c r="Z146" s="9"/>
     </row>
     <row r="147" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="71"/>
-      <c r="B147" s="64"/>
-      <c r="C147" s="65"/>
-      <c r="D147" s="65"/>
-      <c r="E147" s="65"/>
-      <c r="F147" s="66"/>
+      <c r="A147" s="74"/>
+      <c r="B147" s="80"/>
+      <c r="C147" s="66"/>
+      <c r="D147" s="66"/>
+      <c r="E147" s="66"/>
+      <c r="F147" s="81"/>
       <c r="G147" s="9"/>
       <c r="H147" s="9"/>
       <c r="I147" s="9"/>
@@ -13203,12 +13203,12 @@
       <c r="Z147" s="9"/>
     </row>
     <row r="148" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="71"/>
-      <c r="B148" s="64"/>
-      <c r="C148" s="65"/>
-      <c r="D148" s="65"/>
-      <c r="E148" s="65"/>
-      <c r="F148" s="66"/>
+      <c r="A148" s="74"/>
+      <c r="B148" s="80"/>
+      <c r="C148" s="66"/>
+      <c r="D148" s="66"/>
+      <c r="E148" s="66"/>
+      <c r="F148" s="81"/>
       <c r="G148" s="9"/>
       <c r="H148" s="9"/>
       <c r="I148" s="9"/>
@@ -13231,12 +13231,12 @@
       <c r="Z148" s="9"/>
     </row>
     <row r="149" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="71"/>
-      <c r="B149" s="64"/>
-      <c r="C149" s="65"/>
-      <c r="D149" s="65"/>
-      <c r="E149" s="65"/>
-      <c r="F149" s="66"/>
+      <c r="A149" s="74"/>
+      <c r="B149" s="80"/>
+      <c r="C149" s="66"/>
+      <c r="D149" s="66"/>
+      <c r="E149" s="66"/>
+      <c r="F149" s="81"/>
       <c r="G149" s="9"/>
       <c r="H149" s="9"/>
       <c r="I149" s="9"/>
@@ -13259,12 +13259,12 @@
       <c r="Z149" s="9"/>
     </row>
     <row r="150" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="71"/>
-      <c r="B150" s="64"/>
-      <c r="C150" s="65"/>
-      <c r="D150" s="65"/>
-      <c r="E150" s="65"/>
-      <c r="F150" s="66"/>
+      <c r="A150" s="74"/>
+      <c r="B150" s="80"/>
+      <c r="C150" s="66"/>
+      <c r="D150" s="66"/>
+      <c r="E150" s="66"/>
+      <c r="F150" s="81"/>
       <c r="G150" s="9"/>
       <c r="H150" s="9"/>
       <c r="I150" s="9"/>
@@ -13287,12 +13287,12 @@
       <c r="Z150" s="9"/>
     </row>
     <row r="151" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="71"/>
-      <c r="B151" s="64"/>
-      <c r="C151" s="65"/>
-      <c r="D151" s="65"/>
-      <c r="E151" s="65"/>
-      <c r="F151" s="66"/>
+      <c r="A151" s="74"/>
+      <c r="B151" s="80"/>
+      <c r="C151" s="66"/>
+      <c r="D151" s="66"/>
+      <c r="E151" s="66"/>
+      <c r="F151" s="81"/>
       <c r="G151" s="9"/>
       <c r="H151" s="9"/>
       <c r="I151" s="9"/>
@@ -13315,12 +13315,12 @@
       <c r="Z151" s="9"/>
     </row>
     <row r="152" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="71"/>
-      <c r="B152" s="64"/>
-      <c r="C152" s="65"/>
-      <c r="D152" s="65"/>
-      <c r="E152" s="65"/>
-      <c r="F152" s="66"/>
+      <c r="A152" s="74"/>
+      <c r="B152" s="80"/>
+      <c r="C152" s="66"/>
+      <c r="D152" s="66"/>
+      <c r="E152" s="66"/>
+      <c r="F152" s="81"/>
       <c r="G152" s="9"/>
       <c r="H152" s="9"/>
       <c r="I152" s="9"/>
@@ -13343,12 +13343,12 @@
       <c r="Z152" s="9"/>
     </row>
     <row r="153" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="71"/>
-      <c r="B153" s="64"/>
-      <c r="C153" s="65"/>
-      <c r="D153" s="65"/>
-      <c r="E153" s="65"/>
-      <c r="F153" s="66"/>
+      <c r="A153" s="74"/>
+      <c r="B153" s="80"/>
+      <c r="C153" s="66"/>
+      <c r="D153" s="66"/>
+      <c r="E153" s="66"/>
+      <c r="F153" s="81"/>
       <c r="G153" s="9"/>
       <c r="H153" s="9"/>
       <c r="I153" s="9"/>
@@ -13371,12 +13371,12 @@
       <c r="Z153" s="9"/>
     </row>
     <row r="154" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="71"/>
-      <c r="B154" s="64"/>
-      <c r="C154" s="65"/>
-      <c r="D154" s="65"/>
-      <c r="E154" s="65"/>
-      <c r="F154" s="66"/>
+      <c r="A154" s="74"/>
+      <c r="B154" s="80"/>
+      <c r="C154" s="66"/>
+      <c r="D154" s="66"/>
+      <c r="E154" s="66"/>
+      <c r="F154" s="81"/>
       <c r="G154" s="9"/>
       <c r="H154" s="9"/>
       <c r="I154" s="9"/>
@@ -13399,12 +13399,12 @@
       <c r="Z154" s="9"/>
     </row>
     <row r="155" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="71"/>
-      <c r="B155" s="64"/>
-      <c r="C155" s="65"/>
-      <c r="D155" s="65"/>
-      <c r="E155" s="65"/>
-      <c r="F155" s="66"/>
+      <c r="A155" s="74"/>
+      <c r="B155" s="80"/>
+      <c r="C155" s="66"/>
+      <c r="D155" s="66"/>
+      <c r="E155" s="66"/>
+      <c r="F155" s="81"/>
       <c r="G155" s="9"/>
       <c r="H155" s="9"/>
       <c r="I155" s="9"/>
@@ -13427,12 +13427,12 @@
       <c r="Z155" s="9"/>
     </row>
     <row r="156" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="71"/>
-      <c r="B156" s="64"/>
-      <c r="C156" s="65"/>
-      <c r="D156" s="65"/>
-      <c r="E156" s="65"/>
-      <c r="F156" s="66"/>
+      <c r="A156" s="74"/>
+      <c r="B156" s="80"/>
+      <c r="C156" s="66"/>
+      <c r="D156" s="66"/>
+      <c r="E156" s="66"/>
+      <c r="F156" s="81"/>
       <c r="G156" s="9"/>
       <c r="H156" s="9"/>
       <c r="I156" s="9"/>
@@ -13455,12 +13455,12 @@
       <c r="Z156" s="9"/>
     </row>
     <row r="157" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="72"/>
-      <c r="B157" s="67"/>
-      <c r="C157" s="68"/>
-      <c r="D157" s="68"/>
-      <c r="E157" s="68"/>
-      <c r="F157" s="69"/>
+      <c r="A157" s="75"/>
+      <c r="B157" s="85"/>
+      <c r="C157" s="86"/>
+      <c r="D157" s="86"/>
+      <c r="E157" s="86"/>
+      <c r="F157" s="87"/>
       <c r="G157" s="9"/>
       <c r="H157" s="9"/>
       <c r="I157" s="9"/>
@@ -13541,16 +13541,16 @@
       <c r="Z159" s="9"/>
     </row>
     <row r="160" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="70">
+      <c r="A160" s="73">
         <v>36</v>
       </c>
-      <c r="B160" s="86" t="s">
+      <c r="B160" s="82" t="s">
         <v>115</v>
       </c>
-      <c r="C160" s="57"/>
-      <c r="D160" s="57"/>
-      <c r="E160" s="57"/>
-      <c r="F160" s="58"/>
+      <c r="C160" s="58"/>
+      <c r="D160" s="58"/>
+      <c r="E160" s="58"/>
+      <c r="F160" s="57"/>
       <c r="G160" s="9"/>
       <c r="H160" s="9"/>
       <c r="I160" s="9"/>
@@ -13573,14 +13573,14 @@
       <c r="Z160" s="9"/>
     </row>
     <row r="161" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="71"/>
-      <c r="B161" s="87" t="s">
+      <c r="A161" s="74"/>
+      <c r="B161" s="83" t="s">
         <v>1981</v>
       </c>
-      <c r="C161" s="62"/>
-      <c r="D161" s="62"/>
-      <c r="E161" s="62"/>
-      <c r="F161" s="63"/>
+      <c r="C161" s="84"/>
+      <c r="D161" s="84"/>
+      <c r="E161" s="84"/>
+      <c r="F161" s="79"/>
       <c r="G161" s="9"/>
       <c r="H161" s="9"/>
       <c r="I161" s="9"/>
@@ -13603,12 +13603,12 @@
       <c r="Z161" s="9"/>
     </row>
     <row r="162" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="71"/>
-      <c r="B162" s="67"/>
-      <c r="C162" s="68"/>
-      <c r="D162" s="68"/>
-      <c r="E162" s="68"/>
-      <c r="F162" s="69"/>
+      <c r="A162" s="74"/>
+      <c r="B162" s="85"/>
+      <c r="C162" s="86"/>
+      <c r="D162" s="86"/>
+      <c r="E162" s="86"/>
+      <c r="F162" s="87"/>
       <c r="G162" s="9"/>
       <c r="H162" s="9"/>
       <c r="I162" s="9"/>
@@ -13631,12 +13631,12 @@
       <c r="Z162" s="9"/>
     </row>
     <row r="163" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A163" s="71"/>
+      <c r="A163" s="74"/>
       <c r="B163" s="88"/>
-      <c r="C163" s="57"/>
-      <c r="D163" s="57"/>
-      <c r="E163" s="57"/>
-      <c r="F163" s="58"/>
+      <c r="C163" s="58"/>
+      <c r="D163" s="58"/>
+      <c r="E163" s="58"/>
+      <c r="F163" s="57"/>
       <c r="G163" s="9"/>
       <c r="H163" s="9"/>
       <c r="I163" s="9"/>
@@ -13659,14 +13659,14 @@
       <c r="Z163" s="9"/>
     </row>
     <row r="164" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A164" s="71"/>
-      <c r="B164" s="85" t="s">
+      <c r="A164" s="74"/>
+      <c r="B164" s="89" t="s">
         <v>116</v>
       </c>
-      <c r="C164" s="62"/>
-      <c r="D164" s="62"/>
-      <c r="E164" s="62"/>
-      <c r="F164" s="63"/>
+      <c r="C164" s="84"/>
+      <c r="D164" s="84"/>
+      <c r="E164" s="84"/>
+      <c r="F164" s="79"/>
       <c r="G164" s="9"/>
       <c r="H164" s="9"/>
       <c r="I164" s="9"/>
@@ -13689,12 +13689,12 @@
       <c r="Z164" s="9"/>
     </row>
     <row r="165" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A165" s="71"/>
-      <c r="B165" s="64"/>
-      <c r="C165" s="65"/>
-      <c r="D165" s="65"/>
-      <c r="E165" s="65"/>
-      <c r="F165" s="66"/>
+      <c r="A165" s="74"/>
+      <c r="B165" s="80"/>
+      <c r="C165" s="66"/>
+      <c r="D165" s="66"/>
+      <c r="E165" s="66"/>
+      <c r="F165" s="81"/>
       <c r="G165" s="9"/>
       <c r="H165" s="9"/>
       <c r="I165" s="9"/>
@@ -13717,12 +13717,12 @@
       <c r="Z165" s="9"/>
     </row>
     <row r="166" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="71"/>
-      <c r="B166" s="64"/>
-      <c r="C166" s="65"/>
-      <c r="D166" s="65"/>
-      <c r="E166" s="65"/>
-      <c r="F166" s="66"/>
+      <c r="A166" s="74"/>
+      <c r="B166" s="80"/>
+      <c r="C166" s="66"/>
+      <c r="D166" s="66"/>
+      <c r="E166" s="66"/>
+      <c r="F166" s="81"/>
       <c r="G166" s="9"/>
       <c r="H166" s="9"/>
       <c r="I166" s="9"/>
@@ -13745,12 +13745,12 @@
       <c r="Z166" s="9"/>
     </row>
     <row r="167" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="71"/>
-      <c r="B167" s="67"/>
-      <c r="C167" s="68"/>
-      <c r="D167" s="68"/>
-      <c r="E167" s="68"/>
-      <c r="F167" s="69"/>
+      <c r="A167" s="74"/>
+      <c r="B167" s="85"/>
+      <c r="C167" s="86"/>
+      <c r="D167" s="86"/>
+      <c r="E167" s="86"/>
+      <c r="F167" s="87"/>
       <c r="G167" s="9"/>
       <c r="H167" s="9"/>
       <c r="I167" s="9"/>
@@ -13773,7 +13773,7 @@
       <c r="Z167" s="9"/>
     </row>
     <row r="168" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="71"/>
+      <c r="A168" s="74"/>
       <c r="B168" s="47" t="s">
         <v>1982</v>
       </c>
@@ -13803,14 +13803,14 @@
       <c r="Z168" s="9"/>
     </row>
     <row r="169" spans="1:26" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A169" s="71"/>
-      <c r="B169" s="89" t="s">
+      <c r="A169" s="74"/>
+      <c r="B169" s="90" t="s">
         <v>1983</v>
       </c>
-      <c r="C169" s="57"/>
-      <c r="D169" s="57"/>
-      <c r="E169" s="57"/>
-      <c r="F169" s="58"/>
+      <c r="C169" s="58"/>
+      <c r="D169" s="58"/>
+      <c r="E169" s="58"/>
+      <c r="F169" s="57"/>
       <c r="G169" s="29"/>
       <c r="H169" s="29"/>
       <c r="I169" s="29"/>
@@ -13833,14 +13833,14 @@
       <c r="Z169" s="29"/>
     </row>
     <row r="170" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="71"/>
-      <c r="B170" s="90" t="s">
+      <c r="A170" s="74"/>
+      <c r="B170" s="91" t="s">
         <v>117</v>
       </c>
-      <c r="C170" s="57"/>
-      <c r="D170" s="57"/>
-      <c r="E170" s="57"/>
-      <c r="F170" s="58"/>
+      <c r="C170" s="58"/>
+      <c r="D170" s="58"/>
+      <c r="E170" s="58"/>
+      <c r="F170" s="57"/>
       <c r="G170" s="9"/>
       <c r="H170" s="9"/>
       <c r="I170" s="9"/>
@@ -13863,14 +13863,14 @@
       <c r="Z170" s="9"/>
     </row>
     <row r="171" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A171" s="71"/>
-      <c r="B171" s="85" t="s">
+      <c r="A171" s="74"/>
+      <c r="B171" s="89" t="s">
         <v>118</v>
       </c>
-      <c r="C171" s="62"/>
-      <c r="D171" s="62"/>
-      <c r="E171" s="62"/>
-      <c r="F171" s="63"/>
+      <c r="C171" s="84"/>
+      <c r="D171" s="84"/>
+      <c r="E171" s="84"/>
+      <c r="F171" s="79"/>
       <c r="G171" s="9"/>
       <c r="H171" s="9"/>
       <c r="I171" s="9"/>
@@ -13893,12 +13893,12 @@
       <c r="Z171" s="9"/>
     </row>
     <row r="172" spans="1:26" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A172" s="71"/>
-      <c r="B172" s="67"/>
-      <c r="C172" s="68"/>
-      <c r="D172" s="68"/>
-      <c r="E172" s="68"/>
-      <c r="F172" s="69"/>
+      <c r="A172" s="74"/>
+      <c r="B172" s="85"/>
+      <c r="C172" s="86"/>
+      <c r="D172" s="86"/>
+      <c r="E172" s="86"/>
+      <c r="F172" s="87"/>
       <c r="G172" s="9"/>
       <c r="H172" s="9"/>
       <c r="I172" s="9"/>
@@ -13921,7 +13921,7 @@
       <c r="Z172" s="9"/>
     </row>
     <row r="173" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="71"/>
+      <c r="A173" s="74"/>
       <c r="B173" s="19" t="s">
         <v>119</v>
       </c>
@@ -13951,14 +13951,14 @@
       <c r="Z173" s="9"/>
     </row>
     <row r="174" spans="1:26" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="71"/>
-      <c r="B174" s="56" t="s">
+      <c r="A174" s="74"/>
+      <c r="B174" s="102" t="s">
         <v>120</v>
       </c>
-      <c r="C174" s="57"/>
-      <c r="D174" s="57"/>
-      <c r="E174" s="57"/>
-      <c r="F174" s="58"/>
+      <c r="C174" s="58"/>
+      <c r="D174" s="58"/>
+      <c r="E174" s="58"/>
+      <c r="F174" s="57"/>
       <c r="G174" s="9"/>
       <c r="H174" s="9"/>
       <c r="I174" s="9"/>
@@ -13981,14 +13981,14 @@
       <c r="Z174" s="9"/>
     </row>
     <row r="175" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A175" s="71"/>
-      <c r="B175" s="59" t="s">
+      <c r="A175" s="74"/>
+      <c r="B175" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="C175" s="57"/>
-      <c r="D175" s="57"/>
-      <c r="E175" s="57"/>
-      <c r="F175" s="58"/>
+      <c r="C175" s="58"/>
+      <c r="D175" s="58"/>
+      <c r="E175" s="58"/>
+      <c r="F175" s="57"/>
       <c r="G175" s="9"/>
       <c r="H175" s="9"/>
       <c r="I175" s="9"/>
@@ -14011,14 +14011,14 @@
       <c r="Z175" s="9"/>
     </row>
     <row r="176" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A176" s="71"/>
-      <c r="B176" s="59" t="s">
+      <c r="A176" s="74"/>
+      <c r="B176" s="96" t="s">
         <v>122</v>
       </c>
-      <c r="C176" s="57"/>
-      <c r="D176" s="57"/>
-      <c r="E176" s="57"/>
-      <c r="F176" s="58"/>
+      <c r="C176" s="58"/>
+      <c r="D176" s="58"/>
+      <c r="E176" s="58"/>
+      <c r="F176" s="57"/>
       <c r="G176" s="9"/>
       <c r="H176" s="9"/>
       <c r="I176" s="9"/>
@@ -14041,12 +14041,12 @@
       <c r="Z176" s="9"/>
     </row>
     <row r="177" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A177" s="71"/>
+      <c r="A177" s="74"/>
       <c r="B177" s="60"/>
-      <c r="C177" s="57"/>
-      <c r="D177" s="57"/>
-      <c r="E177" s="57"/>
-      <c r="F177" s="58"/>
+      <c r="C177" s="58"/>
+      <c r="D177" s="58"/>
+      <c r="E177" s="58"/>
+      <c r="F177" s="57"/>
       <c r="G177" s="9"/>
       <c r="H177" s="9"/>
       <c r="I177" s="9"/>
@@ -14069,14 +14069,14 @@
       <c r="Z177" s="9"/>
     </row>
     <row r="178" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A178" s="71"/>
-      <c r="B178" s="85" t="s">
+      <c r="A178" s="74"/>
+      <c r="B178" s="89" t="s">
         <v>123</v>
       </c>
-      <c r="C178" s="62"/>
-      <c r="D178" s="62"/>
-      <c r="E178" s="62"/>
-      <c r="F178" s="63"/>
+      <c r="C178" s="84"/>
+      <c r="D178" s="84"/>
+      <c r="E178" s="84"/>
+      <c r="F178" s="79"/>
       <c r="G178" s="9"/>
       <c r="H178" s="9"/>
       <c r="I178" s="9"/>
@@ -14099,12 +14099,12 @@
       <c r="Z178" s="9"/>
     </row>
     <row r="179" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A179" s="71"/>
-      <c r="B179" s="67"/>
-      <c r="C179" s="68"/>
-      <c r="D179" s="68"/>
-      <c r="E179" s="68"/>
-      <c r="F179" s="69"/>
+      <c r="A179" s="74"/>
+      <c r="B179" s="85"/>
+      <c r="C179" s="86"/>
+      <c r="D179" s="86"/>
+      <c r="E179" s="86"/>
+      <c r="F179" s="87"/>
       <c r="G179" s="9"/>
       <c r="H179" s="9"/>
       <c r="I179" s="9"/>
@@ -14127,7 +14127,7 @@
       <c r="Z179" s="9"/>
     </row>
     <row r="180" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A180" s="71"/>
+      <c r="A180" s="74"/>
       <c r="B180" s="19" t="s">
         <v>124</v>
       </c>
@@ -14157,7 +14157,7 @@
       <c r="Z180" s="9"/>
     </row>
     <row r="181" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A181" s="71"/>
+      <c r="A181" s="74"/>
       <c r="B181" s="19" t="s">
         <v>125</v>
       </c>
@@ -14187,7 +14187,7 @@
       <c r="Z181" s="9"/>
     </row>
     <row r="182" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A182" s="71"/>
+      <c r="A182" s="74"/>
       <c r="B182" s="19" t="s">
         <v>126</v>
       </c>
@@ -14217,14 +14217,14 @@
       <c r="Z182" s="9"/>
     </row>
     <row r="183" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A183" s="71"/>
-      <c r="B183" s="59" t="s">
+      <c r="A183" s="74"/>
+      <c r="B183" s="96" t="s">
         <v>127</v>
       </c>
-      <c r="C183" s="57"/>
-      <c r="D183" s="57"/>
-      <c r="E183" s="57"/>
-      <c r="F183" s="58"/>
+      <c r="C183" s="58"/>
+      <c r="D183" s="58"/>
+      <c r="E183" s="58"/>
+      <c r="F183" s="57"/>
       <c r="G183" s="9"/>
       <c r="H183" s="9"/>
       <c r="I183" s="9"/>
@@ -14247,12 +14247,12 @@
       <c r="Z183" s="9"/>
     </row>
     <row r="184" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A184" s="71"/>
+      <c r="A184" s="74"/>
       <c r="B184" s="60"/>
-      <c r="C184" s="57"/>
-      <c r="D184" s="57"/>
-      <c r="E184" s="57"/>
-      <c r="F184" s="58"/>
+      <c r="C184" s="58"/>
+      <c r="D184" s="58"/>
+      <c r="E184" s="58"/>
+      <c r="F184" s="57"/>
       <c r="G184" s="9"/>
       <c r="H184" s="9"/>
       <c r="I184" s="9"/>
@@ -14275,14 +14275,14 @@
       <c r="Z184" s="9"/>
     </row>
     <row r="185" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A185" s="71"/>
-      <c r="B185" s="85" t="s">
+      <c r="A185" s="74"/>
+      <c r="B185" s="89" t="s">
         <v>128</v>
       </c>
-      <c r="C185" s="62"/>
-      <c r="D185" s="62"/>
-      <c r="E185" s="62"/>
-      <c r="F185" s="63"/>
+      <c r="C185" s="84"/>
+      <c r="D185" s="84"/>
+      <c r="E185" s="84"/>
+      <c r="F185" s="79"/>
       <c r="G185" s="9"/>
       <c r="H185" s="9"/>
       <c r="I185" s="9"/>
@@ -14305,12 +14305,12 @@
       <c r="Z185" s="9"/>
     </row>
     <row r="186" spans="1:26" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A186" s="71"/>
-      <c r="B186" s="67"/>
-      <c r="C186" s="68"/>
-      <c r="D186" s="68"/>
-      <c r="E186" s="68"/>
-      <c r="F186" s="69"/>
+      <c r="A186" s="74"/>
+      <c r="B186" s="85"/>
+      <c r="C186" s="86"/>
+      <c r="D186" s="86"/>
+      <c r="E186" s="86"/>
+      <c r="F186" s="87"/>
       <c r="G186" s="9"/>
       <c r="H186" s="9"/>
       <c r="I186" s="9"/>
@@ -14333,14 +14333,14 @@
       <c r="Z186" s="9"/>
     </row>
     <row r="187" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A187" s="71"/>
-      <c r="B187" s="59" t="s">
+      <c r="A187" s="74"/>
+      <c r="B187" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="C187" s="57"/>
-      <c r="D187" s="57"/>
-      <c r="E187" s="57"/>
-      <c r="F187" s="58"/>
+      <c r="C187" s="58"/>
+      <c r="D187" s="58"/>
+      <c r="E187" s="58"/>
+      <c r="F187" s="57"/>
       <c r="G187" s="9"/>
       <c r="H187" s="9"/>
       <c r="I187" s="9"/>
@@ -14363,12 +14363,12 @@
       <c r="Z187" s="9"/>
     </row>
     <row r="188" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A188" s="71"/>
-      <c r="B188" s="59"/>
-      <c r="C188" s="57"/>
-      <c r="D188" s="57"/>
-      <c r="E188" s="57"/>
-      <c r="F188" s="58"/>
+      <c r="A188" s="74"/>
+      <c r="B188" s="96"/>
+      <c r="C188" s="58"/>
+      <c r="D188" s="58"/>
+      <c r="E188" s="58"/>
+      <c r="F188" s="57"/>
       <c r="G188" s="9"/>
       <c r="H188" s="9"/>
       <c r="I188" s="9"/>
@@ -14391,14 +14391,14 @@
       <c r="Z188" s="9"/>
     </row>
     <row r="189" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A189" s="71"/>
-      <c r="B189" s="75" t="s">
+      <c r="A189" s="74"/>
+      <c r="B189" s="62" t="s">
         <v>1984</v>
       </c>
-      <c r="C189" s="57"/>
-      <c r="D189" s="57"/>
-      <c r="E189" s="57"/>
-      <c r="F189" s="58"/>
+      <c r="C189" s="58"/>
+      <c r="D189" s="58"/>
+      <c r="E189" s="58"/>
+      <c r="F189" s="57"/>
       <c r="G189" s="9"/>
       <c r="H189" s="9"/>
       <c r="I189" s="9"/>
@@ -14421,12 +14421,12 @@
       <c r="Z189" s="9"/>
     </row>
     <row r="190" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="71"/>
-      <c r="B190" s="59"/>
-      <c r="C190" s="57"/>
-      <c r="D190" s="57"/>
-      <c r="E190" s="57"/>
-      <c r="F190" s="58"/>
+      <c r="A190" s="74"/>
+      <c r="B190" s="96"/>
+      <c r="C190" s="58"/>
+      <c r="D190" s="58"/>
+      <c r="E190" s="58"/>
+      <c r="F190" s="57"/>
       <c r="G190" s="9"/>
       <c r="H190" s="9"/>
       <c r="I190" s="9"/>
@@ -14449,12 +14449,12 @@
       <c r="Z190" s="9"/>
     </row>
     <row r="191" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A191" s="71"/>
-      <c r="B191" s="59"/>
-      <c r="C191" s="57"/>
-      <c r="D191" s="57"/>
-      <c r="E191" s="57"/>
-      <c r="F191" s="58"/>
+      <c r="A191" s="74"/>
+      <c r="B191" s="96"/>
+      <c r="C191" s="58"/>
+      <c r="D191" s="58"/>
+      <c r="E191" s="58"/>
+      <c r="F191" s="57"/>
       <c r="G191" s="9"/>
       <c r="H191" s="9"/>
       <c r="I191" s="9"/>
@@ -14477,12 +14477,12 @@
       <c r="Z191" s="9"/>
     </row>
     <row r="192" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A192" s="72"/>
-      <c r="B192" s="59"/>
-      <c r="C192" s="57"/>
-      <c r="D192" s="57"/>
-      <c r="E192" s="57"/>
-      <c r="F192" s="58"/>
+      <c r="A192" s="75"/>
+      <c r="B192" s="96"/>
+      <c r="C192" s="58"/>
+      <c r="D192" s="58"/>
+      <c r="E192" s="58"/>
+      <c r="F192" s="57"/>
       <c r="G192" s="9"/>
       <c r="H192" s="9"/>
       <c r="I192" s="9"/>
@@ -14563,18 +14563,18 @@
       <c r="Z194" s="9"/>
     </row>
     <row r="195" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A195" s="70">
+      <c r="A195" s="73">
         <v>37</v>
       </c>
       <c r="B195" s="54" t="s">
         <v>1953</v>
       </c>
-      <c r="C195" s="59" t="s">
+      <c r="C195" s="96" t="s">
         <v>131</v>
       </c>
-      <c r="D195" s="57"/>
-      <c r="E195" s="57"/>
-      <c r="F195" s="58"/>
+      <c r="D195" s="58"/>
+      <c r="E195" s="58"/>
+      <c r="F195" s="57"/>
       <c r="G195" s="9"/>
       <c r="H195" s="9"/>
       <c r="I195" s="9"/>
@@ -14597,16 +14597,16 @@
       <c r="Z195" s="9"/>
     </row>
     <row r="196" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A196" s="71"/>
+      <c r="A196" s="74"/>
       <c r="B196" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C196" s="59" t="s">
+      <c r="C196" s="96" t="s">
         <v>132</v>
       </c>
-      <c r="D196" s="57"/>
-      <c r="E196" s="57"/>
-      <c r="F196" s="58"/>
+      <c r="D196" s="58"/>
+      <c r="E196" s="58"/>
+      <c r="F196" s="57"/>
       <c r="G196" s="9"/>
       <c r="H196" s="9"/>
       <c r="I196" s="9"/>
@@ -14629,16 +14629,16 @@
       <c r="Z196" s="9"/>
     </row>
     <row r="197" spans="1:26" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A197" s="71"/>
+      <c r="A197" s="74"/>
       <c r="B197" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C197" s="81" t="s">
+      <c r="C197" s="97" t="s">
         <v>133</v>
       </c>
-      <c r="D197" s="57"/>
-      <c r="E197" s="57"/>
-      <c r="F197" s="58"/>
+      <c r="D197" s="58"/>
+      <c r="E197" s="58"/>
+      <c r="F197" s="57"/>
       <c r="G197" s="9"/>
       <c r="H197" s="9"/>
       <c r="I197" s="9"/>
@@ -14661,16 +14661,16 @@
       <c r="Z197" s="9"/>
     </row>
     <row r="198" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A198" s="71"/>
+      <c r="A198" s="74"/>
       <c r="B198" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C198" s="59" t="s">
+      <c r="C198" s="96" t="s">
         <v>134</v>
       </c>
-      <c r="D198" s="57"/>
-      <c r="E198" s="57"/>
-      <c r="F198" s="58"/>
+      <c r="D198" s="58"/>
+      <c r="E198" s="58"/>
+      <c r="F198" s="57"/>
       <c r="G198" s="9"/>
       <c r="H198" s="9"/>
       <c r="I198" s="9"/>
@@ -14693,16 +14693,16 @@
       <c r="Z198" s="9"/>
     </row>
     <row r="199" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A199" s="71"/>
+      <c r="A199" s="74"/>
       <c r="B199" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C199" s="59" t="s">
+      <c r="C199" s="96" t="s">
         <v>135</v>
       </c>
-      <c r="D199" s="57"/>
-      <c r="E199" s="57"/>
-      <c r="F199" s="58"/>
+      <c r="D199" s="58"/>
+      <c r="E199" s="58"/>
+      <c r="F199" s="57"/>
       <c r="G199" s="9"/>
       <c r="H199" s="9"/>
       <c r="I199" s="9"/>
@@ -14725,16 +14725,16 @@
       <c r="Z199" s="9"/>
     </row>
     <row r="200" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="71"/>
+      <c r="A200" s="74"/>
       <c r="B200" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C200" s="59" t="s">
+      <c r="C200" s="96" t="s">
         <v>136</v>
       </c>
-      <c r="D200" s="57"/>
-      <c r="E200" s="57"/>
-      <c r="F200" s="58"/>
+      <c r="D200" s="58"/>
+      <c r="E200" s="58"/>
+      <c r="F200" s="57"/>
       <c r="G200" s="9"/>
       <c r="H200" s="9"/>
       <c r="I200" s="9"/>
@@ -14757,16 +14757,16 @@
       <c r="Z200" s="9"/>
     </row>
     <row r="201" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A201" s="71"/>
+      <c r="A201" s="74"/>
       <c r="B201" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C201" s="59" t="s">
+      <c r="C201" s="96" t="s">
         <v>137</v>
       </c>
-      <c r="D201" s="57"/>
-      <c r="E201" s="57"/>
-      <c r="F201" s="57"/>
+      <c r="D201" s="58"/>
+      <c r="E201" s="58"/>
+      <c r="F201" s="58"/>
       <c r="G201" s="9"/>
       <c r="H201" s="9"/>
       <c r="I201" s="9"/>
@@ -14789,16 +14789,16 @@
       <c r="Z201" s="9"/>
     </row>
     <row r="202" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A202" s="71"/>
+      <c r="A202" s="74"/>
       <c r="B202" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C202" s="59" t="s">
+      <c r="C202" s="96" t="s">
         <v>138</v>
       </c>
-      <c r="D202" s="57"/>
-      <c r="E202" s="57"/>
-      <c r="F202" s="58"/>
+      <c r="D202" s="58"/>
+      <c r="E202" s="58"/>
+      <c r="F202" s="57"/>
       <c r="G202" s="9"/>
       <c r="H202" s="9"/>
       <c r="I202" s="9"/>
@@ -14821,16 +14821,16 @@
       <c r="Z202" s="9"/>
     </row>
     <row r="203" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A203" s="71"/>
+      <c r="A203" s="74"/>
       <c r="B203" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C203" s="59" t="s">
+      <c r="C203" s="96" t="s">
         <v>139</v>
       </c>
-      <c r="D203" s="57"/>
-      <c r="E203" s="57"/>
-      <c r="F203" s="58"/>
+      <c r="D203" s="58"/>
+      <c r="E203" s="58"/>
+      <c r="F203" s="57"/>
       <c r="G203" s="9"/>
       <c r="H203" s="9"/>
       <c r="I203" s="9"/>
@@ -14853,16 +14853,16 @@
       <c r="Z203" s="9"/>
     </row>
     <row r="204" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A204" s="71"/>
+      <c r="A204" s="74"/>
       <c r="B204" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C204" s="59" t="s">
+      <c r="C204" s="96" t="s">
         <v>140</v>
       </c>
-      <c r="D204" s="57"/>
-      <c r="E204" s="57"/>
-      <c r="F204" s="58"/>
+      <c r="D204" s="58"/>
+      <c r="E204" s="58"/>
+      <c r="F204" s="57"/>
       <c r="G204" s="9"/>
       <c r="H204" s="9"/>
       <c r="I204" s="9"/>
@@ -14885,16 +14885,16 @@
       <c r="Z204" s="9"/>
     </row>
     <row r="205" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A205" s="71"/>
+      <c r="A205" s="74"/>
       <c r="B205" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C205" s="59" t="s">
+      <c r="C205" s="96" t="s">
         <v>141</v>
       </c>
-      <c r="D205" s="57"/>
-      <c r="E205" s="57"/>
-      <c r="F205" s="58"/>
+      <c r="D205" s="58"/>
+      <c r="E205" s="58"/>
+      <c r="F205" s="57"/>
       <c r="G205" s="9"/>
       <c r="H205" s="9"/>
       <c r="I205" s="9"/>
@@ -14917,16 +14917,16 @@
       <c r="Z205" s="9"/>
     </row>
     <row r="206" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A206" s="71"/>
+      <c r="A206" s="74"/>
       <c r="B206" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C206" s="59" t="s">
+      <c r="C206" s="96" t="s">
         <v>142</v>
       </c>
-      <c r="D206" s="57"/>
-      <c r="E206" s="57"/>
-      <c r="F206" s="58"/>
+      <c r="D206" s="58"/>
+      <c r="E206" s="58"/>
+      <c r="F206" s="57"/>
       <c r="G206" s="9"/>
       <c r="H206" s="9"/>
       <c r="I206" s="9"/>
@@ -14949,16 +14949,16 @@
       <c r="Z206" s="9"/>
     </row>
     <row r="207" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A207" s="71"/>
+      <c r="A207" s="74"/>
       <c r="B207" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C207" s="59" t="s">
+      <c r="C207" s="96" t="s">
         <v>143</v>
       </c>
-      <c r="D207" s="57"/>
-      <c r="E207" s="57"/>
-      <c r="F207" s="58"/>
+      <c r="D207" s="58"/>
+      <c r="E207" s="58"/>
+      <c r="F207" s="57"/>
       <c r="G207" s="9"/>
       <c r="H207" s="9"/>
       <c r="I207" s="9"/>
@@ -14981,16 +14981,16 @@
       <c r="Z207" s="9"/>
     </row>
     <row r="208" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A208" s="71"/>
+      <c r="A208" s="74"/>
       <c r="B208" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C208" s="59" t="s">
+      <c r="C208" s="96" t="s">
         <v>144</v>
       </c>
-      <c r="D208" s="57"/>
-      <c r="E208" s="57"/>
-      <c r="F208" s="58"/>
+      <c r="D208" s="58"/>
+      <c r="E208" s="58"/>
+      <c r="F208" s="57"/>
       <c r="G208" s="9"/>
       <c r="H208" s="9"/>
       <c r="I208" s="9"/>
@@ -15013,16 +15013,16 @@
       <c r="Z208" s="9"/>
     </row>
     <row r="209" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A209" s="71"/>
+      <c r="A209" s="74"/>
       <c r="B209" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C209" s="59" t="s">
+      <c r="C209" s="96" t="s">
         <v>145</v>
       </c>
-      <c r="D209" s="57"/>
-      <c r="E209" s="57"/>
-      <c r="F209" s="58"/>
+      <c r="D209" s="58"/>
+      <c r="E209" s="58"/>
+      <c r="F209" s="57"/>
       <c r="G209" s="9"/>
       <c r="H209" s="9"/>
       <c r="I209" s="9"/>
@@ -15045,16 +15045,16 @@
       <c r="Z209" s="9"/>
     </row>
     <row r="210" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="71"/>
+      <c r="A210" s="74"/>
       <c r="B210" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C210" s="59" t="s">
+      <c r="C210" s="96" t="s">
         <v>146</v>
       </c>
-      <c r="D210" s="57"/>
-      <c r="E210" s="57"/>
-      <c r="F210" s="58"/>
+      <c r="D210" s="58"/>
+      <c r="E210" s="58"/>
+      <c r="F210" s="57"/>
       <c r="G210" s="9"/>
       <c r="H210" s="9"/>
       <c r="I210" s="9"/>
@@ -15077,16 +15077,16 @@
       <c r="Z210" s="9"/>
     </row>
     <row r="211" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="71"/>
+      <c r="A211" s="74"/>
       <c r="B211" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C211" s="59" t="s">
+      <c r="C211" s="96" t="s">
         <v>147</v>
       </c>
-      <c r="D211" s="57"/>
-      <c r="E211" s="57"/>
-      <c r="F211" s="58"/>
+      <c r="D211" s="58"/>
+      <c r="E211" s="58"/>
+      <c r="F211" s="57"/>
       <c r="G211" s="9"/>
       <c r="H211" s="9"/>
       <c r="I211" s="9"/>
@@ -15109,16 +15109,16 @@
       <c r="Z211" s="9"/>
     </row>
     <row r="212" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="71"/>
+      <c r="A212" s="74"/>
       <c r="B212" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C212" s="59" t="s">
+      <c r="C212" s="96" t="s">
         <v>148</v>
       </c>
-      <c r="D212" s="57"/>
-      <c r="E212" s="57"/>
-      <c r="F212" s="58"/>
+      <c r="D212" s="58"/>
+      <c r="E212" s="58"/>
+      <c r="F212" s="57"/>
       <c r="G212" s="9"/>
       <c r="H212" s="9"/>
       <c r="I212" s="9"/>
@@ -15141,16 +15141,16 @@
       <c r="Z212" s="9"/>
     </row>
     <row r="213" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A213" s="71"/>
+      <c r="A213" s="74"/>
       <c r="B213" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C213" s="59" t="s">
+      <c r="C213" s="96" t="s">
         <v>149</v>
       </c>
-      <c r="D213" s="57"/>
-      <c r="E213" s="57"/>
-      <c r="F213" s="58"/>
+      <c r="D213" s="58"/>
+      <c r="E213" s="58"/>
+      <c r="F213" s="57"/>
       <c r="G213" s="9"/>
       <c r="H213" s="9"/>
       <c r="I213" s="9"/>
@@ -15173,16 +15173,16 @@
       <c r="Z213" s="9"/>
     </row>
     <row r="214" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A214" s="71"/>
+      <c r="A214" s="74"/>
       <c r="B214" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C214" s="59" t="s">
+      <c r="C214" s="96" t="s">
         <v>150</v>
       </c>
-      <c r="D214" s="57"/>
-      <c r="E214" s="57"/>
-      <c r="F214" s="58"/>
+      <c r="D214" s="58"/>
+      <c r="E214" s="58"/>
+      <c r="F214" s="57"/>
       <c r="G214" s="9"/>
       <c r="H214" s="9"/>
       <c r="I214" s="9"/>
@@ -15205,16 +15205,16 @@
       <c r="Z214" s="9"/>
     </row>
     <row r="215" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A215" s="71"/>
+      <c r="A215" s="74"/>
       <c r="B215" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C215" s="59" t="s">
+      <c r="C215" s="96" t="s">
         <v>151</v>
       </c>
-      <c r="D215" s="57"/>
-      <c r="E215" s="57"/>
-      <c r="F215" s="58"/>
+      <c r="D215" s="58"/>
+      <c r="E215" s="58"/>
+      <c r="F215" s="57"/>
       <c r="G215" s="9"/>
       <c r="H215" s="9"/>
       <c r="I215" s="9"/>
@@ -15237,16 +15237,16 @@
       <c r="Z215" s="9"/>
     </row>
     <row r="216" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A216" s="71"/>
+      <c r="A216" s="74"/>
       <c r="B216" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C216" s="59" t="s">
+      <c r="C216" s="96" t="s">
         <v>152</v>
       </c>
-      <c r="D216" s="57"/>
-      <c r="E216" s="57"/>
-      <c r="F216" s="58"/>
+      <c r="D216" s="58"/>
+      <c r="E216" s="58"/>
+      <c r="F216" s="57"/>
       <c r="G216" s="9"/>
       <c r="H216" s="9"/>
       <c r="I216" s="9"/>
@@ -15269,16 +15269,16 @@
       <c r="Z216" s="9"/>
     </row>
     <row r="217" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A217" s="71"/>
+      <c r="A217" s="74"/>
       <c r="B217" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C217" s="59" t="s">
+      <c r="C217" s="96" t="s">
         <v>153</v>
       </c>
-      <c r="D217" s="57"/>
-      <c r="E217" s="57"/>
-      <c r="F217" s="58"/>
+      <c r="D217" s="58"/>
+      <c r="E217" s="58"/>
+      <c r="F217" s="57"/>
       <c r="G217" s="9"/>
       <c r="H217" s="9"/>
       <c r="I217" s="9"/>
@@ -15301,16 +15301,16 @@
       <c r="Z217" s="9"/>
     </row>
     <row r="218" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A218" s="71"/>
+      <c r="A218" s="74"/>
       <c r="B218" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C218" s="59" t="s">
+      <c r="C218" s="96" t="s">
         <v>154</v>
       </c>
-      <c r="D218" s="57"/>
-      <c r="E218" s="57"/>
-      <c r="F218" s="58"/>
+      <c r="D218" s="58"/>
+      <c r="E218" s="58"/>
+      <c r="F218" s="57"/>
       <c r="G218" s="9"/>
       <c r="H218" s="9"/>
       <c r="I218" s="9"/>
@@ -15333,16 +15333,16 @@
       <c r="Z218" s="9"/>
     </row>
     <row r="219" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A219" s="72"/>
+      <c r="A219" s="75"/>
       <c r="B219" s="47" t="s">
         <v>1953</v>
       </c>
-      <c r="C219" s="83" t="s">
+      <c r="C219" s="98" t="s">
         <v>1985</v>
       </c>
-      <c r="D219" s="57"/>
-      <c r="E219" s="57"/>
-      <c r="F219" s="58"/>
+      <c r="D219" s="58"/>
+      <c r="E219" s="58"/>
+      <c r="F219" s="57"/>
       <c r="G219" s="9"/>
       <c r="H219" s="9"/>
       <c r="I219" s="9"/>
@@ -15423,16 +15423,16 @@
       <c r="Z221" s="9"/>
     </row>
     <row r="222" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A222" s="73">
+      <c r="A222" s="104">
         <v>38</v>
       </c>
-      <c r="B222" s="84" t="s">
+      <c r="B222" s="99" t="s">
         <v>156</v>
       </c>
-      <c r="C222" s="62"/>
-      <c r="D222" s="62"/>
-      <c r="E222" s="62"/>
-      <c r="F222" s="63"/>
+      <c r="C222" s="84"/>
+      <c r="D222" s="84"/>
+      <c r="E222" s="84"/>
+      <c r="F222" s="79"/>
       <c r="G222" s="9"/>
       <c r="H222" s="9"/>
       <c r="I222" s="9"/>
@@ -15455,12 +15455,12 @@
       <c r="Z222" s="9"/>
     </row>
     <row r="223" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A223" s="71"/>
-      <c r="B223" s="64"/>
-      <c r="C223" s="65"/>
-      <c r="D223" s="65"/>
-      <c r="E223" s="65"/>
-      <c r="F223" s="66"/>
+      <c r="A223" s="74"/>
+      <c r="B223" s="80"/>
+      <c r="C223" s="66"/>
+      <c r="D223" s="66"/>
+      <c r="E223" s="66"/>
+      <c r="F223" s="81"/>
       <c r="G223" s="9"/>
       <c r="H223" s="9"/>
       <c r="I223" s="9"/>
@@ -15483,12 +15483,12 @@
       <c r="Z223" s="9"/>
     </row>
     <row r="224" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A224" s="71"/>
-      <c r="B224" s="64"/>
-      <c r="C224" s="65"/>
-      <c r="D224" s="65"/>
-      <c r="E224" s="65"/>
-      <c r="F224" s="66"/>
+      <c r="A224" s="74"/>
+      <c r="B224" s="80"/>
+      <c r="C224" s="66"/>
+      <c r="D224" s="66"/>
+      <c r="E224" s="66"/>
+      <c r="F224" s="81"/>
       <c r="G224" s="9"/>
       <c r="H224" s="9"/>
       <c r="I224" s="9"/>
@@ -15511,12 +15511,12 @@
       <c r="Z224" s="9"/>
     </row>
     <row r="225" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A225" s="72"/>
-      <c r="B225" s="67"/>
-      <c r="C225" s="68"/>
-      <c r="D225" s="68"/>
-      <c r="E225" s="68"/>
-      <c r="F225" s="69"/>
+      <c r="A225" s="75"/>
+      <c r="B225" s="85"/>
+      <c r="C225" s="86"/>
+      <c r="D225" s="86"/>
+      <c r="E225" s="86"/>
+      <c r="F225" s="87"/>
       <c r="G225" s="9"/>
       <c r="H225" s="9"/>
       <c r="I225" s="9"/>
@@ -15625,16 +15625,16 @@
       <c r="Z228" s="9"/>
     </row>
     <row r="229" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A229" s="70">
+      <c r="A229" s="73">
         <v>39</v>
       </c>
-      <c r="B229" s="61" t="s">
+      <c r="B229" s="103" t="s">
         <v>158</v>
       </c>
-      <c r="C229" s="62"/>
-      <c r="D229" s="62"/>
-      <c r="E229" s="62"/>
-      <c r="F229" s="63"/>
+      <c r="C229" s="84"/>
+      <c r="D229" s="84"/>
+      <c r="E229" s="84"/>
+      <c r="F229" s="79"/>
       <c r="G229" s="9"/>
       <c r="H229" s="9"/>
       <c r="I229" s="9"/>
@@ -15657,12 +15657,12 @@
       <c r="Z229" s="9"/>
     </row>
     <row r="230" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A230" s="71"/>
-      <c r="B230" s="64"/>
-      <c r="C230" s="65"/>
-      <c r="D230" s="65"/>
-      <c r="E230" s="65"/>
-      <c r="F230" s="66"/>
+      <c r="A230" s="74"/>
+      <c r="B230" s="80"/>
+      <c r="C230" s="66"/>
+      <c r="D230" s="66"/>
+      <c r="E230" s="66"/>
+      <c r="F230" s="81"/>
       <c r="G230" s="9"/>
       <c r="H230" s="9"/>
       <c r="I230" s="9"/>
@@ -15685,12 +15685,12 @@
       <c r="Z230" s="9"/>
     </row>
     <row r="231" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A231" s="71"/>
-      <c r="B231" s="64"/>
-      <c r="C231" s="65"/>
-      <c r="D231" s="65"/>
-      <c r="E231" s="65"/>
-      <c r="F231" s="66"/>
+      <c r="A231" s="74"/>
+      <c r="B231" s="80"/>
+      <c r="C231" s="66"/>
+      <c r="D231" s="66"/>
+      <c r="E231" s="66"/>
+      <c r="F231" s="81"/>
       <c r="G231" s="9"/>
       <c r="H231" s="9"/>
       <c r="I231" s="9"/>
@@ -15713,12 +15713,12 @@
       <c r="Z231" s="9"/>
     </row>
     <row r="232" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A232" s="71"/>
-      <c r="B232" s="64"/>
-      <c r="C232" s="65"/>
-      <c r="D232" s="65"/>
-      <c r="E232" s="65"/>
-      <c r="F232" s="66"/>
+      <c r="A232" s="74"/>
+      <c r="B232" s="80"/>
+      <c r="C232" s="66"/>
+      <c r="D232" s="66"/>
+      <c r="E232" s="66"/>
+      <c r="F232" s="81"/>
       <c r="G232" s="9"/>
       <c r="H232" s="9"/>
       <c r="I232" s="9"/>
@@ -15741,12 +15741,12 @@
       <c r="Z232" s="9"/>
     </row>
     <row r="233" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A233" s="71"/>
-      <c r="B233" s="64"/>
-      <c r="C233" s="65"/>
-      <c r="D233" s="65"/>
-      <c r="E233" s="65"/>
-      <c r="F233" s="66"/>
+      <c r="A233" s="74"/>
+      <c r="B233" s="80"/>
+      <c r="C233" s="66"/>
+      <c r="D233" s="66"/>
+      <c r="E233" s="66"/>
+      <c r="F233" s="81"/>
       <c r="G233" s="9"/>
       <c r="H233" s="9"/>
       <c r="I233" s="9"/>
@@ -15769,12 +15769,12 @@
       <c r="Z233" s="9"/>
     </row>
     <row r="234" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A234" s="71"/>
-      <c r="B234" s="64"/>
-      <c r="C234" s="65"/>
-      <c r="D234" s="65"/>
-      <c r="E234" s="65"/>
-      <c r="F234" s="66"/>
+      <c r="A234" s="74"/>
+      <c r="B234" s="80"/>
+      <c r="C234" s="66"/>
+      <c r="D234" s="66"/>
+      <c r="E234" s="66"/>
+      <c r="F234" s="81"/>
       <c r="G234" s="9"/>
       <c r="H234" s="9"/>
       <c r="I234" s="9"/>
@@ -15797,12 +15797,12 @@
       <c r="Z234" s="9"/>
     </row>
     <row r="235" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A235" s="72"/>
-      <c r="B235" s="67"/>
-      <c r="C235" s="68"/>
-      <c r="D235" s="68"/>
-      <c r="E235" s="68"/>
-      <c r="F235" s="69"/>
+      <c r="A235" s="75"/>
+      <c r="B235" s="85"/>
+      <c r="C235" s="86"/>
+      <c r="D235" s="86"/>
+      <c r="E235" s="86"/>
+      <c r="F235" s="87"/>
       <c r="G235" s="9"/>
       <c r="H235" s="9"/>
       <c r="I235" s="9"/>
@@ -37258,79 +37258,90 @@
     </row>
   </sheetData>
   <mergeCells count="181">
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="D56:F56"/>
-    <mergeCell ref="D57:F57"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="D59:F59"/>
-    <mergeCell ref="D60:F60"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="D62:F62"/>
-    <mergeCell ref="D63:F63"/>
-    <mergeCell ref="D64:F64"/>
-    <mergeCell ref="D65:F65"/>
-    <mergeCell ref="D66:F66"/>
-    <mergeCell ref="D69:F69"/>
-    <mergeCell ref="D70:F70"/>
-    <mergeCell ref="D71:F71"/>
-    <mergeCell ref="D72:F72"/>
-    <mergeCell ref="D73:F73"/>
-    <mergeCell ref="D74:F74"/>
-    <mergeCell ref="D75:F75"/>
-    <mergeCell ref="D76:F76"/>
-    <mergeCell ref="D77:F77"/>
-    <mergeCell ref="D78:F78"/>
-    <mergeCell ref="E128:F128"/>
-    <mergeCell ref="D79:F79"/>
-    <mergeCell ref="D80:F80"/>
-    <mergeCell ref="D81:F81"/>
-    <mergeCell ref="D82:F82"/>
-    <mergeCell ref="D83:F83"/>
-    <mergeCell ref="D84:F84"/>
-    <mergeCell ref="D85:F85"/>
-    <mergeCell ref="D101:F101"/>
-    <mergeCell ref="D102:F102"/>
-    <mergeCell ref="E125:F125"/>
-    <mergeCell ref="D103:F103"/>
-    <mergeCell ref="D113:F113"/>
-    <mergeCell ref="D114:F114"/>
-    <mergeCell ref="D115:F115"/>
-    <mergeCell ref="D116:F116"/>
-    <mergeCell ref="D117:F117"/>
-    <mergeCell ref="E126:F126"/>
-    <mergeCell ref="E127:F127"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="B31:C33"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="B174:F174"/>
+    <mergeCell ref="B175:F175"/>
+    <mergeCell ref="B176:F176"/>
+    <mergeCell ref="B177:F177"/>
+    <mergeCell ref="B229:F235"/>
+    <mergeCell ref="A55:A61"/>
+    <mergeCell ref="A69:A77"/>
+    <mergeCell ref="A114:A121"/>
+    <mergeCell ref="A124:A132"/>
+    <mergeCell ref="A135:A157"/>
+    <mergeCell ref="A160:A192"/>
+    <mergeCell ref="A195:A219"/>
+    <mergeCell ref="A222:A225"/>
+    <mergeCell ref="A229:A235"/>
+    <mergeCell ref="A78:A84"/>
+    <mergeCell ref="A88:A100"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A106:A111"/>
+    <mergeCell ref="A123:D123"/>
+    <mergeCell ref="B124:D124"/>
+    <mergeCell ref="B125:D125"/>
+    <mergeCell ref="B126:D126"/>
+    <mergeCell ref="B127:D127"/>
+    <mergeCell ref="B128:D128"/>
+    <mergeCell ref="B129:D129"/>
+    <mergeCell ref="B130:D130"/>
+    <mergeCell ref="B131:D131"/>
+    <mergeCell ref="B132:D132"/>
+    <mergeCell ref="B135:F157"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="B34:C36"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:C39"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="B121:C121"/>
+    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="E124:F124"/>
+    <mergeCell ref="C219:F219"/>
+    <mergeCell ref="B222:F225"/>
+    <mergeCell ref="C212:F212"/>
+    <mergeCell ref="C213:F213"/>
+    <mergeCell ref="C214:F214"/>
+    <mergeCell ref="C215:F215"/>
+    <mergeCell ref="C216:F216"/>
+    <mergeCell ref="C217:F217"/>
+    <mergeCell ref="C218:F218"/>
+    <mergeCell ref="C210:F210"/>
+    <mergeCell ref="C211:F211"/>
+    <mergeCell ref="C203:F203"/>
+    <mergeCell ref="C204:F204"/>
+    <mergeCell ref="C205:F205"/>
+    <mergeCell ref="C206:F206"/>
+    <mergeCell ref="C207:F207"/>
+    <mergeCell ref="C208:F208"/>
+    <mergeCell ref="C209:F209"/>
+    <mergeCell ref="C201:F201"/>
+    <mergeCell ref="C202:F202"/>
+    <mergeCell ref="B192:F192"/>
+    <mergeCell ref="C195:F195"/>
+    <mergeCell ref="C196:F196"/>
+    <mergeCell ref="C197:F197"/>
+    <mergeCell ref="C198:F198"/>
+    <mergeCell ref="C199:F199"/>
+    <mergeCell ref="C200:F200"/>
+    <mergeCell ref="B190:F190"/>
+    <mergeCell ref="B191:F191"/>
+    <mergeCell ref="B178:F179"/>
+    <mergeCell ref="B183:F183"/>
+    <mergeCell ref="B184:F184"/>
+    <mergeCell ref="B185:F186"/>
+    <mergeCell ref="B187:F187"/>
+    <mergeCell ref="B188:F188"/>
+    <mergeCell ref="B189:F189"/>
     <mergeCell ref="B160:F160"/>
     <mergeCell ref="B161:F162"/>
     <mergeCell ref="B163:F163"/>
@@ -37355,90 +37366,79 @@
     <mergeCell ref="D119:F119"/>
     <mergeCell ref="D120:F120"/>
     <mergeCell ref="D121:F121"/>
-    <mergeCell ref="B190:F190"/>
-    <mergeCell ref="B191:F191"/>
-    <mergeCell ref="B178:F179"/>
-    <mergeCell ref="B183:F183"/>
-    <mergeCell ref="B184:F184"/>
-    <mergeCell ref="B185:F186"/>
-    <mergeCell ref="B187:F187"/>
-    <mergeCell ref="B188:F188"/>
-    <mergeCell ref="B189:F189"/>
-    <mergeCell ref="C201:F201"/>
-    <mergeCell ref="C202:F202"/>
-    <mergeCell ref="B192:F192"/>
-    <mergeCell ref="C195:F195"/>
-    <mergeCell ref="C196:F196"/>
-    <mergeCell ref="C197:F197"/>
-    <mergeCell ref="C198:F198"/>
-    <mergeCell ref="C199:F199"/>
-    <mergeCell ref="C200:F200"/>
-    <mergeCell ref="C210:F210"/>
-    <mergeCell ref="C211:F211"/>
-    <mergeCell ref="C203:F203"/>
-    <mergeCell ref="C204:F204"/>
-    <mergeCell ref="C205:F205"/>
-    <mergeCell ref="C206:F206"/>
-    <mergeCell ref="C207:F207"/>
-    <mergeCell ref="C208:F208"/>
-    <mergeCell ref="C209:F209"/>
-    <mergeCell ref="C219:F219"/>
-    <mergeCell ref="B222:F225"/>
-    <mergeCell ref="C212:F212"/>
-    <mergeCell ref="C213:F213"/>
-    <mergeCell ref="C214:F214"/>
-    <mergeCell ref="C215:F215"/>
-    <mergeCell ref="C216:F216"/>
-    <mergeCell ref="C217:F217"/>
-    <mergeCell ref="C218:F218"/>
-    <mergeCell ref="B129:D129"/>
-    <mergeCell ref="B130:D130"/>
-    <mergeCell ref="B131:D131"/>
-    <mergeCell ref="B132:D132"/>
-    <mergeCell ref="B135:F157"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="B34:C36"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:C39"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="B121:C121"/>
-    <mergeCell ref="E123:F123"/>
-    <mergeCell ref="E124:F124"/>
-    <mergeCell ref="B174:F174"/>
-    <mergeCell ref="B175:F175"/>
-    <mergeCell ref="B176:F176"/>
-    <mergeCell ref="B177:F177"/>
-    <mergeCell ref="B229:F235"/>
-    <mergeCell ref="A55:A61"/>
-    <mergeCell ref="A69:A77"/>
-    <mergeCell ref="A114:A121"/>
-    <mergeCell ref="A124:A132"/>
-    <mergeCell ref="A135:A157"/>
-    <mergeCell ref="A160:A192"/>
-    <mergeCell ref="A195:A219"/>
-    <mergeCell ref="A222:A225"/>
-    <mergeCell ref="A229:A235"/>
-    <mergeCell ref="A78:A84"/>
-    <mergeCell ref="A88:A100"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A106:A111"/>
-    <mergeCell ref="A123:D123"/>
-    <mergeCell ref="B124:D124"/>
-    <mergeCell ref="B125:D125"/>
-    <mergeCell ref="B126:D126"/>
-    <mergeCell ref="B127:D127"/>
-    <mergeCell ref="B128:D128"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="B31:C33"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="E128:F128"/>
+    <mergeCell ref="D79:F79"/>
+    <mergeCell ref="D80:F80"/>
+    <mergeCell ref="D81:F81"/>
+    <mergeCell ref="D82:F82"/>
+    <mergeCell ref="D83:F83"/>
+    <mergeCell ref="D84:F84"/>
+    <mergeCell ref="D85:F85"/>
+    <mergeCell ref="D101:F101"/>
+    <mergeCell ref="D102:F102"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="D103:F103"/>
+    <mergeCell ref="D113:F113"/>
+    <mergeCell ref="D114:F114"/>
+    <mergeCell ref="D115:F115"/>
+    <mergeCell ref="D116:F116"/>
+    <mergeCell ref="D117:F117"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="D70:F70"/>
+    <mergeCell ref="D71:F71"/>
+    <mergeCell ref="D72:F72"/>
+    <mergeCell ref="D73:F73"/>
+    <mergeCell ref="D74:F74"/>
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="D76:F76"/>
+    <mergeCell ref="D77:F77"/>
+    <mergeCell ref="D78:F78"/>
+    <mergeCell ref="D59:F59"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="D63:F63"/>
+    <mergeCell ref="D64:F64"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="D55:F55"/>
+    <mergeCell ref="D56:F56"/>
+    <mergeCell ref="D57:F57"/>
+    <mergeCell ref="D58:F58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="5" orientation="landscape"/>
@@ -37484,10 +37484,10 @@
       <c r="G1" s="108" t="s">
         <v>165</v>
       </c>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="81"/>
       <c r="L1" s="32"/>
       <c r="M1" s="33" t="s">
         <v>166</v>

</xml_diff>